<commit_message>
Add PrecioCompare landing page
</commit_message>
<xml_diff>
--- a/backend/excel_template.xlsx
+++ b/backend/excel_template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Frand\Documents\Bots\ElectrodomesticsBot\backend\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Frand\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{63375BA3-ECE9-4547-A012-1BD6C24330A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92466A16-5C18-4DA3-BFD9-653AB19E1405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="15700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="88">
   <si>
     <t>Interés</t>
   </si>
@@ -45,7 +45,7 @@
     <t>Cuotas</t>
   </si>
   <si>
-    <t>Prueba</t>
+    <t>Mi comercio</t>
   </si>
   <si>
     <t>Ecommerce</t>
@@ -288,10 +288,16 @@
     <t>MONTES</t>
   </si>
   <si>
+    <t>MI COMERCIO</t>
+  </si>
+  <si>
     <t>Markup</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>INSERTAR COSTO</t>
   </si>
 </sst>
 </file>
@@ -490,7 +496,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -594,13 +600,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="12" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -762,7 +783,6 @@
     <xf numFmtId="44" fontId="1" fillId="13" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -796,9 +816,7 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="164" fontId="10" fillId="14" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1043,14 +1061,14 @@
     <row r="2" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="62" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
-      <c r="H2" s="64"/>
+      <c r="C2" s="61" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="63"/>
     </row>
     <row r="3" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
@@ -1094,9 +1112,13 @@
       <c r="D4" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="54"/>
+      <c r="E4" s="54">
+        <v>55499</v>
+      </c>
       <c r="F4" s="54"/>
-      <c r="G4" s="55"/>
+      <c r="G4" s="55">
+        <v>58608</v>
+      </c>
       <c r="H4" s="56"/>
       <c r="I4" s="53" t="s">
         <v>10</v>
@@ -1115,10 +1137,14 @@
       <c r="D5" s="10">
         <v>-0.15</v>
       </c>
-      <c r="E5" s="58"/>
-      <c r="F5" s="58"/>
-      <c r="G5" s="59"/>
-      <c r="H5" s="59"/>
+      <c r="E5" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="57"/>
+      <c r="G5" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5" s="58"/>
       <c r="I5" s="11" t="s">
         <v>13</v>
       </c>
@@ -1136,10 +1162,14 @@
       <c r="D6" s="10">
         <v>-0.04</v>
       </c>
-      <c r="E6" s="58"/>
-      <c r="F6" s="59"/>
-      <c r="G6" s="59"/>
-      <c r="H6" s="59"/>
+      <c r="E6" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="58"/>
+      <c r="G6" s="58">
+        <v>0</v>
+      </c>
+      <c r="H6" s="58"/>
       <c r="I6" s="12" t="s">
         <v>15</v>
       </c>
@@ -1157,10 +1187,14 @@
       <c r="D7" s="9">
         <v>0</v>
       </c>
-      <c r="E7" s="58"/>
-      <c r="F7" s="59"/>
-      <c r="G7" s="59"/>
-      <c r="H7" s="59"/>
+      <c r="E7" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="58"/>
+      <c r="G7" s="58">
+        <v>0</v>
+      </c>
+      <c r="H7" s="58"/>
       <c r="I7" s="12" t="s">
         <v>16</v>
       </c>
@@ -1178,10 +1212,14 @@
       <c r="D8" s="9">
         <v>0</v>
       </c>
-      <c r="E8" s="58"/>
-      <c r="F8" s="59"/>
-      <c r="G8" s="59"/>
-      <c r="H8" s="59"/>
+      <c r="E8" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="58"/>
+      <c r="G8" s="58">
+        <v>0</v>
+      </c>
+      <c r="H8" s="58"/>
       <c r="I8" s="12" t="s">
         <v>17</v>
       </c>
@@ -1199,10 +1237,14 @@
       <c r="D9" s="9">
         <v>0.05</v>
       </c>
-      <c r="E9" s="58"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
-      <c r="H9" s="59"/>
+      <c r="E9" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="58"/>
+      <c r="G9" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9" s="58"/>
       <c r="I9" s="12" t="s">
         <v>18</v>
       </c>
@@ -1220,10 +1262,14 @@
       <c r="D10" s="9">
         <v>0</v>
       </c>
-      <c r="E10" s="60"/>
-      <c r="F10" s="59"/>
-      <c r="G10" s="59"/>
-      <c r="H10" s="59"/>
+      <c r="E10" s="59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="58"/>
+      <c r="G10" s="58">
+        <v>0</v>
+      </c>
+      <c r="H10" s="58"/>
       <c r="I10" s="12" t="s">
         <v>19</v>
       </c>
@@ -1241,10 +1287,14 @@
       <c r="D11" s="9">
         <v>0.1</v>
       </c>
-      <c r="E11" s="60"/>
-      <c r="F11" s="59"/>
-      <c r="G11" s="59"/>
-      <c r="H11" s="59"/>
+      <c r="E11" s="59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="58"/>
+      <c r="G11" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H11" s="58"/>
       <c r="I11" s="12" t="s">
         <v>20</v>
       </c>
@@ -1262,10 +1312,14 @@
       <c r="D12" s="9">
         <v>0</v>
       </c>
-      <c r="E12" s="59"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="59"/>
-      <c r="H12" s="59"/>
+      <c r="E12" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="59"/>
+      <c r="G12" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H12" s="58"/>
       <c r="I12" s="12" t="s">
         <v>21</v>
       </c>
@@ -1283,10 +1337,14 @@
       <c r="D13" s="9">
         <v>0.15</v>
       </c>
-      <c r="E13" s="59"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="59"/>
-      <c r="H13" s="59"/>
+      <c r="E13" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="59"/>
+      <c r="G13" s="58">
+        <v>1.95E-2</v>
+      </c>
+      <c r="H13" s="58"/>
       <c r="I13" s="12" t="s">
         <v>22</v>
       </c>
@@ -1304,10 +1362,14 @@
       <c r="D14" s="9">
         <v>0</v>
       </c>
-      <c r="E14" s="59"/>
-      <c r="F14" s="60"/>
-      <c r="G14" s="59"/>
-      <c r="H14" s="59"/>
+      <c r="E14" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="59"/>
+      <c r="G14" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14" s="58"/>
       <c r="I14" s="12" t="s">
         <v>23</v>
       </c>
@@ -1325,10 +1387,14 @@
       <c r="D15" s="9">
         <v>0.21</v>
       </c>
-      <c r="E15" s="60"/>
-      <c r="F15" s="60"/>
-      <c r="G15" s="59"/>
-      <c r="H15" s="59"/>
+      <c r="E15" s="59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="59"/>
+      <c r="G15" s="58">
+        <v>7.0199999999999999E-2</v>
+      </c>
+      <c r="H15" s="58"/>
       <c r="I15" s="12" t="s">
         <v>24</v>
       </c>
@@ -1346,10 +1412,14 @@
       <c r="D16" s="10">
         <v>-0.05</v>
       </c>
-      <c r="E16" s="58"/>
-      <c r="F16" s="59"/>
-      <c r="G16" s="59"/>
-      <c r="H16" s="59"/>
+      <c r="E16" s="57">
+        <v>0</v>
+      </c>
+      <c r="F16" s="58"/>
+      <c r="G16" s="58">
+        <v>0</v>
+      </c>
+      <c r="H16" s="58"/>
       <c r="I16" s="17" t="s">
         <v>26</v>
       </c>
@@ -1367,10 +1437,14 @@
       <c r="D17" s="10">
         <v>-0.05</v>
       </c>
-      <c r="E17" s="58"/>
-      <c r="F17" s="59"/>
-      <c r="G17" s="59"/>
-      <c r="H17" s="59"/>
+      <c r="E17" s="57">
+        <v>0</v>
+      </c>
+      <c r="F17" s="58"/>
+      <c r="G17" s="58">
+        <v>0</v>
+      </c>
+      <c r="H17" s="58"/>
       <c r="I17" s="17" t="s">
         <v>27</v>
       </c>
@@ -1388,10 +1462,14 @@
       <c r="D18" s="10">
         <v>-0.05</v>
       </c>
-      <c r="E18" s="58"/>
-      <c r="F18" s="59"/>
-      <c r="G18" s="59"/>
-      <c r="H18" s="59"/>
+      <c r="E18" s="57">
+        <v>0</v>
+      </c>
+      <c r="F18" s="58"/>
+      <c r="G18" s="58">
+        <v>0</v>
+      </c>
+      <c r="H18" s="58"/>
       <c r="I18" s="17" t="s">
         <v>28</v>
       </c>
@@ -1409,10 +1487,14 @@
       <c r="D19" s="9">
         <v>0</v>
       </c>
-      <c r="E19" s="58"/>
-      <c r="F19" s="59"/>
-      <c r="G19" s="59"/>
-      <c r="H19" s="59"/>
+      <c r="E19" s="57">
+        <v>0</v>
+      </c>
+      <c r="F19" s="58"/>
+      <c r="G19" s="58">
+        <v>0</v>
+      </c>
+      <c r="H19" s="58"/>
       <c r="I19" s="17" t="s">
         <v>29</v>
       </c>
@@ -1430,10 +1512,14 @@
       <c r="D20" s="9">
         <v>0</v>
       </c>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
-      <c r="G20" s="59"/>
-      <c r="H20" s="59"/>
+      <c r="E20" s="59">
+        <v>0</v>
+      </c>
+      <c r="F20" s="59"/>
+      <c r="G20" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H20" s="58"/>
       <c r="I20" s="17" t="s">
         <v>30</v>
       </c>
@@ -1451,10 +1537,14 @@
       <c r="D21" s="9">
         <v>0.09</v>
       </c>
-      <c r="E21" s="60"/>
-      <c r="F21" s="60"/>
-      <c r="G21" s="59"/>
-      <c r="H21" s="59"/>
+      <c r="E21" s="59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="59"/>
+      <c r="G21" s="58">
+        <v>1.95E-2</v>
+      </c>
+      <c r="H21" s="58"/>
       <c r="I21" s="17" t="s">
         <v>31</v>
       </c>
@@ -1472,10 +1562,14 @@
       <c r="D22" s="9">
         <v>0</v>
       </c>
-      <c r="E22" s="60"/>
-      <c r="F22" s="60"/>
-      <c r="G22" s="59"/>
-      <c r="H22" s="59"/>
+      <c r="E22" s="59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="59"/>
+      <c r="G22" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H22" s="58"/>
       <c r="I22" s="17" t="s">
         <v>32</v>
       </c>
@@ -1493,10 +1587,14 @@
       <c r="D23" s="9">
         <v>0.15</v>
       </c>
-      <c r="E23" s="60"/>
-      <c r="F23" s="60"/>
-      <c r="G23" s="59"/>
-      <c r="H23" s="59"/>
+      <c r="E23" s="59">
+        <v>3.0598E-2</v>
+      </c>
+      <c r="F23" s="59"/>
+      <c r="G23" s="58">
+        <v>7.0199999999999999E-2</v>
+      </c>
+      <c r="H23" s="58"/>
       <c r="I23" s="17" t="s">
         <v>33</v>
       </c>
@@ -1514,10 +1612,14 @@
       <c r="D24" s="9">
         <v>0</v>
       </c>
-      <c r="E24" s="60"/>
-      <c r="F24" s="60"/>
-      <c r="G24" s="59"/>
-      <c r="H24" s="59"/>
+      <c r="E24" s="59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="59"/>
+      <c r="G24" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H24" s="58"/>
       <c r="I24" s="17" t="s">
         <v>34</v>
       </c>
@@ -1535,10 +1637,14 @@
       <c r="D25" s="9">
         <v>0.18</v>
       </c>
-      <c r="E25" s="60"/>
-      <c r="F25" s="60"/>
-      <c r="G25" s="59"/>
-      <c r="H25" s="59"/>
+      <c r="E25" s="59">
+        <v>8.9997999999999995E-2</v>
+      </c>
+      <c r="F25" s="59"/>
+      <c r="G25" s="58">
+        <v>0.1</v>
+      </c>
+      <c r="H25" s="58"/>
       <c r="I25" s="17" t="s">
         <v>35</v>
       </c>
@@ -1556,10 +1662,14 @@
       <c r="D26" s="10">
         <v>-0.15</v>
       </c>
-      <c r="E26" s="60"/>
-      <c r="F26" s="58"/>
-      <c r="G26" s="59"/>
-      <c r="H26" s="59"/>
+      <c r="E26" s="59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="57"/>
+      <c r="G26" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H26" s="58"/>
       <c r="I26" s="19" t="s">
         <v>13</v>
       </c>
@@ -1577,10 +1687,14 @@
       <c r="D27" s="10">
         <v>-0.04</v>
       </c>
-      <c r="E27" s="58"/>
-      <c r="F27" s="59"/>
-      <c r="G27" s="59"/>
-      <c r="H27" s="59"/>
+      <c r="E27" s="57">
+        <v>0</v>
+      </c>
+      <c r="F27" s="58"/>
+      <c r="G27" s="58">
+        <v>0</v>
+      </c>
+      <c r="H27" s="58"/>
       <c r="I27" s="19" t="s">
         <v>37</v>
       </c>
@@ -1598,10 +1712,14 @@
       <c r="D28" s="9">
         <v>0</v>
       </c>
-      <c r="E28" s="58"/>
-      <c r="F28" s="59"/>
-      <c r="G28" s="59"/>
-      <c r="H28" s="59"/>
+      <c r="E28" s="57">
+        <v>0</v>
+      </c>
+      <c r="F28" s="58"/>
+      <c r="G28" s="58">
+        <v>0</v>
+      </c>
+      <c r="H28" s="58"/>
       <c r="I28" s="19" t="s">
         <v>38</v>
       </c>
@@ -1619,10 +1737,14 @@
       <c r="D29" s="9">
         <v>0</v>
       </c>
-      <c r="E29" s="58"/>
-      <c r="F29" s="59"/>
-      <c r="G29" s="59"/>
-      <c r="H29" s="59"/>
+      <c r="E29" s="57">
+        <v>0</v>
+      </c>
+      <c r="F29" s="58"/>
+      <c r="G29" s="58">
+        <v>0</v>
+      </c>
+      <c r="H29" s="58"/>
       <c r="I29" s="19" t="s">
         <v>39</v>
       </c>
@@ -1640,10 +1762,14 @@
       <c r="D30" s="9">
         <v>0.05</v>
       </c>
-      <c r="E30" s="58"/>
-      <c r="F30" s="59"/>
-      <c r="G30" s="59"/>
-      <c r="H30" s="59"/>
+      <c r="E30" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" s="58"/>
+      <c r="G30" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H30" s="58"/>
       <c r="I30" s="19" t="s">
         <v>40</v>
       </c>
@@ -1661,10 +1787,14 @@
       <c r="D31" s="9">
         <v>0</v>
       </c>
-      <c r="E31" s="59"/>
-      <c r="F31" s="59"/>
-      <c r="G31" s="59"/>
-      <c r="H31" s="60"/>
+      <c r="E31" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" s="58"/>
+      <c r="G31" s="58">
+        <v>0</v>
+      </c>
+      <c r="H31" s="59"/>
       <c r="I31" s="19" t="s">
         <v>41</v>
       </c>
@@ -1682,10 +1812,14 @@
       <c r="D32" s="9">
         <v>0.05</v>
       </c>
-      <c r="E32" s="60"/>
-      <c r="F32" s="59"/>
-      <c r="G32" s="59"/>
-      <c r="H32" s="60"/>
+      <c r="E32" s="59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" s="58"/>
+      <c r="G32" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H32" s="59"/>
       <c r="I32" s="19" t="s">
         <v>42</v>
       </c>
@@ -1703,10 +1837,14 @@
       <c r="D33" s="9">
         <v>0</v>
       </c>
-      <c r="E33" s="58"/>
-      <c r="F33" s="59"/>
-      <c r="G33" s="59"/>
-      <c r="H33" s="59"/>
+      <c r="E33" s="57">
+        <v>0</v>
+      </c>
+      <c r="F33" s="58"/>
+      <c r="G33" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H33" s="58"/>
       <c r="I33" s="20" t="s">
         <v>43</v>
       </c>
@@ -1724,10 +1862,14 @@
       <c r="D34" s="9">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E34" s="58"/>
-      <c r="F34" s="59"/>
-      <c r="G34" s="59"/>
-      <c r="H34" s="61"/>
+      <c r="E34" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="58"/>
+      <c r="G34" s="58">
+        <v>0.09</v>
+      </c>
+      <c r="H34" s="60"/>
       <c r="I34" s="20" t="s">
         <v>44</v>
       </c>
@@ -1745,10 +1887,14 @@
       <c r="D35" s="9">
         <v>0</v>
       </c>
-      <c r="E35" s="58"/>
-      <c r="F35" s="59"/>
-      <c r="G35" s="59"/>
-      <c r="H35" s="60"/>
+      <c r="E35" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="58"/>
+      <c r="G35" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H35" s="59"/>
       <c r="I35" s="20" t="s">
         <v>45</v>
       </c>
@@ -1766,10 +1912,14 @@
       <c r="D36" s="9">
         <v>0.09</v>
       </c>
-      <c r="E36" s="58"/>
-      <c r="F36" s="60"/>
-      <c r="G36" s="59"/>
-      <c r="H36" s="60"/>
+      <c r="E36" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" s="59"/>
+      <c r="G36" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H36" s="59"/>
       <c r="I36" s="20" t="s">
         <v>46</v>
       </c>
@@ -1787,10 +1937,14 @@
       <c r="D37" s="9">
         <v>0</v>
       </c>
-      <c r="E37" s="60"/>
-      <c r="F37" s="60"/>
-      <c r="G37" s="59"/>
-      <c r="H37" s="60"/>
+      <c r="E37" s="59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F37" s="59"/>
+      <c r="G37" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H37" s="59"/>
       <c r="I37" s="20" t="s">
         <v>47</v>
       </c>
@@ -1808,10 +1962,14 @@
       <c r="D38" s="9">
         <v>0.18</v>
       </c>
-      <c r="E38" s="60"/>
-      <c r="F38" s="60"/>
-      <c r="G38" s="59"/>
-      <c r="H38" s="60"/>
+      <c r="E38" s="59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F38" s="59"/>
+      <c r="G38" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H38" s="59"/>
       <c r="I38" s="20" t="s">
         <v>48</v>
       </c>
@@ -1829,10 +1987,14 @@
       <c r="D39" s="10">
         <v>-0.15</v>
       </c>
-      <c r="E39" s="58"/>
-      <c r="F39" s="58"/>
-      <c r="G39" s="59"/>
-      <c r="H39" s="59"/>
+      <c r="E39" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39" s="57"/>
+      <c r="G39" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H39" s="58"/>
       <c r="I39" s="22" t="s">
         <v>13</v>
       </c>
@@ -1850,10 +2012,14 @@
       <c r="D40" s="10">
         <v>-0.04</v>
       </c>
-      <c r="E40" s="58"/>
-      <c r="F40" s="59"/>
-      <c r="G40" s="59"/>
-      <c r="H40" s="59"/>
+      <c r="E40" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F40" s="58"/>
+      <c r="G40" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H40" s="58"/>
       <c r="I40" s="22" t="s">
         <v>50</v>
       </c>
@@ -1871,10 +2037,14 @@
       <c r="D41" s="9">
         <v>0</v>
       </c>
-      <c r="E41" s="58"/>
-      <c r="F41" s="59"/>
-      <c r="G41" s="59"/>
-      <c r="H41" s="59"/>
+      <c r="E41" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41" s="58"/>
+      <c r="G41" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H41" s="58"/>
       <c r="I41" s="22" t="s">
         <v>51</v>
       </c>
@@ -1892,10 +2062,14 @@
       <c r="D42" s="9">
         <v>0</v>
       </c>
-      <c r="E42" s="58"/>
-      <c r="F42" s="59"/>
-      <c r="G42" s="59"/>
-      <c r="H42" s="59"/>
+      <c r="E42" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F42" s="58"/>
+      <c r="G42" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H42" s="58"/>
       <c r="I42" s="22" t="s">
         <v>52</v>
       </c>
@@ -1913,10 +2087,14 @@
       <c r="D43" s="9">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E43" s="58"/>
-      <c r="F43" s="59"/>
-      <c r="G43" s="59"/>
-      <c r="H43" s="59"/>
+      <c r="E43" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F43" s="58"/>
+      <c r="G43" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H43" s="58"/>
       <c r="I43" s="22" t="s">
         <v>53</v>
       </c>
@@ -1934,10 +2112,14 @@
       <c r="D44" s="9">
         <v>0</v>
       </c>
-      <c r="E44" s="58"/>
-      <c r="F44" s="59"/>
-      <c r="G44" s="59"/>
-      <c r="H44" s="60"/>
+      <c r="E44" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F44" s="58"/>
+      <c r="G44" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H44" s="59"/>
       <c r="I44" s="23" t="s">
         <v>54</v>
       </c>
@@ -1955,10 +2137,14 @@
       <c r="D45" s="9">
         <v>0.12</v>
       </c>
-      <c r="E45" s="58"/>
-      <c r="F45" s="60"/>
-      <c r="G45" s="59"/>
-      <c r="H45" s="59"/>
+      <c r="E45" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F45" s="59"/>
+      <c r="G45" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H45" s="58"/>
       <c r="I45" s="22" t="s">
         <v>55</v>
       </c>
@@ -1976,10 +2162,14 @@
       <c r="D46" s="9">
         <v>0.25</v>
       </c>
-      <c r="E46" s="60"/>
-      <c r="F46" s="60"/>
-      <c r="G46" s="59"/>
-      <c r="H46" s="60"/>
+      <c r="E46" s="59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F46" s="59"/>
+      <c r="G46" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H46" s="59"/>
       <c r="I46" s="23" t="s">
         <v>56</v>
       </c>
@@ -1997,10 +2187,14 @@
       <c r="D47" s="9">
         <v>0.39</v>
       </c>
-      <c r="E47" s="60"/>
-      <c r="F47" s="60"/>
-      <c r="G47" s="59"/>
-      <c r="H47" s="60"/>
+      <c r="E47" s="59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F47" s="59"/>
+      <c r="G47" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H47" s="59"/>
       <c r="I47" s="23" t="s">
         <v>57</v>
       </c>
@@ -2018,10 +2212,14 @@
       <c r="D48" s="10">
         <v>-0.04</v>
       </c>
-      <c r="E48" s="58"/>
-      <c r="F48" s="58"/>
-      <c r="G48" s="59"/>
-      <c r="H48" s="59"/>
+      <c r="E48" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F48" s="57"/>
+      <c r="G48" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H48" s="58"/>
       <c r="I48" s="25" t="s">
         <v>59</v>
       </c>
@@ -2039,10 +2237,14 @@
       <c r="D49" s="9">
         <v>0</v>
       </c>
-      <c r="E49" s="58"/>
-      <c r="F49" s="58"/>
-      <c r="G49" s="59"/>
-      <c r="H49" s="59"/>
+      <c r="E49" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F49" s="57"/>
+      <c r="G49" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H49" s="58"/>
       <c r="I49" s="25" t="s">
         <v>60</v>
       </c>
@@ -2060,10 +2262,14 @@
       <c r="D50" s="9">
         <v>0</v>
       </c>
-      <c r="E50" s="58"/>
-      <c r="F50" s="58"/>
-      <c r="G50" s="59"/>
-      <c r="H50" s="59"/>
+      <c r="E50" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F50" s="57"/>
+      <c r="G50" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H50" s="58"/>
       <c r="I50" s="25" t="s">
         <v>61</v>
       </c>
@@ -2081,10 +2287,14 @@
       <c r="D51" s="9">
         <v>0.05</v>
       </c>
-      <c r="E51" s="58"/>
-      <c r="F51" s="58"/>
-      <c r="G51" s="59"/>
-      <c r="H51" s="59"/>
+      <c r="E51" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F51" s="57"/>
+      <c r="G51" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H51" s="58"/>
       <c r="I51" s="25" t="s">
         <v>62</v>
       </c>
@@ -2102,10 +2312,14 @@
       <c r="D52" s="9">
         <v>0</v>
       </c>
-      <c r="E52" s="58"/>
-      <c r="F52" s="58"/>
-      <c r="G52" s="59"/>
-      <c r="H52" s="59"/>
+      <c r="E52" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F52" s="57"/>
+      <c r="G52" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H52" s="58"/>
       <c r="I52" s="25" t="s">
         <v>63</v>
       </c>
@@ -2123,10 +2337,14 @@
       <c r="D53" s="9">
         <v>0.12</v>
       </c>
-      <c r="E53" s="60"/>
-      <c r="F53" s="58"/>
-      <c r="G53" s="59"/>
-      <c r="H53" s="59"/>
+      <c r="E53" s="59" t="s">
+        <v>11</v>
+      </c>
+      <c r="F53" s="57"/>
+      <c r="G53" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H53" s="58"/>
       <c r="I53" s="25" t="s">
         <v>64</v>
       </c>
@@ -2144,10 +2362,14 @@
       <c r="D54" s="10">
         <v>-7.0000000000000007E-2</v>
       </c>
-      <c r="E54" s="58"/>
-      <c r="F54" s="60"/>
-      <c r="G54" s="59"/>
-      <c r="H54" s="59"/>
+      <c r="E54" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F54" s="59"/>
+      <c r="G54" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H54" s="58"/>
       <c r="I54" s="27" t="s">
         <v>66</v>
       </c>
@@ -2165,10 +2387,14 @@
       <c r="D55" s="9">
         <v>0</v>
       </c>
-      <c r="E55" s="58"/>
-      <c r="F55" s="58"/>
-      <c r="G55" s="59"/>
-      <c r="H55" s="59"/>
+      <c r="E55" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F55" s="57"/>
+      <c r="G55" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H55" s="58"/>
       <c r="I55" s="27" t="s">
         <v>67</v>
       </c>
@@ -2186,10 +2412,14 @@
       <c r="D56" s="9">
         <v>0.06</v>
       </c>
-      <c r="E56" s="58"/>
-      <c r="F56" s="58"/>
-      <c r="G56" s="59"/>
-      <c r="H56" s="59"/>
+      <c r="E56" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F56" s="57"/>
+      <c r="G56" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H56" s="58"/>
       <c r="I56" s="27" t="s">
         <v>68</v>
       </c>
@@ -2207,10 +2437,14 @@
       <c r="D57" s="10">
         <v>-0.09</v>
       </c>
-      <c r="E57" s="58"/>
-      <c r="F57" s="58"/>
-      <c r="G57" s="59"/>
-      <c r="H57" s="59"/>
+      <c r="E57" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F57" s="57"/>
+      <c r="G57" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H57" s="58"/>
       <c r="I57" s="29" t="s">
         <v>66</v>
       </c>
@@ -2228,10 +2462,14 @@
       <c r="D58" s="10">
         <v>-0.04</v>
       </c>
-      <c r="E58" s="58"/>
-      <c r="F58" s="58"/>
-      <c r="G58" s="59"/>
-      <c r="H58" s="59"/>
+      <c r="E58" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F58" s="57"/>
+      <c r="G58" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H58" s="58"/>
       <c r="I58" s="29" t="s">
         <v>70</v>
       </c>
@@ -2249,10 +2487,14 @@
       <c r="D59" s="9">
         <v>0</v>
       </c>
-      <c r="E59" s="58"/>
-      <c r="F59" s="58"/>
-      <c r="G59" s="59"/>
-      <c r="H59" s="59"/>
+      <c r="E59" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F59" s="57"/>
+      <c r="G59" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H59" s="58"/>
       <c r="I59" s="29" t="s">
         <v>71</v>
       </c>
@@ -2270,10 +2512,14 @@
       <c r="D60" s="9">
         <v>0</v>
       </c>
-      <c r="E60" s="58"/>
-      <c r="F60" s="58"/>
-      <c r="G60" s="59"/>
-      <c r="H60" s="59"/>
+      <c r="E60" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F60" s="57"/>
+      <c r="G60" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H60" s="58"/>
       <c r="I60" s="29" t="s">
         <v>72</v>
       </c>
@@ -2291,10 +2537,14 @@
       <c r="D61" s="9">
         <v>0.05</v>
       </c>
-      <c r="E61" s="58"/>
-      <c r="F61" s="60"/>
-      <c r="G61" s="59"/>
-      <c r="H61" s="59"/>
+      <c r="E61" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F61" s="59"/>
+      <c r="G61" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H61" s="58"/>
       <c r="I61" s="29" t="s">
         <v>73</v>
       </c>
@@ -2312,10 +2562,14 @@
       <c r="D62" s="9">
         <v>0</v>
       </c>
-      <c r="E62" s="58"/>
-      <c r="F62" s="60"/>
-      <c r="G62" s="59"/>
-      <c r="H62" s="59"/>
+      <c r="E62" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F62" s="59"/>
+      <c r="G62" s="58" t="s">
+        <v>11</v>
+      </c>
+      <c r="H62" s="58"/>
       <c r="I62" s="29" t="s">
         <v>74</v>
       </c>
@@ -2333,10 +2587,14 @@
       <c r="D63" s="9">
         <v>0.15</v>
       </c>
-      <c r="E63" s="58"/>
-      <c r="F63" s="58"/>
-      <c r="G63" s="61"/>
-      <c r="H63" s="60"/>
+      <c r="E63" s="57" t="s">
+        <v>11</v>
+      </c>
+      <c r="F63" s="57"/>
+      <c r="G63" s="60" t="s">
+        <v>11</v>
+      </c>
+      <c r="H63" s="59"/>
       <c r="I63" s="31" t="s">
         <v>75</v>
       </c>
@@ -2417,103 +2675,108 @@
   <cols>
     <col min="1" max="1" width="21.26953125" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="4" max="4" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2"/>
       <c r="B1" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="C1" s="65" t="s">
+      <c r="C1" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="64"/>
-      <c r="E1" s="67" t="s">
+      <c r="D1" s="63"/>
+      <c r="E1" s="66" t="s">
         <v>81</v>
       </c>
-      <c r="F1" s="64"/>
-      <c r="G1" s="66" t="s">
+      <c r="F1" s="63"/>
+      <c r="G1" s="65" t="s">
         <v>82</v>
       </c>
-      <c r="H1" s="64"/>
-      <c r="I1" s="70" t="s">
+      <c r="H1" s="63"/>
+      <c r="I1" s="69" t="s">
         <v>83</v>
       </c>
-      <c r="J1" s="64"/>
-      <c r="K1" s="68" t="s">
-        <v>3</v>
-      </c>
-      <c r="L1" s="69"/>
-    </row>
-    <row r="2" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J1" s="63"/>
+      <c r="K1" s="67" t="s">
+        <v>84</v>
+      </c>
+      <c r="L1" s="68"/>
+    </row>
+    <row r="2" spans="1:13" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1"/>
-      <c r="B2" s="57">
-        <v>275706.34000000003</v>
+      <c r="B2" s="70" t="s">
+        <v>87</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="37" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="38" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="39" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="40" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K2" s="2"/>
       <c r="L2" s="41" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B3" s="42" t="s">
         <v>9</v>
       </c>
       <c r="C3" s="43">
         <f>Datos!E4</f>
-        <v>0</v>
-      </c>
-      <c r="D3" s="9">
-        <f>(C3/$B$2)-1</f>
-        <v>-1</v>
+        <v>55499</v>
+      </c>
+      <c r="D3" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),(C3/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E3" s="44">
         <f>Datos!F4</f>
         <v>0</v>
       </c>
-      <c r="F3" s="9">
-        <f>(E3/$B$2)-1</f>
-        <v>-1</v>
+      <c r="F3" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),(E3/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G3" s="45">
         <f>Datos!G4</f>
-        <v>0</v>
-      </c>
-      <c r="H3" s="9">
-        <f>(G3/$B$2)-1</f>
-        <v>-1</v>
+        <v>58608</v>
+      </c>
+      <c r="H3" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),(G3/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I3" s="46">
         <f>Datos!H4</f>
         <v>0</v>
       </c>
-      <c r="J3" s="9">
-        <f>(I3/$B$2)-1</f>
-        <v>-1</v>
+      <c r="J3" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),(I3/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K3" s="47"/>
-      <c r="L3" s="9">
-        <f>(K3/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L3" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),(K3/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="M3" s="36">
         <f>K3*0.05</f>
@@ -2533,40 +2796,40 @@
         <v>-</v>
       </c>
       <c r="D4" s="9" t="str">
-        <f>IF(ISNUMBER(C4),((C4*Datos!$B5)/(1+Datos!$C5)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C4),ISNUMBER($B$2)),((C4*Datos!$B5)/(1+Datos!$C5)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E4" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F5),$E$3*(1-Datos!F5)/Datos!B5,"-")</f>
         <v>-</v>
       </c>
       <c r="F4" s="9" t="str">
-        <f>IF(ISNUMBER(E4),((E4*Datos!$B5)/(1+Datos!$C5)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E4),ISNUMBER($B$2)),((E4*Datos!$B5)/(1+Datos!$C5)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G4" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G5),$G$3*(1-Datos!G5)/Datos!B5,"-")</f>
         <v>-</v>
       </c>
       <c r="H4" s="9" t="str">
-        <f>IF(ISNUMBER(G4),((G4*Datos!$B5)/(1+Datos!$C5)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="I4" s="71" t="str">
+        <f>IF(AND(ISNUMBER(G4),ISNUMBER($B$2)),((G4*Datos!$B5)/(1+Datos!$C5)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="I4" s="8" t="str">
         <f>IF(ISNUMBER(Datos!H5),$I$3*(1-Datos!H5)/Datos!B5,"-")</f>
         <v>-</v>
       </c>
       <c r="J4" s="9" t="str">
-        <f>IF(ISNUMBER(I4),((I4*Datos!$B5)/(1+Datos!$C5)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I4),ISNUMBER($B$2)),((I4*Datos!$B5)/(1+Datos!$C5)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K4" s="48">
         <f>$K$3*(1+Datos!D5)/Datos!B5</f>
         <v>0</v>
       </c>
-      <c r="L4" s="9">
-        <f>((K4*Datos!$B5)/(1+Datos!$C5)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L4" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K4*Datos!$B5)/(1+Datos!$C5)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2582,40 +2845,40 @@
         <v>-</v>
       </c>
       <c r="D5" s="9" t="str">
-        <f>IF(ISNUMBER(C5),((C5*Datos!$B6)/(1+Datos!$C6)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C5),ISNUMBER($B$2)),((C5*Datos!$B6)/(1+Datos!$C6)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E5" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F6),$E$3*(1+Datos!F6)/Datos!B6,"-")</f>
         <v>-</v>
       </c>
       <c r="F5" s="9" t="str">
-        <f>IF(ISNUMBER(E5),((E5*Datos!$B6)/(1+Datos!$C6)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G5" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E5),ISNUMBER($B$2)),((E5*Datos!$B6)/(1+Datos!$C6)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G5" s="48">
         <f>IF(ISNUMBER(Datos!G6),$G$3*(1+Datos!G6)/Datos!B6,"-")</f>
-        <v>-</v>
+        <v>19536</v>
       </c>
       <c r="H5" s="9" t="str">
-        <f>IF(ISNUMBER(G5),((G5*Datos!$B6)/(1+Datos!$C6)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G5),ISNUMBER($B$2)),((G5*Datos!$B6)/(1+Datos!$C6)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I5" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H6),$I$3*(1+Datos!H6)/Datos!B6,"-")</f>
         <v>-</v>
       </c>
       <c r="J5" s="9" t="str">
-        <f>IF(ISNUMBER(I5),((I5*Datos!$B6)/(1+Datos!$C6)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I5),ISNUMBER($B$2)),((I5*Datos!$B6)/(1+Datos!$C6)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K5" s="48">
         <f>$K$3*(1+Datos!D6)/Datos!B6</f>
         <v>0</v>
       </c>
-      <c r="L5" s="9">
-        <f>((K5*Datos!$B6)/(1+Datos!$C6)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L5" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K5*Datos!$B6)/(1+Datos!$C6)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2631,40 +2894,40 @@
         <v>-</v>
       </c>
       <c r="D6" s="9" t="str">
-        <f>IF(ISNUMBER(C6),((C6*Datos!$B7)/(1+Datos!$C7)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C6),ISNUMBER($B$2)),((C6*Datos!$B7)/(1+Datos!$C7)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E6" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F7),$E$3*(1+Datos!F7)/Datos!B7,"-")</f>
         <v>-</v>
       </c>
       <c r="F6" s="9" t="str">
-        <f>IF(ISNUMBER(E6),((E6*Datos!$B7)/(1+Datos!$C7)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G6" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E6),ISNUMBER($B$2)),((E6*Datos!$B7)/(1+Datos!$C7)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G6" s="48">
         <f>IF(ISNUMBER(Datos!G7),$G$3*(1+Datos!G7)/Datos!B7,"-")</f>
-        <v>-</v>
+        <v>9768</v>
       </c>
       <c r="H6" s="9" t="str">
-        <f>IF(ISNUMBER(G6),((G6*Datos!$B7)/(1+Datos!$C7)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G6),ISNUMBER($B$2)),((G6*Datos!$B7)/(1+Datos!$C7)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I6" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H7),$I$3*(1+Datos!H7)/Datos!B7,"-")</f>
         <v>-</v>
       </c>
       <c r="J6" s="9" t="str">
-        <f>IF(ISNUMBER(I6),((I6*Datos!$B7)/(1+Datos!$C7)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I6),ISNUMBER($B$2)),((I6*Datos!$B7)/(1+Datos!$C7)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K6" s="48">
         <f>$K$3*(1+Datos!D7)/Datos!B7</f>
         <v>0</v>
       </c>
-      <c r="L6" s="9">
-        <f>((K6*Datos!$B7)/(1+Datos!$C7)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L6" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K6*Datos!$B7)/(1+Datos!$C7)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2680,40 +2943,40 @@
         <v>-</v>
       </c>
       <c r="D7" s="9" t="str">
-        <f>IF(ISNUMBER(C7),((C7*Datos!$B8)/(1+Datos!$C8)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C7),ISNUMBER($B$2)),((C7*Datos!$B8)/(1+Datos!$C8)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E7" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F8),$E$3*(1+Datos!F8)/Datos!B8,"-")</f>
         <v>-</v>
       </c>
       <c r="F7" s="9" t="str">
-        <f>IF(ISNUMBER(E7),((E7*Datos!$B8)/(1+Datos!$C8)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G7" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E7),ISNUMBER($B$2)),((E7*Datos!$B8)/(1+Datos!$C8)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G7" s="48">
         <f>IF(ISNUMBER(Datos!G8),$G$3*(1+Datos!G8)/Datos!B8,"-")</f>
-        <v>-</v>
+        <v>6512</v>
       </c>
       <c r="H7" s="9" t="str">
-        <f>IF(ISNUMBER(G7),((G7*Datos!$B8)/(1+Datos!$C8)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G7),ISNUMBER($B$2)),((G7*Datos!$B8)/(1+Datos!$C8)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I7" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H8),$I$3*(1+Datos!H8)/Datos!B8,"-")</f>
         <v>-</v>
       </c>
       <c r="J7" s="9" t="str">
-        <f>IF(ISNUMBER(I7),((I7*Datos!$B8)/(1+Datos!$C8)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I7),ISNUMBER($B$2)),((I7*Datos!$B8)/(1+Datos!$C8)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K7" s="48">
         <f>$K$3*(1+Datos!D8)/Datos!B8</f>
         <v>0</v>
       </c>
-      <c r="L7" s="9">
-        <f>((K7*Datos!$B8)/(1+Datos!$C8)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L7" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K7*Datos!$B8)/(1+Datos!$C8)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2729,40 +2992,40 @@
         <v>-</v>
       </c>
       <c r="D8" s="9" t="str">
-        <f>IF(ISNUMBER(C8),((C8*Datos!$B9)/(1+Datos!$C9)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C8),ISNUMBER($B$2)),((C8*Datos!$B9)/(1+Datos!$C9)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E8" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F9),$E$3*(1+Datos!F9)/Datos!B9,"-")</f>
         <v>-</v>
       </c>
       <c r="F8" s="9" t="str">
-        <f>IF(ISNUMBER(E8),((E8*Datos!$B9)/(1+Datos!$C9)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E8),ISNUMBER($B$2)),((E8*Datos!$B9)/(1+Datos!$C9)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G8" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G9),$G$3*(1+Datos!G9)/Datos!B9,"-")</f>
         <v>-</v>
       </c>
       <c r="H8" s="9" t="str">
-        <f>IF(ISNUMBER(G8),((G8*Datos!$B9)/(1+Datos!$C9)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G8),ISNUMBER($B$2)),((G8*Datos!$B9)/(1+Datos!$C9)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I8" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H9),$I$3*(1+Datos!H9)/Datos!B9,"-")</f>
         <v>-</v>
       </c>
       <c r="J8" s="9" t="str">
-        <f>IF(ISNUMBER(I8),((I8*Datos!$B9)/(1+Datos!$C9)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I8),ISNUMBER($B$2)),((I8*Datos!$B9)/(1+Datos!$C9)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K8" s="48">
         <f>$K$3*(1+Datos!D9)/Datos!B9</f>
         <v>0</v>
       </c>
-      <c r="L8" s="9">
-        <f>((K8*Datos!$B9)/(1+Datos!$C9)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L8" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K8*Datos!$B9)/(1+Datos!$C9)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2778,40 +3041,40 @@
         <v>-</v>
       </c>
       <c r="D9" s="9" t="str">
-        <f>IF(ISNUMBER(C9),((C9*Datos!$B10)/(1+Datos!$C10)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C9),ISNUMBER($B$2)),((C9*Datos!$B10)/(1+Datos!$C10)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E9" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F10),$E$3*(1+Datos!F10)/Datos!B10,"-")</f>
         <v>-</v>
       </c>
       <c r="F9" s="9" t="str">
-        <f>IF(ISNUMBER(E9),((E9*Datos!$B10)/(1+Datos!$C10)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G9" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E9),ISNUMBER($B$2)),((E9*Datos!$B10)/(1+Datos!$C10)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G9" s="48">
         <f>IF(ISNUMBER(Datos!G10),$G$3*(1+Datos!G10)/Datos!B10,"-")</f>
-        <v>-</v>
+        <v>4884</v>
       </c>
       <c r="H9" s="9" t="str">
-        <f>IF(ISNUMBER(G9),((G9*Datos!$B10)/(1+Datos!$C10)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G9),ISNUMBER($B$2)),((G9*Datos!$B10)/(1+Datos!$C10)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I9" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H10),$I$3*(1+Datos!H10)/Datos!B10,"-")</f>
         <v>-</v>
       </c>
       <c r="J9" s="9" t="str">
-        <f>IF(ISNUMBER(I9),((I9*Datos!$B10)/(1+Datos!$C10)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I9),ISNUMBER($B$2)),((I9*Datos!$B10)/(1+Datos!$C10)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K9" s="48">
         <f>$K$3*(1+Datos!D10)/Datos!B10</f>
         <v>0</v>
       </c>
-      <c r="L9" s="9">
-        <f>((K9*Datos!$B10)/(1+Datos!$C10)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L9" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K9*Datos!$B10)/(1+Datos!$C10)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2827,40 +3090,40 @@
         <v>-</v>
       </c>
       <c r="D10" s="9" t="str">
-        <f>IF(ISNUMBER(C10),((C10*Datos!$B11)/(1+Datos!$C11)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C10),ISNUMBER($B$2)),((C10*Datos!$B11)/(1+Datos!$C11)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E10" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F11),$E$3*(1+Datos!F11)/Datos!B11,"-")</f>
         <v>-</v>
       </c>
       <c r="F10" s="9" t="str">
-        <f>IF(ISNUMBER(E10),((E10*Datos!$B11)/(1+Datos!$C11)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E10),ISNUMBER($B$2)),((E10*Datos!$B11)/(1+Datos!$C11)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G10" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G11),$G$3*(1+Datos!G11)/Datos!B11,"-")</f>
         <v>-</v>
       </c>
       <c r="H10" s="9" t="str">
-        <f>IF(ISNUMBER(G10),((G10*Datos!$B11)/(1+Datos!$C11)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G10),ISNUMBER($B$2)),((G10*Datos!$B11)/(1+Datos!$C11)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I10" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H11),$I$3*(1+Datos!H11)/Datos!B11,"-")</f>
         <v>-</v>
       </c>
       <c r="J10" s="9" t="str">
-        <f>IF(ISNUMBER(I10),((I10*Datos!$B11)/(1+Datos!$C11)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I10),ISNUMBER($B$2)),((I10*Datos!$B11)/(1+Datos!$C11)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K10" s="48">
         <f>$K$3*(1+Datos!D11)/Datos!B11</f>
         <v>0</v>
       </c>
-      <c r="L10" s="9">
-        <f>((K10*Datos!$B11)/(1+Datos!$C11)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L10" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K10*Datos!$B11)/(1+Datos!$C11)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2876,40 +3139,40 @@
         <v>-</v>
       </c>
       <c r="D11" s="9" t="str">
-        <f>IF(ISNUMBER(C11),((C11*Datos!$B12)/(1+Datos!$C12)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C11),ISNUMBER($B$2)),((C11*Datos!$B12)/(1+Datos!$C12)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E11" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F12),$E$3*(1+Datos!F12)/Datos!B12,"-")</f>
         <v>-</v>
       </c>
       <c r="F11" s="9" t="str">
-        <f>IF(ISNUMBER(E11),((E11*Datos!$B12)/(1+Datos!$C12)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E11),ISNUMBER($B$2)),((E11*Datos!$B12)/(1+Datos!$C12)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G11" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G12),$G$3*(1+Datos!G12)/Datos!B12,"-")</f>
         <v>-</v>
       </c>
       <c r="H11" s="9" t="str">
-        <f>IF(ISNUMBER(G11),((G11*Datos!$B12)/(1+Datos!$C12)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G11),ISNUMBER($B$2)),((G11*Datos!$B12)/(1+Datos!$C12)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I11" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H12),$I$3*(1+Datos!H12)/Datos!B12,"-")</f>
         <v>-</v>
       </c>
       <c r="J11" s="9" t="str">
-        <f>IF(ISNUMBER(I11),((I11*Datos!$B12)/(1+Datos!$C12)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I11),ISNUMBER($B$2)),((I11*Datos!$B12)/(1+Datos!$C12)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K11" s="48">
         <f>$K$3*(1+Datos!D12)/Datos!B12</f>
         <v>0</v>
       </c>
-      <c r="L11" s="9">
-        <f>((K11*Datos!$B12)/(1+Datos!$C12)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L11" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K11*Datos!$B12)/(1+Datos!$C12)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2925,40 +3188,40 @@
         <v>-</v>
       </c>
       <c r="D12" s="9" t="str">
-        <f>IF(ISNUMBER(C12),((C12*Datos!$B13)/(1+Datos!$C13)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C12),ISNUMBER($B$2)),((C12*Datos!$B13)/(1+Datos!$C13)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E12" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F13),$E$3*(1+Datos!F13)/Datos!B13,"-")</f>
         <v>-</v>
       </c>
       <c r="F12" s="9" t="str">
-        <f>IF(ISNUMBER(E12),((E12*Datos!$B13)/(1+Datos!$C13)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G12" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E12),ISNUMBER($B$2)),((E12*Datos!$B13)/(1+Datos!$C13)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G12" s="48">
         <f>IF(ISNUMBER(Datos!G13),$G$3*(1+Datos!G13)/Datos!B13,"-")</f>
-        <v>-</v>
+        <v>3983.3904000000007</v>
       </c>
       <c r="H12" s="9" t="str">
-        <f>IF(ISNUMBER(G12),((G12*Datos!$B13)/(1+Datos!$C13)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G12),ISNUMBER($B$2)),((G12*Datos!$B13)/(1+Datos!$C13)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I12" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H13),$I$3*(1+Datos!H13)/Datos!B13,"-")</f>
         <v>-</v>
       </c>
       <c r="J12" s="9" t="str">
-        <f>IF(ISNUMBER(I12),((I12*Datos!$B13)/(1+Datos!$C13)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I12),ISNUMBER($B$2)),((I12*Datos!$B13)/(1+Datos!$C13)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K12" s="48">
         <f>$K$3*(1+Datos!D13)/Datos!B13</f>
         <v>0</v>
       </c>
-      <c r="L12" s="9">
-        <f>((K12*Datos!$B13)/(1+Datos!$C13)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L12" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K12*Datos!$B13)/(1+Datos!$C13)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2974,40 +3237,40 @@
         <v>-</v>
       </c>
       <c r="D13" s="9" t="str">
-        <f>IF(ISNUMBER(C13),((C13*Datos!$B14)/(1+Datos!$C14)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C13),ISNUMBER($B$2)),((C13*Datos!$B14)/(1+Datos!$C14)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E13" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F14),$E$3*(1+Datos!F14)/Datos!B14,"-")</f>
         <v>-</v>
       </c>
       <c r="F13" s="9" t="str">
-        <f>IF(ISNUMBER(E13),((E13*Datos!$B14)/(1+Datos!$C14)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E13),ISNUMBER($B$2)),((E13*Datos!$B14)/(1+Datos!$C14)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G13" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G14),$G$3*(1+Datos!G14)/Datos!B14,"-")</f>
         <v>-</v>
       </c>
       <c r="H13" s="9" t="str">
-        <f>IF(ISNUMBER(G13),((G13*Datos!$B14)/(1+Datos!$C14)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G13),ISNUMBER($B$2)),((G13*Datos!$B14)/(1+Datos!$C14)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I13" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H14),$I$3*(1+Datos!H14)/Datos!B14,"-")</f>
         <v>-</v>
       </c>
       <c r="J13" s="9" t="str">
-        <f>IF(ISNUMBER(I13),((I13*Datos!$B14)/(1+Datos!$C14)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I13),ISNUMBER($B$2)),((I13*Datos!$B14)/(1+Datos!$C14)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K13" s="48">
         <f>$K$3*(1+Datos!D14)/Datos!B14</f>
         <v>0</v>
       </c>
-      <c r="L13" s="9">
-        <f>((K13*Datos!$B14)/(1+Datos!$C14)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L13" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K13*Datos!$B14)/(1+Datos!$C14)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3023,40 +3286,40 @@
         <v>-</v>
       </c>
       <c r="D14" s="9" t="str">
-        <f>IF(ISNUMBER(C14),((C14*Datos!$B15)/(1+Datos!$C15)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C14),ISNUMBER($B$2)),((C14*Datos!$B15)/(1+Datos!$C15)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E14" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F15),$E$3*(1+Datos!F15)/Datos!B15,"-")</f>
         <v>-</v>
       </c>
       <c r="F14" s="9" t="str">
-        <f>IF(ISNUMBER(E14),((E14*Datos!$B15)/(1+Datos!$C15)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G14" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E14),ISNUMBER($B$2)),((E14*Datos!$B15)/(1+Datos!$C15)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G14" s="48">
         <f>IF(ISNUMBER(Datos!G15),$G$3*(1+Datos!G15)/Datos!B15,"-")</f>
-        <v>-</v>
+        <v>3484.5712000000003</v>
       </c>
       <c r="H14" s="9" t="str">
-        <f>IF(ISNUMBER(G14),((G14*Datos!$B15)/(1+Datos!$C15)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G14),ISNUMBER($B$2)),((G14*Datos!$B15)/(1+Datos!$C15)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I14" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H15),$I$3*(1+Datos!H15)/Datos!B15,"-")</f>
         <v>-</v>
       </c>
       <c r="J14" s="9" t="str">
-        <f>IF(ISNUMBER(I14),((I14*Datos!$B15)/(1+Datos!$C15)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I14),ISNUMBER($B$2)),((I14*Datos!$B15)/(1+Datos!$C15)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K14" s="48">
         <f>$K$3*(1+Datos!D15)/Datos!B15</f>
         <v>0</v>
       </c>
-      <c r="L14" s="9">
-        <f>((K14*Datos!$B15)/(1+Datos!$C15)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L14" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K14*Datos!$B15)/(1+Datos!$C15)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3066,45 +3329,45 @@
       <c r="B15" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="48" t="str">
+      <c r="C15" s="48">
         <f>IF(ISNUMBER(Datos!E16),$C$3*(1+Datos!E16)/Datos!B16,"-")</f>
-        <v>-</v>
+        <v>18499.666666666668</v>
       </c>
       <c r="D15" s="9" t="str">
-        <f>IF(ISNUMBER(C15),((C15*Datos!$B16)/(1+Datos!$C16)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C15),ISNUMBER($B$2)),((C15*Datos!$B16)/(1+Datos!$C16)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E15" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F16),$E$3*(1+Datos!F16)/Datos!B16,"-")</f>
         <v>-</v>
       </c>
       <c r="F15" s="9" t="str">
-        <f>IF(ISNUMBER(E15),((E15*Datos!$B16)/(1+Datos!$C16)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G15" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E15),ISNUMBER($B$2)),((E15*Datos!$B16)/(1+Datos!$C16)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G15" s="48">
         <f>IF(ISNUMBER(Datos!G16),$G$3*(1+Datos!G16)/Datos!B16,"-")</f>
-        <v>-</v>
+        <v>19536</v>
       </c>
       <c r="H15" s="9" t="str">
-        <f>IF(ISNUMBER(G15),((G15*Datos!$B16)/(1+Datos!$C16)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G15),ISNUMBER($B$2)),((G15*Datos!$B16)/(1+Datos!$C16)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I15" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H16),$I$3*(1+Datos!H16)/Datos!B16,"-")</f>
         <v>-</v>
       </c>
       <c r="J15" s="9" t="str">
-        <f>IF(ISNUMBER(I15),((I15*Datos!$B16)/(1+Datos!$C16)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I15),ISNUMBER($B$2)),((I15*Datos!$B16)/(1+Datos!$C16)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K15" s="48">
         <f>$K$3*(1+Datos!D16)/Datos!B16</f>
         <v>0</v>
       </c>
-      <c r="L15" s="9">
-        <f>((K15*Datos!$B16)/(1+Datos!$C16)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L15" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K15*Datos!$B16)/(1+Datos!$C16)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3114,45 +3377,45 @@
       <c r="B16" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="48" t="str">
+      <c r="C16" s="48">
         <f>IF(ISNUMBER(Datos!E17),$C$3*(1+Datos!E17)/Datos!B17,"-")</f>
-        <v>-</v>
+        <v>9249.8333333333339</v>
       </c>
       <c r="D16" s="9" t="str">
-        <f>IF(ISNUMBER(C16),((C16*Datos!$B17)/(1+Datos!$C17)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C16),ISNUMBER($B$2)),((C16*Datos!$B17)/(1+Datos!$C17)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E16" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F17),$E$3*(1+Datos!F17)/Datos!B17,"-")</f>
         <v>-</v>
       </c>
       <c r="F16" s="9" t="str">
-        <f>IF(ISNUMBER(E16),((E16*Datos!$B17)/(1+Datos!$C17)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G16" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E16),ISNUMBER($B$2)),((E16*Datos!$B17)/(1+Datos!$C17)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G16" s="48">
         <f>IF(ISNUMBER(Datos!G17),$G$3*(1+Datos!G17)/Datos!B17,"-")</f>
-        <v>-</v>
+        <v>9768</v>
       </c>
       <c r="H16" s="9" t="str">
-        <f>IF(ISNUMBER(G16),((G16*Datos!$B17)/(1+Datos!$C17)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G16),ISNUMBER($B$2)),((G16*Datos!$B17)/(1+Datos!$C17)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I16" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H17),$I$3*(1+Datos!H17)/Datos!B17,"-")</f>
         <v>-</v>
       </c>
       <c r="J16" s="9" t="str">
-        <f>IF(ISNUMBER(I16),((I16*Datos!$B17)/(1+Datos!$C17)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I16),ISNUMBER($B$2)),((I16*Datos!$B17)/(1+Datos!$C17)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K16" s="48">
         <f>$K$3*(1+Datos!D17)/Datos!B17</f>
         <v>0</v>
       </c>
-      <c r="L16" s="9">
-        <f>((K16*Datos!$B17)/(1+Datos!$C17)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L16" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K16*Datos!$B17)/(1+Datos!$C17)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3162,45 +3425,45 @@
       <c r="B17" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="48" t="str">
+      <c r="C17" s="48">
         <f>IF(ISNUMBER(Datos!E18),$C$3*(1+Datos!E18)/Datos!B18,"-")</f>
-        <v>-</v>
+        <v>4624.916666666667</v>
       </c>
       <c r="D17" s="9" t="str">
-        <f>IF(ISNUMBER(C17),((C17*Datos!$B18)/(1+Datos!$C18)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C17),ISNUMBER($B$2)),((C17*Datos!$B18)/(1+Datos!$C18)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E17" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F18),$E$3*(1+Datos!F18)/Datos!B18,"-")</f>
         <v>-</v>
       </c>
       <c r="F17" s="9" t="str">
-        <f>IF(ISNUMBER(E17),((E17*Datos!$B18)/(1+Datos!$C18)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G17" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E17),ISNUMBER($B$2)),((E17*Datos!$B18)/(1+Datos!$C18)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G17" s="48">
         <f>IF(ISNUMBER(Datos!G18),$G$3*(1+Datos!G18)/Datos!B18,"-")</f>
-        <v>-</v>
+        <v>4884</v>
       </c>
       <c r="H17" s="9" t="str">
-        <f>IF(ISNUMBER(G17),((G17*Datos!$B18)/(1+Datos!$C18)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G17),ISNUMBER($B$2)),((G17*Datos!$B18)/(1+Datos!$C18)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I17" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H18),$I$3*(1+Datos!H18)/Datos!B18,"-")</f>
         <v>-</v>
       </c>
       <c r="J17" s="9" t="str">
-        <f>IF(ISNUMBER(I17),((I17*Datos!$B18)/(1+Datos!$C18)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I17),ISNUMBER($B$2)),((I17*Datos!$B18)/(1+Datos!$C18)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K17" s="48">
         <f>$K$3*(1+Datos!D18)/Datos!B18</f>
         <v>0</v>
       </c>
-      <c r="L17" s="9">
-        <f>((K17*Datos!$B18)/(1+Datos!$C18)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L17" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K17*Datos!$B18)/(1+Datos!$C18)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3210,45 +3473,45 @@
       <c r="B18" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="48" t="str">
+      <c r="C18" s="48">
         <f>IF(ISNUMBER(Datos!E19),$C$3*(1+Datos!E19)/Datos!B19,"-")</f>
-        <v>-</v>
+        <v>4624.916666666667</v>
       </c>
       <c r="D18" s="9" t="str">
-        <f>IF(ISNUMBER(C18),((C18*Datos!$B19)/(1+Datos!$C19)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C18),ISNUMBER($B$2)),((C18*Datos!$B19)/(1+Datos!$C19)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E18" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F19),$E$3*(1+Datos!F19)/Datos!B19,"-")</f>
         <v>-</v>
       </c>
       <c r="F18" s="9" t="str">
-        <f>IF(ISNUMBER(E18),((E18*Datos!$B19)/(1+Datos!$C19)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G18" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E18),ISNUMBER($B$2)),((E18*Datos!$B19)/(1+Datos!$C19)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G18" s="48">
         <f>IF(ISNUMBER(Datos!G19),$G$3*(1+Datos!G19)/Datos!B19,"-")</f>
-        <v>-</v>
+        <v>4884</v>
       </c>
       <c r="H18" s="9" t="str">
-        <f>IF(ISNUMBER(G18),((G18*Datos!$B19)/(1+Datos!$C19)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G18),ISNUMBER($B$2)),((G18*Datos!$B19)/(1+Datos!$C19)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I18" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H19),$I$3*(1+Datos!H19)/Datos!B19,"-")</f>
         <v>-</v>
       </c>
       <c r="J18" s="9" t="str">
-        <f>IF(ISNUMBER(I18),((I18*Datos!$B19)/(1+Datos!$C19)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I18),ISNUMBER($B$2)),((I18*Datos!$B19)/(1+Datos!$C19)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K18" s="48">
         <f>$K$3*(1+Datos!D19)/Datos!B19</f>
         <v>0</v>
       </c>
-      <c r="L18" s="9">
-        <f>((K18*Datos!$B19)/(1+Datos!$C19)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L18" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K18*Datos!$B19)/(1+Datos!$C19)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3258,45 +3521,45 @@
       <c r="B19" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="48" t="str">
+      <c r="C19" s="48">
         <f>IF(ISNUMBER(Datos!E20),$C$3*(1+Datos!E20)/Datos!B20,"-")</f>
-        <v>-</v>
+        <v>3699.9333333333334</v>
       </c>
       <c r="D19" s="9" t="str">
-        <f>IF(ISNUMBER(C19),((C19*Datos!$B20)/(1+Datos!$C20)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C19),ISNUMBER($B$2)),((C19*Datos!$B20)/(1+Datos!$C20)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E19" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F20),$E$3*(1+Datos!F20)/Datos!B20,"-")</f>
         <v>-</v>
       </c>
       <c r="F19" s="9" t="str">
-        <f>IF(ISNUMBER(E19),((E19*Datos!$B20)/(1+Datos!$C20)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E19),ISNUMBER($B$2)),((E19*Datos!$B20)/(1+Datos!$C20)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G19" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G20),$G$3*(1+Datos!G20)/Datos!B20,"-")</f>
         <v>-</v>
       </c>
       <c r="H19" s="9" t="str">
-        <f>IF(ISNUMBER(G19),((G19*Datos!$B20)/(1+Datos!$C20)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G19),ISNUMBER($B$2)),((G19*Datos!$B20)/(1+Datos!$C20)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I19" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H20),$I$3*(1+Datos!H20)/Datos!B20,"-")</f>
         <v>-</v>
       </c>
       <c r="J19" s="9" t="str">
-        <f>IF(ISNUMBER(I19),((I19*Datos!$B20)/(1+Datos!$C20)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I19),ISNUMBER($B$2)),((I19*Datos!$B20)/(1+Datos!$C20)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K19" s="48">
         <f>$K$3*(1+Datos!D20)/Datos!B20</f>
         <v>0</v>
       </c>
-      <c r="L19" s="9">
-        <f>((K19*Datos!$B20)/(1+Datos!$C20)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L19" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K19*Datos!$B20)/(1+Datos!$C20)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3311,40 +3574,40 @@
         <v>-</v>
       </c>
       <c r="D20" s="9" t="str">
-        <f>IF(ISNUMBER(C20),((C20*Datos!$B21)/(1+Datos!$C21)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C20),ISNUMBER($B$2)),((C20*Datos!$B21)/(1+Datos!$C21)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E20" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F21),$E$3*(1+Datos!F21)/Datos!B21,"-")</f>
         <v>-</v>
       </c>
       <c r="F20" s="9" t="str">
-        <f>IF(ISNUMBER(E20),((E20*Datos!$B21)/(1+Datos!$C21)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G20" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E20),ISNUMBER($B$2)),((E20*Datos!$B21)/(1+Datos!$C21)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G20" s="48">
         <f>IF(ISNUMBER(Datos!G21),$G$3*(1+Datos!G21)/Datos!B21,"-")</f>
-        <v>-</v>
+        <v>3983.3904000000007</v>
       </c>
       <c r="H20" s="9" t="str">
-        <f>IF(ISNUMBER(G20),((G20*Datos!$B21)/(1+Datos!$C21)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G20),ISNUMBER($B$2)),((G20*Datos!$B21)/(1+Datos!$C21)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I20" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H21),$I$3*(1+Datos!H21)/Datos!B21,"-")</f>
         <v>-</v>
       </c>
       <c r="J20" s="9" t="str">
-        <f>IF(ISNUMBER(I20),((I20*Datos!$B21)/(1+Datos!$C21)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I20),ISNUMBER($B$2)),((I20*Datos!$B21)/(1+Datos!$C21)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K20" s="48">
         <f>$K$3*(1+Datos!D21)/Datos!B21</f>
         <v>0</v>
       </c>
-      <c r="L20" s="9">
-        <f>((K20*Datos!$B21)/(1+Datos!$C21)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L20" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K20*Datos!$B21)/(1+Datos!$C21)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3359,40 +3622,40 @@
         <v>-</v>
       </c>
       <c r="D21" s="9" t="str">
-        <f>IF(ISNUMBER(C21),((C21*Datos!$B22)/(1+Datos!$C22)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C21),ISNUMBER($B$2)),((C21*Datos!$B22)/(1+Datos!$C22)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E21" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F22),$E$3*(1+Datos!F22)/Datos!B22,"-")</f>
         <v>-</v>
       </c>
       <c r="F21" s="9" t="str">
-        <f>IF(ISNUMBER(E21),((E21*Datos!$B22)/(1+Datos!$C22)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E21),ISNUMBER($B$2)),((E21*Datos!$B22)/(1+Datos!$C22)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G21" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G22),$G$3*(1+Datos!G22)/Datos!B22,"-")</f>
         <v>-</v>
       </c>
       <c r="H21" s="9" t="str">
-        <f>IF(ISNUMBER(G21),((G21*Datos!$B22)/(1+Datos!$C22)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G21),ISNUMBER($B$2)),((G21*Datos!$B22)/(1+Datos!$C22)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I21" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H22),$I$3*(1+Datos!H22)/Datos!B22,"-")</f>
         <v>-</v>
       </c>
       <c r="J21" s="9" t="str">
-        <f>IF(ISNUMBER(I21),((I21*Datos!$B22)/(1+Datos!$C22)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I21),ISNUMBER($B$2)),((I21*Datos!$B22)/(1+Datos!$C22)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K21" s="48">
         <f>$K$3*(1+Datos!D22)/Datos!B22</f>
         <v>0</v>
       </c>
-      <c r="L21" s="9">
-        <f>((K21*Datos!$B22)/(1+Datos!$C22)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L21" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K21*Datos!$B22)/(1+Datos!$C22)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3402,45 +3665,45 @@
       <c r="B22" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="48" t="str">
+      <c r="C22" s="48">
         <f>IF(ISNUMBER(Datos!E23),$C$3*(1+Datos!E23)/Datos!B23,"-")</f>
-        <v>-</v>
+        <v>3177.6199112222221</v>
       </c>
       <c r="D22" s="9" t="str">
-        <f>IF(ISNUMBER(C22),((C22*Datos!$B23)/(1+Datos!$C23)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C22),ISNUMBER($B$2)),((C22*Datos!$B23)/(1+Datos!$C23)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E22" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F23),$E$3*(1+Datos!F23)/Datos!B23,"-")</f>
         <v>-</v>
       </c>
       <c r="F22" s="9" t="str">
-        <f>IF(ISNUMBER(E22),((E22*Datos!$B23)/(1+Datos!$C23)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G22" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E22),ISNUMBER($B$2)),((E22*Datos!$B23)/(1+Datos!$C23)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G22" s="48">
         <f>IF(ISNUMBER(Datos!G23),$G$3*(1+Datos!G23)/Datos!B23,"-")</f>
-        <v>-</v>
+        <v>3484.5712000000003</v>
       </c>
       <c r="H22" s="9" t="str">
-        <f>IF(ISNUMBER(G22),((G22*Datos!$B23)/(1+Datos!$C23)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G22),ISNUMBER($B$2)),((G22*Datos!$B23)/(1+Datos!$C23)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I22" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H23),$I$3*(1+Datos!H23)/Datos!B23,"-")</f>
         <v>-</v>
       </c>
       <c r="J22" s="9" t="str">
-        <f>IF(ISNUMBER(I22),((I22*Datos!$B23)/(1+Datos!$C23)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I22),ISNUMBER($B$2)),((I22*Datos!$B23)/(1+Datos!$C23)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K22" s="48">
         <f>$K$3*(1+Datos!D23)/Datos!B23</f>
         <v>0</v>
       </c>
-      <c r="L22" s="9">
-        <f>((K22*Datos!$B23)/(1+Datos!$C23)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L22" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K22*Datos!$B23)/(1+Datos!$C23)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3455,40 +3718,40 @@
         <v>-</v>
       </c>
       <c r="D23" s="9" t="str">
-        <f>IF(ISNUMBER(C23),((C23*Datos!$B24)/(1+Datos!$C24)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C23),ISNUMBER($B$2)),((C23*Datos!$B24)/(1+Datos!$C24)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E23" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F24),$E$3*(1+Datos!F24)/Datos!B24,"-")</f>
         <v>-</v>
       </c>
       <c r="F23" s="9" t="str">
-        <f>IF(ISNUMBER(E23),((E23*Datos!$B24)/(1+Datos!$C24)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E23),ISNUMBER($B$2)),((E23*Datos!$B24)/(1+Datos!$C24)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G23" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G24),$G$3*(1+Datos!G24)/Datos!B24,"-")</f>
         <v>-</v>
       </c>
       <c r="H23" s="9" t="str">
-        <f>IF(ISNUMBER(G23),((G23*Datos!$B24)/(1+Datos!$C24)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G23),ISNUMBER($B$2)),((G23*Datos!$B24)/(1+Datos!$C24)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I23" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H24),$I$3*(1+Datos!H24)/Datos!B24,"-")</f>
         <v>-</v>
       </c>
       <c r="J23" s="9" t="str">
-        <f>IF(ISNUMBER(I23),((I23*Datos!$B24)/(1+Datos!$C24)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I23),ISNUMBER($B$2)),((I23*Datos!$B24)/(1+Datos!$C24)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K23" s="48">
         <f>$K$3*(1+Datos!D24)/Datos!B24</f>
         <v>0</v>
       </c>
-      <c r="L23" s="9">
-        <f>((K23*Datos!$B24)/(1+Datos!$C24)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L23" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K23*Datos!$B24)/(1+Datos!$C24)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="24" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3498,45 +3761,45 @@
       <c r="B24" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="48" t="str">
+      <c r="C24" s="48">
         <f>IF(ISNUMBER(Datos!E25),$C$3*(1+Datos!E25)/Datos!B25,"-")</f>
-        <v>-</v>
+        <v>3024.6899500999998</v>
       </c>
       <c r="D24" s="9" t="str">
-        <f>IF(ISNUMBER(C24),((C24*Datos!$B25)/(1+Datos!$C25)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C24),ISNUMBER($B$2)),((C24*Datos!$B25)/(1+Datos!$C25)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E24" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F25),$E$3*(1+Datos!F25)/Datos!B25,"-")</f>
         <v>-</v>
       </c>
       <c r="F24" s="9" t="str">
-        <f>IF(ISNUMBER(E24),((E24*Datos!$B25)/(1+Datos!$C25)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G24" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E24),ISNUMBER($B$2)),((E24*Datos!$B25)/(1+Datos!$C25)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G24" s="48">
         <f>IF(ISNUMBER(Datos!G25),$G$3*(1+Datos!G25)/Datos!B25,"-")</f>
-        <v>-</v>
+        <v>3223.44</v>
       </c>
       <c r="H24" s="9" t="str">
-        <f>IF(ISNUMBER(G24),((G24*Datos!$B25)/(1+Datos!$C25)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G24),ISNUMBER($B$2)),((G24*Datos!$B25)/(1+Datos!$C25)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I24" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H25),$I$3*(1+Datos!H25)/Datos!B25,"-")</f>
         <v>-</v>
       </c>
       <c r="J24" s="9" t="str">
-        <f>IF(ISNUMBER(I24),((I24*Datos!$B25)/(1+Datos!$C25)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I24),ISNUMBER($B$2)),((I24*Datos!$B25)/(1+Datos!$C25)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K24" s="48">
         <f>$K$3*(1+Datos!D25)/Datos!B25</f>
         <v>0</v>
       </c>
-      <c r="L24" s="9">
-        <f>((K24*Datos!$B25)/(1+Datos!$C25)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L24" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K24*Datos!$B25)/(1+Datos!$C25)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3552,40 +3815,40 @@
         <v>-</v>
       </c>
       <c r="D25" s="9" t="str">
-        <f>IF(ISNUMBER(C25),((C25*Datos!$B26)/(1+Datos!$C26)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C25),ISNUMBER($B$2)),((C25*Datos!$B26)/(1+Datos!$C26)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E25" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F26),$E$3*(1+Datos!F26)/Datos!B26,"-")</f>
         <v>-</v>
       </c>
       <c r="F25" s="9" t="str">
-        <f>IF(ISNUMBER(E25),((E25*Datos!$B26)/(1+Datos!$C26)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E25),ISNUMBER($B$2)),((E25*Datos!$B26)/(1+Datos!$C26)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G25" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G26),$G$3*(1+Datos!G26)/Datos!B26,"-")</f>
         <v>-</v>
       </c>
       <c r="H25" s="9" t="str">
-        <f>IF(ISNUMBER(G25),((G25*Datos!$B26)/(1+Datos!$C26)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G25),ISNUMBER($B$2)),((G25*Datos!$B26)/(1+Datos!$C26)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I25" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H26),$I$3*(1+Datos!H26)/Datos!B26,"-")</f>
         <v>-</v>
       </c>
       <c r="J25" s="9" t="str">
-        <f>IF(ISNUMBER(I25),((I25*Datos!$B26)/(1+Datos!$C26)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I25),ISNUMBER($B$2)),((I25*Datos!$B26)/(1+Datos!$C26)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K25" s="48">
         <f>$K$3*(1+Datos!D26)/Datos!B26</f>
         <v>0</v>
       </c>
-      <c r="L25" s="9">
-        <f>((K25*Datos!$B26)/(1+Datos!$C26)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L25" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K25*Datos!$B26)/(1+Datos!$C26)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3596,45 +3859,45 @@
       <c r="B26" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="C26" s="48" t="str">
+      <c r="C26" s="48">
         <f>IF(ISNUMBER(Datos!E27),$C$3*(1+Datos!E27)/Datos!B27,"-")</f>
-        <v>-</v>
+        <v>18499.666666666668</v>
       </c>
       <c r="D26" s="9" t="str">
-        <f>IF(ISNUMBER(C26),((C26*Datos!$B27)/(1+Datos!$C27)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C26),ISNUMBER($B$2)),((C26*Datos!$B27)/(1+Datos!$C27)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E26" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F27),$E$3*(1+Datos!F27)/Datos!B27,"-")</f>
         <v>-</v>
       </c>
       <c r="F26" s="9" t="str">
-        <f>IF(ISNUMBER(E26),((E26*Datos!$B27)/(1+Datos!$C27)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G26" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E26),ISNUMBER($B$2)),((E26*Datos!$B27)/(1+Datos!$C27)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G26" s="48">
         <f>IF(ISNUMBER(Datos!G27),$G$3*(1+Datos!G27)/Datos!B27,"-")</f>
-        <v>-</v>
+        <v>19536</v>
       </c>
       <c r="H26" s="9" t="str">
-        <f>IF(ISNUMBER(G26),((G26*Datos!$B27)/(1+Datos!$C27)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G26),ISNUMBER($B$2)),((G26*Datos!$B27)/(1+Datos!$C27)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I26" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H27),$I$3*(1+Datos!H27)/Datos!B27,"-")</f>
         <v>-</v>
       </c>
       <c r="J26" s="9" t="str">
-        <f>IF(ISNUMBER(I26),((I26*Datos!$B27)/(1+Datos!$C27)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I26),ISNUMBER($B$2)),((I26*Datos!$B27)/(1+Datos!$C27)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K26" s="48">
         <f>$K$3*(1+Datos!D27)/Datos!B27</f>
         <v>0</v>
       </c>
-      <c r="L26" s="9">
-        <f>((K26*Datos!$B27)/(1+Datos!$C27)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L26" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K26*Datos!$B27)/(1+Datos!$C27)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3645,45 +3908,45 @@
       <c r="B27" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="C27" s="48" t="str">
+      <c r="C27" s="48">
         <f>IF(ISNUMBER(Datos!E28),$C$3*(1+Datos!E28)/Datos!B28,"-")</f>
-        <v>-</v>
+        <v>9249.8333333333339</v>
       </c>
       <c r="D27" s="9" t="str">
-        <f>IF(ISNUMBER(C27),((C27*Datos!$B28)/(1+Datos!$C28)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C27),ISNUMBER($B$2)),((C27*Datos!$B28)/(1+Datos!$C28)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E27" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F28),$E$3*(1+Datos!F28)/Datos!B28,"-")</f>
         <v>-</v>
       </c>
       <c r="F27" s="9" t="str">
-        <f>IF(ISNUMBER(E27),((E27*Datos!$B28)/(1+Datos!$C28)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G27" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E27),ISNUMBER($B$2)),((E27*Datos!$B28)/(1+Datos!$C28)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G27" s="48">
         <f>IF(ISNUMBER(Datos!G28),$G$3*(1+Datos!G28)/Datos!B28,"-")</f>
-        <v>-</v>
+        <v>9768</v>
       </c>
       <c r="H27" s="9" t="str">
-        <f>IF(ISNUMBER(G27),((G27*Datos!$B28)/(1+Datos!$C28)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G27),ISNUMBER($B$2)),((G27*Datos!$B28)/(1+Datos!$C28)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I27" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H28),$I$3*(1+Datos!H28)/Datos!B28,"-")</f>
         <v>-</v>
       </c>
       <c r="J27" s="9" t="str">
-        <f>IF(ISNUMBER(I27),((I27*Datos!$B28)/(1+Datos!$C28)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I27),ISNUMBER($B$2)),((I27*Datos!$B28)/(1+Datos!$C28)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K27" s="48">
         <f>$K$3*(1+Datos!D28)/Datos!B28</f>
         <v>0</v>
       </c>
-      <c r="L27" s="9">
-        <f>((K27*Datos!$B28)/(1+Datos!$C28)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L27" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K27*Datos!$B28)/(1+Datos!$C28)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="28" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3694,45 +3957,45 @@
       <c r="B28" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="C28" s="48" t="str">
+      <c r="C28" s="48">
         <f>IF(ISNUMBER(Datos!E29),$C$3*(1+Datos!E29)/Datos!B29,"-")</f>
-        <v>-</v>
+        <v>6166.5555555555557</v>
       </c>
       <c r="D28" s="9" t="str">
-        <f>IF(ISNUMBER(C28),((C28*Datos!$B29)/(1+Datos!$C29)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C28),ISNUMBER($B$2)),((C28*Datos!$B29)/(1+Datos!$C29)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E28" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F29),$E$3*(1+Datos!F29)/Datos!B29,"-")</f>
         <v>-</v>
       </c>
       <c r="F28" s="9" t="str">
-        <f>IF(ISNUMBER(E28),((E28*Datos!$B29)/(1+Datos!$C29)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G28" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E28),ISNUMBER($B$2)),((E28*Datos!$B29)/(1+Datos!$C29)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G28" s="48">
         <f>IF(ISNUMBER(Datos!G29),$G$3*(1+Datos!G29)/Datos!B29,"-")</f>
-        <v>-</v>
+        <v>6512</v>
       </c>
       <c r="H28" s="9" t="str">
-        <f>IF(ISNUMBER(G28),((G28*Datos!$B29)/(1+Datos!$C29)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G28),ISNUMBER($B$2)),((G28*Datos!$B29)/(1+Datos!$C29)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I28" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H29),$I$3*(1+Datos!H29)/Datos!B29,"-")</f>
         <v>-</v>
       </c>
       <c r="J28" s="9" t="str">
-        <f>IF(ISNUMBER(I28),((I28*Datos!$B29)/(1+Datos!$C29)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I28),ISNUMBER($B$2)),((I28*Datos!$B29)/(1+Datos!$C29)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K28" s="48">
         <f>$K$3*(1+Datos!D29)/Datos!B29</f>
         <v>0</v>
       </c>
-      <c r="L28" s="9">
-        <f>((K28*Datos!$B29)/(1+Datos!$C29)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L28" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K28*Datos!$B29)/(1+Datos!$C29)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3748,40 +4011,40 @@
         <v>-</v>
       </c>
       <c r="D29" s="9" t="str">
-        <f>IF(ISNUMBER(C29),((C29*Datos!$B30)/(1+Datos!$C30)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C29),ISNUMBER($B$2)),((C29*Datos!$B30)/(1+Datos!$C30)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E29" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F30),$E$3*(1+Datos!F30)/Datos!B30,"-")</f>
         <v>-</v>
       </c>
       <c r="F29" s="9" t="str">
-        <f>IF(ISNUMBER(E29),((E29*Datos!$B30)/(1+Datos!$C30)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E29),ISNUMBER($B$2)),((E29*Datos!$B30)/(1+Datos!$C30)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G29" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G30),$G$3*(1+Datos!G30)/Datos!B30,"-")</f>
         <v>-</v>
       </c>
       <c r="H29" s="9" t="str">
-        <f>IF(ISNUMBER(G29),((G29*Datos!$B30)/(1+Datos!$C30)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G29),ISNUMBER($B$2)),((G29*Datos!$B30)/(1+Datos!$C30)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I29" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H30),$I$3*(1+Datos!H30)/Datos!B30,"-")</f>
         <v>-</v>
       </c>
       <c r="J29" s="9" t="str">
-        <f>IF(ISNUMBER(I29),((I29*Datos!$B30)/(1+Datos!$C30)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I29),ISNUMBER($B$2)),((I29*Datos!$B30)/(1+Datos!$C30)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K29" s="48">
         <f>$K$3*(1+Datos!D30)/Datos!B30</f>
         <v>0</v>
       </c>
-      <c r="L29" s="9">
-        <f>((K29*Datos!$B30)/(1+Datos!$C30)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L29" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K29*Datos!$B30)/(1+Datos!$C30)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3797,40 +4060,40 @@
         <v>-</v>
       </c>
       <c r="D30" s="9" t="str">
-        <f>IF(ISNUMBER(C30),((C30*Datos!$B31)/(1+Datos!$C31)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C30),ISNUMBER($B$2)),((C30*Datos!$B31)/(1+Datos!$C31)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E30" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F31),$E$3*(1+Datos!F31)/Datos!B31,"-")</f>
         <v>-</v>
       </c>
       <c r="F30" s="9" t="str">
-        <f>IF(ISNUMBER(E30),((E30*Datos!$B31)/(1+Datos!$C31)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G30" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E30),ISNUMBER($B$2)),((E30*Datos!$B31)/(1+Datos!$C31)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G30" s="48">
         <f>IF(ISNUMBER(Datos!G31),$G$3*(1+Datos!G31)/Datos!B31,"-")</f>
-        <v>-</v>
+        <v>5860.8</v>
       </c>
       <c r="H30" s="9" t="str">
-        <f>IF(ISNUMBER(G30),((G30*Datos!$B31)/(1+Datos!$C31)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G30),ISNUMBER($B$2)),((G30*Datos!$B31)/(1+Datos!$C31)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I30" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H31),$I$3*(1+Datos!H31)/Datos!B31,"-")</f>
         <v>-</v>
       </c>
       <c r="J30" s="9" t="str">
-        <f>IF(ISNUMBER(I30),((I30*Datos!$B31)/(1+Datos!$C31)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I30),ISNUMBER($B$2)),((I30*Datos!$B31)/(1+Datos!$C31)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K30" s="48">
         <f>$K$3*(1+Datos!D31)/Datos!B31</f>
         <v>0</v>
       </c>
-      <c r="L30" s="9">
-        <f>((K30*Datos!$B31)/(1+Datos!$C31)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L30" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K30*Datos!$B31)/(1+Datos!$C31)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3846,40 +4109,40 @@
         <v>-</v>
       </c>
       <c r="D31" s="9" t="str">
-        <f>IF(ISNUMBER(C31),((C31*Datos!$B32)/(1+Datos!$C32)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C31),ISNUMBER($B$2)),((C31*Datos!$B32)/(1+Datos!$C32)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E31" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F32),$E$3*(1+Datos!F32)/Datos!B32,"-")</f>
         <v>-</v>
       </c>
       <c r="F31" s="9" t="str">
-        <f>IF(ISNUMBER(E31),((E31*Datos!$B32)/(1+Datos!$C32)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E31),ISNUMBER($B$2)),((E31*Datos!$B32)/(1+Datos!$C32)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G31" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G32),$G$3*(1+Datos!G32)/Datos!B32,"-")</f>
         <v>-</v>
       </c>
       <c r="H31" s="9" t="str">
-        <f>IF(ISNUMBER(G31),((G31*Datos!$B32)/(1+Datos!$C32)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G31),ISNUMBER($B$2)),((G31*Datos!$B32)/(1+Datos!$C32)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I31" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H32),$I$3*(1+Datos!H32)/Datos!B32,"-")</f>
         <v>-</v>
       </c>
       <c r="J31" s="9" t="str">
-        <f>IF(ISNUMBER(I31),((I31*Datos!$B32)/(1+Datos!$C32)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I31),ISNUMBER($B$2)),((I31*Datos!$B32)/(1+Datos!$C32)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K31" s="48">
         <f>$K$3*(1+Datos!D32)/Datos!B32</f>
         <v>0</v>
       </c>
-      <c r="L31" s="9">
-        <f>((K31*Datos!$B32)/(1+Datos!$C32)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L31" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K31*Datos!$B32)/(1+Datos!$C32)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="32" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3890,45 +4153,45 @@
       <c r="B32" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="C32" s="48" t="str">
+      <c r="C32" s="48">
         <f>IF(ISNUMBER(Datos!E33),$C$3*(1+Datos!E33)/Datos!B33,"-")</f>
-        <v>-</v>
+        <v>4624.916666666667</v>
       </c>
       <c r="D32" s="9" t="str">
-        <f>IF(ISNUMBER(C32),((C32*Datos!$B33)/(1+Datos!$C33)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C32),ISNUMBER($B$2)),((C32*Datos!$B33)/(1+Datos!$C33)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E32" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F33),$E$3*(1+Datos!F33)/Datos!B33,"-")</f>
         <v>-</v>
       </c>
       <c r="F32" s="9" t="str">
-        <f>IF(ISNUMBER(E32),((E32*Datos!$B33)/(1+Datos!$C33)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E32),ISNUMBER($B$2)),((E32*Datos!$B33)/(1+Datos!$C33)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G32" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G33),$G$3*(1+Datos!G33)/Datos!B33,"-")</f>
         <v>-</v>
       </c>
       <c r="H32" s="9" t="str">
-        <f>IF(ISNUMBER(G32),((G32*Datos!$B33)/(1+Datos!$C33)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G32),ISNUMBER($B$2)),((G32*Datos!$B33)/(1+Datos!$C33)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I32" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H33),$I$3*(1+Datos!H33)/Datos!B33,"-")</f>
         <v>-</v>
       </c>
       <c r="J32" s="9" t="str">
-        <f>IF(ISNUMBER(I32),((I32*Datos!$B33)/(1+Datos!$C33)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I32),ISNUMBER($B$2)),((I32*Datos!$B33)/(1+Datos!$C33)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K32" s="48">
         <f>$K$3*(1+Datos!D33)/Datos!B33</f>
         <v>0</v>
       </c>
-      <c r="L32" s="9">
-        <f>((K32*Datos!$B33)/(1+Datos!$C33)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L32" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K32*Datos!$B33)/(1+Datos!$C33)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="33" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3944,40 +4207,40 @@
         <v>-</v>
       </c>
       <c r="D33" s="9" t="str">
-        <f>IF(ISNUMBER(C33),((C33*Datos!$B34)/(1+Datos!$C34)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C33),ISNUMBER($B$2)),((C33*Datos!$B34)/(1+Datos!$C34)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E33" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F34),$E$3*(1+Datos!F34)/Datos!B34,"-")</f>
         <v>-</v>
       </c>
       <c r="F33" s="9" t="str">
-        <f>IF(ISNUMBER(E33),((E33*Datos!$B34)/(1+Datos!$C34)/$B$2)-1,"-")</f>
-        <v>-</v>
-      </c>
-      <c r="G33" s="48" t="str">
+        <f>IF(AND(ISNUMBER(E33),ISNUMBER($B$2)),((E33*Datos!$B34)/(1+Datos!$C34)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
+      </c>
+      <c r="G33" s="48">
         <f>IF(ISNUMBER(Datos!G34),$G$3*(1+Datos!G34)/Datos!B34,"-")</f>
-        <v>-</v>
+        <v>5323.56</v>
       </c>
       <c r="H33" s="9" t="str">
-        <f>IF(ISNUMBER(G33),((G33*Datos!$B34)/(1+Datos!$C34)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G33),ISNUMBER($B$2)),((G33*Datos!$B34)/(1+Datos!$C34)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I33" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H34),$I$3*(1+Datos!H34)/Datos!B34,"-")</f>
         <v>-</v>
       </c>
       <c r="J33" s="9" t="str">
-        <f>IF(ISNUMBER(I33),((I33*Datos!$B34)/(1+Datos!$C34)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I33),ISNUMBER($B$2)),((I33*Datos!$B34)/(1+Datos!$C34)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K33" s="48">
         <f>$K$3*(1+Datos!D34)/Datos!B34</f>
         <v>0</v>
       </c>
-      <c r="L33" s="9">
-        <f>((K33*Datos!$B34)/(1+Datos!$C34)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L33" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K33*Datos!$B34)/(1+Datos!$C34)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="34" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3993,40 +4256,40 @@
         <v>-</v>
       </c>
       <c r="D34" s="9" t="str">
-        <f>IF(ISNUMBER(C34),((C34*Datos!$B35)/(1+Datos!$C35)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C34),ISNUMBER($B$2)),((C34*Datos!$B35)/(1+Datos!$C35)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E34" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F35),$E$3*(1+Datos!F35)/Datos!B35,"-")</f>
         <v>-</v>
       </c>
       <c r="F34" s="9" t="str">
-        <f>IF(ISNUMBER(E34),((E34*Datos!$B35)/(1+Datos!$C35)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E34),ISNUMBER($B$2)),((E34*Datos!$B35)/(1+Datos!$C35)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G34" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G35),$G$3*(1+Datos!G35)/Datos!B35,"-")</f>
         <v>-</v>
       </c>
       <c r="H34" s="9" t="str">
-        <f>IF(ISNUMBER(G34),((G34*Datos!$B35)/(1+Datos!$C35)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G34),ISNUMBER($B$2)),((G34*Datos!$B35)/(1+Datos!$C35)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I34" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H35),$I$3*(1+Datos!H35)/Datos!B35,"-")</f>
         <v>-</v>
       </c>
       <c r="J34" s="9" t="str">
-        <f>IF(ISNUMBER(I34),((I34*Datos!$B35)/(1+Datos!$C35)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I34),ISNUMBER($B$2)),((I34*Datos!$B35)/(1+Datos!$C35)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K34" s="48">
         <f>$K$3*(1+Datos!D35)/Datos!B35</f>
         <v>0</v>
       </c>
-      <c r="L34" s="9">
-        <f>((K34*Datos!$B35)/(1+Datos!$C35)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L34" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K34*Datos!$B35)/(1+Datos!$C35)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="35" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4042,40 +4305,40 @@
         <v>-</v>
       </c>
       <c r="D35" s="9" t="str">
-        <f>IF(ISNUMBER(C35),((C35*Datos!$B36)/(1+Datos!$C36)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C35),ISNUMBER($B$2)),((C35*Datos!$B36)/(1+Datos!$C36)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E35" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F36),$E$3*(1+Datos!F36)/Datos!B36,"-")</f>
         <v>-</v>
       </c>
       <c r="F35" s="9" t="str">
-        <f>IF(ISNUMBER(E35),((E35*Datos!$B36)/(1+Datos!$C36)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E35),ISNUMBER($B$2)),((E35*Datos!$B36)/(1+Datos!$C36)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G35" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G36),$G$3*(1+Datos!G36)/Datos!B36,"-")</f>
         <v>-</v>
       </c>
       <c r="H35" s="9" t="str">
-        <f>IF(ISNUMBER(G35),((G35*Datos!$B36)/(1+Datos!$C36)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G35),ISNUMBER($B$2)),((G35*Datos!$B36)/(1+Datos!$C36)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I35" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H36),$I$3*(1+Datos!H36)/Datos!B36,"-")</f>
         <v>-</v>
       </c>
       <c r="J35" s="9" t="str">
-        <f>IF(ISNUMBER(I35),((I35*Datos!$B36)/(1+Datos!$C36)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I35),ISNUMBER($B$2)),((I35*Datos!$B36)/(1+Datos!$C36)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K35" s="48">
         <f>$K$3*(1+Datos!D36)/Datos!B36</f>
         <v>0</v>
       </c>
-      <c r="L35" s="9">
-        <f>((K35*Datos!$B36)/(1+Datos!$C36)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L35" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K35*Datos!$B36)/(1+Datos!$C36)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="36" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4091,40 +4354,40 @@
         <v>-</v>
       </c>
       <c r="D36" s="9" t="str">
-        <f>IF(ISNUMBER(C36),((C36*Datos!$B37)/(1+Datos!$C37)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C36),ISNUMBER($B$2)),((C36*Datos!$B37)/(1+Datos!$C37)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E36" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F37),$E$3*(1+Datos!F37)/Datos!B37,"-")</f>
         <v>-</v>
       </c>
       <c r="F36" s="9" t="str">
-        <f>IF(ISNUMBER(E36),((E36*Datos!$B37)/(1+Datos!$C37)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E36),ISNUMBER($B$2)),((E36*Datos!$B37)/(1+Datos!$C37)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G36" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G37),$G$3*(1+Datos!G37)/Datos!B37,"-")</f>
         <v>-</v>
       </c>
       <c r="H36" s="9" t="str">
-        <f>IF(ISNUMBER(G36),((G36*Datos!$B37)/(1+Datos!$C37)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G36),ISNUMBER($B$2)),((G36*Datos!$B37)/(1+Datos!$C37)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I36" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H37),$I$3*(1+Datos!H37)/Datos!B37,"-")</f>
         <v>-</v>
       </c>
       <c r="J36" s="9" t="str">
-        <f>IF(ISNUMBER(I36),((I36*Datos!$B37)/(1+Datos!$C37)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I36),ISNUMBER($B$2)),((I36*Datos!$B37)/(1+Datos!$C37)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K36" s="48">
         <f>$K$3*(1+Datos!D37)/Datos!B37</f>
         <v>0</v>
       </c>
-      <c r="L36" s="9">
-        <f>((K36*Datos!$B37)/(1+Datos!$C37)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L36" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K36*Datos!$B37)/(1+Datos!$C37)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="37" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4140,40 +4403,40 @@
         <v>-</v>
       </c>
       <c r="D37" s="9" t="str">
-        <f>IF(ISNUMBER(C37),((C37*Datos!$B38)/(1+Datos!$C38)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C37),ISNUMBER($B$2)),((C37*Datos!$B38)/(1+Datos!$C38)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E37" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F38),$E$3*(1+Datos!F38)/Datos!B38,"-")</f>
         <v>-</v>
       </c>
       <c r="F37" s="9" t="str">
-        <f>IF(ISNUMBER(E37),((E37*Datos!$B38)/(1+Datos!$C38)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E37),ISNUMBER($B$2)),((E37*Datos!$B38)/(1+Datos!$C38)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G37" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G38),$G$3*(1+Datos!G38)/Datos!B38,"-")</f>
         <v>-</v>
       </c>
       <c r="H37" s="9" t="str">
-        <f>IF(ISNUMBER(G37),((G37*Datos!$B38)/(1+Datos!$C38)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G37),ISNUMBER($B$2)),((G37*Datos!$B38)/(1+Datos!$C38)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I37" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H38),$I$3*(1+Datos!H38)/Datos!B38,"-")</f>
         <v>-</v>
       </c>
       <c r="J37" s="9" t="str">
-        <f>IF(ISNUMBER(I37),((I37*Datos!$B38)/(1+Datos!$C38)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I37),ISNUMBER($B$2)),((I37*Datos!$B38)/(1+Datos!$C38)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K37" s="48">
         <f>$K$3*(1+Datos!D38)/Datos!B38</f>
         <v>0</v>
       </c>
-      <c r="L37" s="9">
-        <f>((K37*Datos!$B38)/(1+Datos!$C38)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L37" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K37*Datos!$B38)/(1+Datos!$C38)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="38" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4189,40 +4452,40 @@
         <v>-</v>
       </c>
       <c r="D38" s="9" t="str">
-        <f>IF(ISNUMBER(C38),((C38*Datos!$B39)/(1+Datos!$C39)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C38),ISNUMBER($B$2)),((C38*Datos!$B39)/(1+Datos!$C39)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E38" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F39),$E$3*(1+Datos!F39)/Datos!B39,"-")</f>
         <v>-</v>
       </c>
       <c r="F38" s="9" t="str">
-        <f>IF(ISNUMBER(E38),((E38*Datos!$B39)/(1+Datos!$C39)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E38),ISNUMBER($B$2)),((E38*Datos!$B39)/(1+Datos!$C39)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G38" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G39),$G$3*(1+Datos!G39)/Datos!B39,"-")</f>
         <v>-</v>
       </c>
       <c r="H38" s="9" t="str">
-        <f>IF(ISNUMBER(G38),((G38*Datos!$B39)/(1+Datos!$C39)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G38),ISNUMBER($B$2)),((G38*Datos!$B39)/(1+Datos!$C39)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I38" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H39),$I$3*(1+Datos!H39)/Datos!B39,"-")</f>
         <v>-</v>
       </c>
       <c r="J38" s="9" t="str">
-        <f>IF(ISNUMBER(I38),((I38*Datos!$B39)/(1+Datos!$C39)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I38),ISNUMBER($B$2)),((I38*Datos!$B39)/(1+Datos!$C39)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K38" s="48">
         <f>$K$3*(1+Datos!D39)/Datos!B39</f>
         <v>0</v>
       </c>
-      <c r="L38" s="9">
-        <f>((K38*Datos!$B39)/(1+Datos!$C39)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L38" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K38*Datos!$B39)/(1+Datos!$C39)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="39" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4238,40 +4501,40 @@
         <v>-</v>
       </c>
       <c r="D39" s="9" t="str">
-        <f>IF(ISNUMBER(C39),((C39*Datos!$B40)/(1+Datos!$C40)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C39),ISNUMBER($B$2)),((C39*Datos!$B40)/(1+Datos!$C40)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E39" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F40),$E$3*(1+Datos!F40)/Datos!B40,"-")</f>
         <v>-</v>
       </c>
       <c r="F39" s="9" t="str">
-        <f>IF(ISNUMBER(E39),((E39*Datos!$B40)/(1+Datos!$C40)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E39),ISNUMBER($B$2)),((E39*Datos!$B40)/(1+Datos!$C40)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G39" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G40),$G$3*(1+Datos!G40)/Datos!B40,"-")</f>
         <v>-</v>
       </c>
       <c r="H39" s="9" t="str">
-        <f>IF(ISNUMBER(G39),((G39*Datos!$B40)/(1+Datos!$C40)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G39),ISNUMBER($B$2)),((G39*Datos!$B40)/(1+Datos!$C40)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I39" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H40),$I$3*(1+Datos!H40)/Datos!B40,"-")</f>
         <v>-</v>
       </c>
       <c r="J39" s="9" t="str">
-        <f>IF(ISNUMBER(I39),((I39*Datos!$B40)/(1+Datos!$C40)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I39),ISNUMBER($B$2)),((I39*Datos!$B40)/(1+Datos!$C40)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K39" s="48">
         <f>$K$3*(1+Datos!D40)/Datos!B40</f>
         <v>0</v>
       </c>
-      <c r="L39" s="9">
-        <f>((K39*Datos!$B40)/(1+Datos!$C40)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L39" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K39*Datos!$B40)/(1+Datos!$C40)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="40" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4287,40 +4550,40 @@
         <v>-</v>
       </c>
       <c r="D40" s="9" t="str">
-        <f>IF(ISNUMBER(C40),((C40*Datos!$B41)/(1+Datos!$C41)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C40),ISNUMBER($B$2)),((C40*Datos!$B41)/(1+Datos!$C41)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E40" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F41),$E$3*(1+Datos!F41)/Datos!B41,"-")</f>
         <v>-</v>
       </c>
       <c r="F40" s="9" t="str">
-        <f>IF(ISNUMBER(E40),((E40*Datos!$B41)/(1+Datos!$C41)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E40),ISNUMBER($B$2)),((E40*Datos!$B41)/(1+Datos!$C41)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G40" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G41),$G$3*(1+Datos!G41)/Datos!B41,"-")</f>
         <v>-</v>
       </c>
       <c r="H40" s="9" t="str">
-        <f>IF(ISNUMBER(G40),((G40*Datos!$B41)/(1+Datos!$C41)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G40),ISNUMBER($B$2)),((G40*Datos!$B41)/(1+Datos!$C41)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I40" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H41),$I$3*(1+Datos!H41)/Datos!B41,"-")</f>
         <v>-</v>
       </c>
       <c r="J40" s="9" t="str">
-        <f>IF(ISNUMBER(I40),((I40*Datos!$B41)/(1+Datos!$C41)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I40),ISNUMBER($B$2)),((I40*Datos!$B41)/(1+Datos!$C41)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K40" s="48">
         <f>$K$3*(1+Datos!D41)/Datos!B41</f>
         <v>0</v>
       </c>
-      <c r="L40" s="9">
-        <f>((K40*Datos!$B41)/(1+Datos!$C41)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L40" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K40*Datos!$B41)/(1+Datos!$C41)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="41" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4336,40 +4599,40 @@
         <v>-</v>
       </c>
       <c r="D41" s="9" t="str">
-        <f>IF(ISNUMBER(C41),((C41*Datos!$B42)/(1+Datos!$C42)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C41),ISNUMBER($B$2)),((C41*Datos!$B42)/(1+Datos!$C42)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E41" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F42),$E$3*(1+Datos!F42)/Datos!B42,"-")</f>
         <v>-</v>
       </c>
       <c r="F41" s="9" t="str">
-        <f>IF(ISNUMBER(E41),((E41*Datos!$B42)/(1+Datos!$C42)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E41),ISNUMBER($B$2)),((E41*Datos!$B42)/(1+Datos!$C42)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G41" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G42),$G$3*(1+Datos!G42)/Datos!B42,"-")</f>
         <v>-</v>
       </c>
       <c r="H41" s="9" t="str">
-        <f>IF(ISNUMBER(G41),((G41*Datos!$B42)/(1+Datos!$C42)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G41),ISNUMBER($B$2)),((G41*Datos!$B42)/(1+Datos!$C42)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I41" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H42),$I$3*(1+Datos!H42)/Datos!B42,"-")</f>
         <v>-</v>
       </c>
       <c r="J41" s="9" t="str">
-        <f>IF(ISNUMBER(I41),((I41*Datos!$B42)/(1+Datos!$C42)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I41),ISNUMBER($B$2)),((I41*Datos!$B42)/(1+Datos!$C42)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K41" s="48">
         <f>$K$3*(1+Datos!D42)/Datos!B42</f>
         <v>0</v>
       </c>
-      <c r="L41" s="9">
-        <f>((K41*Datos!$B42)/(1+Datos!$C42)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L41" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K41*Datos!$B42)/(1+Datos!$C42)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4385,40 +4648,40 @@
         <v>-</v>
       </c>
       <c r="D42" s="9" t="str">
-        <f>IF(ISNUMBER(C42),((C42*Datos!$B43)/(1+Datos!$C43)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C42),ISNUMBER($B$2)),((C42*Datos!$B43)/(1+Datos!$C43)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E42" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F43),$E$3*(1+Datos!F43)/Datos!B43,"-")</f>
         <v>-</v>
       </c>
       <c r="F42" s="9" t="str">
-        <f>IF(ISNUMBER(E42),((E42*Datos!$B43)/(1+Datos!$C43)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E42),ISNUMBER($B$2)),((E42*Datos!$B43)/(1+Datos!$C43)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G42" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G43),$G$3*(1+Datos!G43)/Datos!B43,"-")</f>
         <v>-</v>
       </c>
       <c r="H42" s="9" t="str">
-        <f>IF(ISNUMBER(G42),((G42*Datos!$B43)/(1+Datos!$C43)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G42),ISNUMBER($B$2)),((G42*Datos!$B43)/(1+Datos!$C43)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I42" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H43),$I$3*(1+Datos!H43)/Datos!B43,"-")</f>
         <v>-</v>
       </c>
       <c r="J42" s="9" t="str">
-        <f>IF(ISNUMBER(I42),((I42*Datos!$B43)/(1+Datos!$C43)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I42),ISNUMBER($B$2)),((I42*Datos!$B43)/(1+Datos!$C43)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K42" s="48">
         <f>$K$3*(1+Datos!D43)/Datos!B43</f>
         <v>0</v>
       </c>
-      <c r="L42" s="9">
-        <f>((K42*Datos!$B43)/(1+Datos!$C43)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L42" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K42*Datos!$B43)/(1+Datos!$C43)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="43" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4434,40 +4697,40 @@
         <v>-</v>
       </c>
       <c r="D43" s="9" t="str">
-        <f>IF(ISNUMBER(C43),((C43*Datos!$B44)/(1+Datos!$C44)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C43),ISNUMBER($B$2)),((C43*Datos!$B44)/(1+Datos!$C44)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E43" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F44),$E$3*(1+Datos!F44)/Datos!B44,"-")</f>
         <v>-</v>
       </c>
       <c r="F43" s="9" t="str">
-        <f>IF(ISNUMBER(E43),((E43*Datos!$B44)/(1+Datos!$C44)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E43),ISNUMBER($B$2)),((E43*Datos!$B44)/(1+Datos!$C44)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G43" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G44),$G$3*(1+Datos!G44)/Datos!B44,"-")</f>
         <v>-</v>
       </c>
       <c r="H43" s="9" t="str">
-        <f>IF(ISNUMBER(G43),((G43*Datos!$B44)/(1+Datos!$C44)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G43),ISNUMBER($B$2)),((G43*Datos!$B44)/(1+Datos!$C44)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I43" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H44),$I$3*(1+Datos!H44)/Datos!B44,"-")</f>
         <v>-</v>
       </c>
       <c r="J43" s="9" t="str">
-        <f>IF(ISNUMBER(I43),((I43*Datos!$B44)/(1+Datos!$C44)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I43),ISNUMBER($B$2)),((I43*Datos!$B44)/(1+Datos!$C44)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K43" s="48">
         <f>$K$3*(1+Datos!D44)/Datos!B44</f>
         <v>0</v>
       </c>
-      <c r="L43" s="9">
-        <f>((K43*Datos!$B45)/(1+Datos!$C45)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L43" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K43*Datos!$B44)/(1+Datos!$C44)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="44" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4483,40 +4746,40 @@
         <v>-</v>
       </c>
       <c r="D44" s="9" t="str">
-        <f>IF(ISNUMBER(C44),((C44*Datos!$B45)/(1+Datos!$C45)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C44),ISNUMBER($B$2)),((C44*Datos!$B45)/(1+Datos!$C45)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E44" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F45),$E$3*(1+Datos!F45)/Datos!B45,"-")</f>
         <v>-</v>
       </c>
       <c r="F44" s="9" t="str">
-        <f>IF(ISNUMBER(E44),((E44*Datos!$B45)/(1+Datos!$C45)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E44),ISNUMBER($B$2)),((E44*Datos!$B45)/(1+Datos!$C45)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G44" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G45),$G$3*(1+Datos!G45)/Datos!B45,"-")</f>
         <v>-</v>
       </c>
       <c r="H44" s="9" t="str">
-        <f>IF(ISNUMBER(G44),((G44*Datos!$B45)/(1+Datos!$C45)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G44),ISNUMBER($B$2)),((G44*Datos!$B45)/(1+Datos!$C45)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I44" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H45),$I$3*(1+Datos!H45)/Datos!B45,"-")</f>
         <v>-</v>
       </c>
       <c r="J44" s="9" t="str">
-        <f>IF(ISNUMBER(I44),((I44*Datos!$B45)/(1+Datos!$C45)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I44),ISNUMBER($B$2)),((I44*Datos!$B45)/(1+Datos!$C45)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K44" s="48">
         <f>$K$3*(1+Datos!D45)/Datos!B45</f>
         <v>0</v>
       </c>
-      <c r="L44" s="9">
-        <f>((K44*Datos!$B45)/(1+Datos!$C45)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L44" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K44*Datos!$B45)/(1+Datos!$C45)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="45" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4532,40 +4795,40 @@
         <v>-</v>
       </c>
       <c r="D45" s="9" t="str">
-        <f>IF(ISNUMBER(C45),((C45*Datos!$B46)/(1+Datos!$C46)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C45),ISNUMBER($B$2)),((C45*Datos!$B46)/(1+Datos!$C46)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E45" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F46),$E$3*(1+Datos!F46)/Datos!B46,"-")</f>
         <v>-</v>
       </c>
       <c r="F45" s="9" t="str">
-        <f>IF(ISNUMBER(E45),((E45*Datos!$B46)/(1+Datos!$C46)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E45),ISNUMBER($B$2)),((E45*Datos!$B46)/(1+Datos!$C46)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G45" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G46),$G$3*(1+Datos!G46)/Datos!B46,"-")</f>
         <v>-</v>
       </c>
       <c r="H45" s="9" t="str">
-        <f>IF(ISNUMBER(G45),((G45*Datos!$B46)/(1+Datos!$C46)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G45),ISNUMBER($B$2)),((G45*Datos!$B46)/(1+Datos!$C46)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I45" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H46),$I$3*(1+Datos!H46)/Datos!B46,"-")</f>
         <v>-</v>
       </c>
       <c r="J45" s="9" t="str">
-        <f>IF(ISNUMBER(I45),((I45*Datos!$B46)/(1+Datos!$C46)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I45),ISNUMBER($B$2)),((I45*Datos!$B46)/(1+Datos!$C46)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K45" s="48">
         <f>$K$3*(1+Datos!D46)/Datos!B46</f>
         <v>0</v>
       </c>
-      <c r="L45" s="9">
-        <f>((K45*Datos!$B46)/(1+Datos!$C46)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L45" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K45*Datos!$B46)/(1+Datos!$C46)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="46" spans="1:12" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4581,40 +4844,40 @@
         <v>-</v>
       </c>
       <c r="D46" s="9" t="str">
-        <f>IF(ISNUMBER(C46),((C46*Datos!$B47)/(1+Datos!$C47)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C46),ISNUMBER($B$2)),((C46*Datos!$B47)/(1+Datos!$C47)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E46" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F47),$E$3*(1+Datos!F47)/Datos!B47,"-")</f>
         <v>-</v>
       </c>
       <c r="F46" s="9" t="str">
-        <f>IF(ISNUMBER(E46),((E46*Datos!$B47)/(1+Datos!$C47)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E46),ISNUMBER($B$2)),((E46*Datos!$B47)/(1+Datos!$C47)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G46" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G47),$G$3*(1+Datos!G47)/Datos!B47,"-")</f>
         <v>-</v>
       </c>
       <c r="H46" s="9" t="str">
-        <f>IF(ISNUMBER(G46),((G46*Datos!$B47)/(1+Datos!$C47)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G46),ISNUMBER($B$2)),((G46*Datos!$B47)/(1+Datos!$C47)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I46" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H47),$I$3*(1+Datos!H47)/Datos!B47,"-")</f>
         <v>-</v>
       </c>
       <c r="J46" s="9" t="str">
-        <f>IF(ISNUMBER(I46),((I46*Datos!$B47)/(1+Datos!$C47)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I46),ISNUMBER($B$2)),((I46*Datos!$B47)/(1+Datos!$C47)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K46" s="48">
         <f>$K$3*(1+Datos!D47)/Datos!B47</f>
         <v>0</v>
       </c>
-      <c r="L46" s="9">
-        <f>((K46*Datos!$B47)/(1+Datos!$C47)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L46" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K46*Datos!$B47)/(1+Datos!$C47)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="47" spans="1:12" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
@@ -4630,40 +4893,40 @@
         <v>-</v>
       </c>
       <c r="D47" s="9" t="str">
-        <f>IF(ISNUMBER(C47),((C47*Datos!$B48)/(1+Datos!$C48)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C47),ISNUMBER($B$2)),((C47*Datos!$B48)/(1+Datos!$C48)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E47" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F48),$E$3*(1+Datos!F48)/Datos!B48,"-")</f>
         <v>-</v>
       </c>
       <c r="F47" s="9" t="str">
-        <f>IF(ISNUMBER(E47),((E47*Datos!$B48)/(1+Datos!$C48)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E47),ISNUMBER($B$2)),((E47*Datos!$B48)/(1+Datos!$C48)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G47" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G48),$G$3*(1+Datos!G48)/Datos!B48,"-")</f>
         <v>-</v>
       </c>
       <c r="H47" s="9" t="str">
-        <f>IF(ISNUMBER(G47),((G47*Datos!$B48)/(1+Datos!$C48)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G47),ISNUMBER($B$2)),((G47*Datos!$B48)/(1+Datos!$C48)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I47" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H48),$I$3*(1+Datos!H48)/Datos!B48,"-")</f>
         <v>-</v>
       </c>
       <c r="J47" s="9" t="str">
-        <f>IF(ISNUMBER(I47),((I47*Datos!$B48)/(1+Datos!$C48)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I47),ISNUMBER($B$2)),((I47*Datos!$B48)/(1+Datos!$C48)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K47" s="48">
         <f>$K$3*(1+Datos!D48)/Datos!B48</f>
         <v>0</v>
       </c>
-      <c r="L47" s="9">
-        <f>((K47*Datos!$B48)/(1+Datos!$C48)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L47" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K47*Datos!$B48)/(1+Datos!$C48)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="48" spans="1:12" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
@@ -4679,40 +4942,40 @@
         <v>-</v>
       </c>
       <c r="D48" s="9" t="str">
-        <f>IF(ISNUMBER(C48),((C48*Datos!$B49)/(1+Datos!$C49)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C48),ISNUMBER($B$2)),((C48*Datos!$B49)/(1+Datos!$C49)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E48" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F49),$E$3*(1+Datos!F49)/Datos!B49,"-")</f>
         <v>-</v>
       </c>
       <c r="F48" s="9" t="str">
-        <f>IF(ISNUMBER(E48),((E48*Datos!$B49)/(1+Datos!$C49)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E48),ISNUMBER($B$2)),((E48*Datos!$B49)/(1+Datos!$C49)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G48" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G49),$G$3*(1+Datos!G49)/Datos!B49,"-")</f>
         <v>-</v>
       </c>
       <c r="H48" s="9" t="str">
-        <f>IF(ISNUMBER(G48),((G48*Datos!$B49)/(1+Datos!$C49)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G48),ISNUMBER($B$2)),((G48*Datos!$B49)/(1+Datos!$C49)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I48" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H49),$I$3*(1+Datos!H49)/Datos!B49,"-")</f>
         <v>-</v>
       </c>
       <c r="J48" s="9" t="str">
-        <f>IF(ISNUMBER(I48),((I48*Datos!$B49)/(1+Datos!$C49)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I48),ISNUMBER($B$2)),((I48*Datos!$B49)/(1+Datos!$C49)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K48" s="48">
         <f>$K$3*(1+Datos!D49)/Datos!B49</f>
         <v>0</v>
       </c>
-      <c r="L48" s="9">
-        <f>((K48*Datos!$B49)/(1+Datos!$C49)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L48" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K48*Datos!$B49)/(1+Datos!$C49)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="49" spans="1:13" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
@@ -4728,40 +4991,40 @@
         <v>-</v>
       </c>
       <c r="D49" s="9" t="str">
-        <f>IF(ISNUMBER(C49),((C49*Datos!$B50)/(1+Datos!$C50)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C49),ISNUMBER($B$2)),((C49*Datos!$B50)/(1+Datos!$C50)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E49" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F50),$E$3*(1+Datos!F50)/Datos!B50,"-")</f>
         <v>-</v>
       </c>
       <c r="F49" s="9" t="str">
-        <f>IF(ISNUMBER(E49),((E49*Datos!$B50)/(1+Datos!$C50)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E49),ISNUMBER($B$2)),((E49*Datos!$B50)/(1+Datos!$C50)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G49" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G50),$G$3*(1+Datos!G50)/Datos!B50,"-")</f>
         <v>-</v>
       </c>
       <c r="H49" s="9" t="str">
-        <f>IF(ISNUMBER(G49),((G49*Datos!$B50)/(1+Datos!$C50)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G49),ISNUMBER($B$2)),((G49*Datos!$B50)/(1+Datos!$C50)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I49" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H50),$I$3*(1+Datos!H50)/Datos!B50,"-")</f>
         <v>-</v>
       </c>
       <c r="J49" s="9" t="str">
-        <f>IF(ISNUMBER(I49),((I49*Datos!$B50)/(1+Datos!$C50)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I49),ISNUMBER($B$2)),((I49*Datos!$B50)/(1+Datos!$C50)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K49" s="48">
         <f>$K$3*(1+Datos!D50)/Datos!B50</f>
         <v>0</v>
       </c>
-      <c r="L49" s="9">
-        <f>((K49*Datos!$B50)/(1+Datos!$C50)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L49" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K49*Datos!$B50)/(1+Datos!$C50)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="50" spans="1:13" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
@@ -4777,40 +5040,40 @@
         <v>-</v>
       </c>
       <c r="D50" s="9" t="str">
-        <f>IF(ISNUMBER(C50),((C50*Datos!$B51)/(1+Datos!$C51)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C50),ISNUMBER($B$2)),((C50*Datos!$B51)/(1+Datos!$C51)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E50" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F51),$E$3*(1+Datos!F51)/Datos!B51,"-")</f>
         <v>-</v>
       </c>
       <c r="F50" s="9" t="str">
-        <f>IF(ISNUMBER(E50),((E50*Datos!$B51)/(1+Datos!$C51)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E50),ISNUMBER($B$2)),((E50*Datos!$B51)/(1+Datos!$C51)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G50" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G51),$G$3*(1+Datos!G51)/Datos!B51,"-")</f>
         <v>-</v>
       </c>
       <c r="H50" s="9" t="str">
-        <f>IF(ISNUMBER(G50),((G50*Datos!$B51)/(1+Datos!$C51)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G50),ISNUMBER($B$2)),((G50*Datos!$B51)/(1+Datos!$C51)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I50" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H51),$I$3*(1+Datos!H51)/Datos!B51,"-")</f>
         <v>-</v>
       </c>
       <c r="J50" s="9" t="str">
-        <f>IF(ISNUMBER(I50),((I50*Datos!$B51)/(1+Datos!$C51)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I50),ISNUMBER($B$2)),((I50*Datos!$B51)/(1+Datos!$C51)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K50" s="48">
         <f>$K$3*(1+Datos!D51)/Datos!B51</f>
         <v>0</v>
       </c>
-      <c r="L50" s="9">
-        <f>((K50*Datos!$B51)/(1+Datos!$C51)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L50" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K50*Datos!$B51)/(1+Datos!$C51)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="51" spans="1:13" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
@@ -4826,40 +5089,40 @@
         <v>-</v>
       </c>
       <c r="D51" s="9" t="str">
-        <f>IF(ISNUMBER(C51),((C51*Datos!$B52)/(1+Datos!$C52)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C51),ISNUMBER($B$2)),((C51*Datos!$B52)/(1+Datos!$C52)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E51" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F52),$E$3*(1+Datos!F52)/Datos!B52,"-")</f>
         <v>-</v>
       </c>
       <c r="F51" s="9" t="str">
-        <f>IF(ISNUMBER(E51),((E51*Datos!$B52)/(1+Datos!$C52)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E51),ISNUMBER($B$2)),((E51*Datos!$B52)/(1+Datos!$C52)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G51" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G52),$G$3*(1+Datos!G52)/Datos!B52,"-")</f>
         <v>-</v>
       </c>
       <c r="H51" s="9" t="str">
-        <f>IF(ISNUMBER(G51),((G51*Datos!$B52)/(1+Datos!$C52)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G51),ISNUMBER($B$2)),((G51*Datos!$B52)/(1+Datos!$C52)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I51" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H52),$I$3*(1+Datos!H52)/Datos!B52,"-")</f>
         <v>-</v>
       </c>
       <c r="J51" s="9" t="str">
-        <f>IF(ISNUMBER(I51),((I51*Datos!$B52)/(1+Datos!$C52)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I51),ISNUMBER($B$2)),((I51*Datos!$B52)/(1+Datos!$C52)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K51" s="48">
         <f>$K$3*(1+Datos!D52)/Datos!B52</f>
         <v>0</v>
       </c>
-      <c r="L51" s="9">
-        <f>((K51*Datos!$B52)/(1+Datos!$C52)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L51" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K51*Datos!$B52)/(1+Datos!$C52)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="52" spans="1:13" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
@@ -4875,40 +5138,40 @@
         <v>-</v>
       </c>
       <c r="D52" s="9" t="str">
-        <f>IF(ISNUMBER(C52),((C52*Datos!$B53)/(1+Datos!$C53)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C52),ISNUMBER($B$2)),((C52*Datos!$B53)/(1+Datos!$C53)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E52" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F53),$E$3*(1+Datos!F53)/Datos!B53,"-")</f>
         <v>-</v>
       </c>
       <c r="F52" s="9" t="str">
-        <f>IF(ISNUMBER(E52),((E52*Datos!$B53)/(1+Datos!$C53)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E52),ISNUMBER($B$2)),((E52*Datos!$B53)/(1+Datos!$C53)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G52" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G53),$G$3*(1+Datos!G53)/Datos!B53,"-")</f>
         <v>-</v>
       </c>
       <c r="H52" s="9" t="str">
-        <f>IF(ISNUMBER(G52),((G52*Datos!$B53)/(1+Datos!$C53)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G52),ISNUMBER($B$2)),((G52*Datos!$B53)/(1+Datos!$C53)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I52" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H53),$I$3*(1+Datos!H53)/Datos!B53,"-")</f>
         <v>-</v>
       </c>
       <c r="J52" s="9" t="str">
-        <f>IF(ISNUMBER(I52),((I52*Datos!$B53)/(1+Datos!$C53)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I52),ISNUMBER($B$2)),((I52*Datos!$B53)/(1+Datos!$C53)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K52" s="48">
         <f>$K$3*(1+Datos!D53)/Datos!B53</f>
         <v>0</v>
       </c>
-      <c r="L52" s="9">
-        <f>((K52*Datos!$B53)/(1+Datos!$C53)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L52" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K52*Datos!$B53)/(1+Datos!$C53)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="53" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4924,40 +5187,40 @@
         <v>-</v>
       </c>
       <c r="D53" s="9" t="str">
-        <f>IF(ISNUMBER(C53),((C53*Datos!$B54)/(1+Datos!$C54)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C53),ISNUMBER($B$2)),((C53*Datos!$B54)/(1+Datos!$C54)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E53" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F54),$E$3*(1+Datos!F54)/Datos!B54,"-")</f>
         <v>-</v>
       </c>
       <c r="F53" s="9" t="str">
-        <f>IF(ISNUMBER(E53),((E53*Datos!$B54)/(1+Datos!$C54)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E53),ISNUMBER($B$2)),((E53*Datos!$B54)/(1+Datos!$C54)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G53" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G54),$G$3*(1+Datos!G54)/Datos!B54,"-")</f>
         <v>-</v>
       </c>
       <c r="H53" s="9" t="str">
-        <f>IF(ISNUMBER(G53),((G53*Datos!$B54)/(1+Datos!$C54)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G53),ISNUMBER($B$2)),((G53*Datos!$B54)/(1+Datos!$C54)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I53" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H54),$I$3*(1+Datos!H54)/Datos!B54,"-")</f>
         <v>-</v>
       </c>
       <c r="J53" s="9" t="str">
-        <f>IF(ISNUMBER(I53),((I53*Datos!$B54)/(1+Datos!$C54)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I53),ISNUMBER($B$2)),((I53*Datos!$B54)/(1+Datos!$C54)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K53" s="48">
         <f>$K$3*(1+Datos!D54)/Datos!B54</f>
         <v>0</v>
       </c>
-      <c r="L53" s="9">
-        <f>((K53*Datos!$B54)/(1+Datos!$C54)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L53" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K53*Datos!$B54)/(1+Datos!$C54)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="54" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4973,40 +5236,40 @@
         <v>-</v>
       </c>
       <c r="D54" s="9" t="str">
-        <f>IF(ISNUMBER(C54),((C54*Datos!$B55)/(1+Datos!$C55)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C54),ISNUMBER($B$2)),((C54*Datos!$B55)/(1+Datos!$C55)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E54" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F55),$E$3*(1+Datos!F55)/Datos!B55,"-")</f>
         <v>-</v>
       </c>
       <c r="F54" s="9" t="str">
-        <f>IF(ISNUMBER(E54),((E54*Datos!$B55)/(1+Datos!$C55)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E54),ISNUMBER($B$2)),((E54*Datos!$B55)/(1+Datos!$C55)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G54" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G55),$G$3*(1+Datos!G55)/Datos!B55,"-")</f>
         <v>-</v>
       </c>
       <c r="H54" s="9" t="str">
-        <f>IF(ISNUMBER(G54),((G54*Datos!$B55)/(1+Datos!$C55)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G54),ISNUMBER($B$2)),((G54*Datos!$B55)/(1+Datos!$C55)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I54" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H55),$I$3*(1+Datos!H55)/Datos!B55,"-")</f>
         <v>-</v>
       </c>
       <c r="J54" s="9" t="str">
-        <f>IF(ISNUMBER(I54),((I54*Datos!$B55)/(1+Datos!$C55)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I54),ISNUMBER($B$2)),((I54*Datos!$B55)/(1+Datos!$C55)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K54" s="48">
         <f>$K$3*(1+Datos!D55)/Datos!B55</f>
         <v>0</v>
       </c>
-      <c r="L54" s="9">
-        <f>((K54*Datos!$B55)/(1+Datos!$C55)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L54" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K54*Datos!$B55)/(1+Datos!$C55)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="55" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -5022,40 +5285,40 @@
         <v>-</v>
       </c>
       <c r="D55" s="9" t="str">
-        <f>IF(ISNUMBER(C55),((C55*Datos!$B56)/(1+Datos!$C56)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C55),ISNUMBER($B$2)),((C55*Datos!$B56)/(1+Datos!$C56)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E55" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F56),$E$3*(1+Datos!F56)/Datos!B56,"-")</f>
         <v>-</v>
       </c>
       <c r="F55" s="9" t="str">
-        <f>IF(ISNUMBER(E55),((E55*Datos!$B56)/(1+Datos!$C56)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E55),ISNUMBER($B$2)),((E55*Datos!$B56)/(1+Datos!$C56)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G55" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G56),$G$3*(1+Datos!G56)/Datos!B56,"-")</f>
         <v>-</v>
       </c>
       <c r="H55" s="9" t="str">
-        <f>IF(ISNUMBER(G55),((G55*Datos!$B56)/(1+Datos!$C56)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G55),ISNUMBER($B$2)),((G55*Datos!$B56)/(1+Datos!$C56)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I55" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H56),$I$3*(1+Datos!H56)/Datos!B56,"-")</f>
         <v>-</v>
       </c>
       <c r="J55" s="9" t="str">
-        <f>IF(ISNUMBER(I55),((I55*Datos!$B56)/(1+Datos!$C56)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I55),ISNUMBER($B$2)),((I55*Datos!$B56)/(1+Datos!$C56)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K55" s="48">
         <f>$K$3*(1+Datos!D56)/Datos!B56</f>
         <v>0</v>
       </c>
-      <c r="L55" s="9">
-        <f>((K55*Datos!$B56)/(1+Datos!$C56)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L55" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K55*Datos!$B56)/(1+Datos!$C56)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="56" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -5071,40 +5334,40 @@
         <v>-</v>
       </c>
       <c r="D56" s="9" t="str">
-        <f>IF(ISNUMBER(C56),((C56*Datos!$B57)/(1+Datos!$C57)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C56),ISNUMBER($B$2)),((C56*Datos!$B57)/(1+Datos!$C57)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E56" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F57),$E$3*(1+Datos!F57)/Datos!B57,"-")</f>
         <v>-</v>
       </c>
       <c r="F56" s="9" t="str">
-        <f>IF(ISNUMBER(E56),((E56*Datos!$B57)/(1+Datos!$C57)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E56),ISNUMBER($B$2)),((E56*Datos!$B57)/(1+Datos!$C57)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G56" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G57),$G$3*(1+Datos!G57)/Datos!B57,"-")</f>
         <v>-</v>
       </c>
       <c r="H56" s="9" t="str">
-        <f>IF(ISNUMBER(G56),((G56*Datos!$B57)/(1+Datos!$C57)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G56),ISNUMBER($B$2)),((G56*Datos!$B57)/(1+Datos!$C57)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I56" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H57),$I$3*(1+Datos!H57)/Datos!B57,"-")</f>
         <v>-</v>
       </c>
       <c r="J56" s="9" t="str">
-        <f>IF(ISNUMBER(I56),((I56*Datos!$B57)/(1+Datos!$C57)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I56),ISNUMBER($B$2)),((I56*Datos!$B57)/(1+Datos!$C57)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K56" s="48">
         <f>$K$3*(1+Datos!D57)/Datos!B57</f>
         <v>0</v>
       </c>
-      <c r="L56" s="9">
-        <f>((K56*Datos!$B57)/(1+Datos!$C57)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L56" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K56*Datos!$B57)/(1+Datos!$C57)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="M56" s="49"/>
     </row>
@@ -5121,40 +5384,40 @@
         <v>-</v>
       </c>
       <c r="D57" s="9" t="str">
-        <f>IF(ISNUMBER(C57),((C57*Datos!$B58)/(1+Datos!$C58)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C57),ISNUMBER($B$2)),((C57*Datos!$B58)/(1+Datos!$C58)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E57" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F58),$E$3*(1+Datos!F58)/Datos!B58,"-")</f>
         <v>-</v>
       </c>
       <c r="F57" s="9" t="str">
-        <f>IF(ISNUMBER(E57),((E57*Datos!$B58)/(1+Datos!$C58)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E57),ISNUMBER($B$2)),((E57*Datos!$B58)/(1+Datos!$C58)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G57" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G58),$G$3*(1+Datos!G58)/Datos!B58,"-")</f>
         <v>-</v>
       </c>
       <c r="H57" s="9" t="str">
-        <f>IF(ISNUMBER(G57),((G57*Datos!$B58)/(1+Datos!$C58)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G57),ISNUMBER($B$2)),((G57*Datos!$B58)/(1+Datos!$C58)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I57" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H58),$I$3*(1+Datos!H58)/Datos!B58,"-")</f>
         <v>-</v>
       </c>
       <c r="J57" s="9" t="str">
-        <f>IF(ISNUMBER(I57),((I57*Datos!$B58)/(1+Datos!$C58)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I57),ISNUMBER($B$2)),((I57*Datos!$B58)/(1+Datos!$C58)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K57" s="48">
         <f>$K$3*(1+Datos!D58)/Datos!B58</f>
         <v>0</v>
       </c>
-      <c r="L57" s="9">
-        <f>((K57*Datos!$B58)/(1+Datos!$C58)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L57" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K57*Datos!$B58)/(1+Datos!$C58)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="58" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -5170,40 +5433,40 @@
         <v>-</v>
       </c>
       <c r="D58" s="9" t="str">
-        <f>IF(ISNUMBER(C58),((C58*Datos!$B59)/(1+Datos!$C59)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C58),ISNUMBER($B$2)),((C58*Datos!$B59)/(1+Datos!$C59)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E58" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F59),$E$3*(1+Datos!F59)/Datos!B59,"-")</f>
         <v>-</v>
       </c>
       <c r="F58" s="9" t="str">
-        <f>IF(ISNUMBER(E58),((E58*Datos!$B59)/(1+Datos!$C59)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E58),ISNUMBER($B$2)),((E58*Datos!$B59)/(1+Datos!$C59)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G58" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G59),$G$3*(1+Datos!G59)/Datos!B59,"-")</f>
         <v>-</v>
       </c>
       <c r="H58" s="9" t="str">
-        <f>IF(ISNUMBER(G58),((G58*Datos!$B59)/(1+Datos!$C59)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G58),ISNUMBER($B$2)),((G58*Datos!$B59)/(1+Datos!$C59)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I58" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H59),$I$3*(1+Datos!H59)/Datos!B59,"-")</f>
         <v>-</v>
       </c>
       <c r="J58" s="9" t="str">
-        <f>IF(ISNUMBER(I58),((I58*Datos!$B59)/(1+Datos!$C59)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I58),ISNUMBER($B$2)),((I58*Datos!$B59)/(1+Datos!$C59)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K58" s="48">
         <f>$K$3*(1+Datos!D59)/Datos!B59</f>
         <v>0</v>
       </c>
-      <c r="L58" s="9">
-        <f>((K58*Datos!$B59)/(1+Datos!$C59)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L58" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K58*Datos!$B59)/(1+Datos!$C59)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="59" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -5219,40 +5482,40 @@
         <v>-</v>
       </c>
       <c r="D59" s="9" t="str">
-        <f>IF(ISNUMBER(C59),((C59*Datos!$B60)/(1+Datos!$C60)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C59),ISNUMBER($B$2)),((C59*Datos!$B60)/(1+Datos!$C60)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E59" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F60),$E$3*(1+Datos!F60)/Datos!B60,"-")</f>
         <v>-</v>
       </c>
       <c r="F59" s="9" t="str">
-        <f>IF(ISNUMBER(E59),((E59*Datos!$B60)/(1+Datos!$C60)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E59),ISNUMBER($B$2)),((E59*Datos!$B60)/(1+Datos!$C60)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G59" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G60),$G$3*(1+Datos!G60)/Datos!B60,"-")</f>
         <v>-</v>
       </c>
       <c r="H59" s="9" t="str">
-        <f>IF(ISNUMBER(G59),((G59*Datos!$B60)/(1+Datos!$C60)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G59),ISNUMBER($B$2)),((G59*Datos!$B60)/(1+Datos!$C60)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I59" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H60),$I$3*(1+Datos!H60)/Datos!B60,"-")</f>
         <v>-</v>
       </c>
       <c r="J59" s="9" t="str">
-        <f>IF(ISNUMBER(I59),((I59*Datos!$B60)/(1+Datos!$C60)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I59),ISNUMBER($B$2)),((I59*Datos!$B60)/(1+Datos!$C60)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K59" s="48">
         <f>$K$3*(1+Datos!D60)/Datos!B60</f>
         <v>0</v>
       </c>
-      <c r="L59" s="9">
-        <f>((K59*Datos!$B60)/(1+Datos!$C60)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L59" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K59*Datos!$B60)/(1+Datos!$C60)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="60" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -5268,40 +5531,40 @@
         <v>-</v>
       </c>
       <c r="D60" s="9" t="str">
-        <f>IF(ISNUMBER(C60),((C60*Datos!$B61)/(1+Datos!$C61)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C60),ISNUMBER($B$2)),((C60*Datos!$B61)/(1+Datos!$C61)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E60" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F61),$E$3*(1+Datos!F61)/Datos!B61,"-")</f>
         <v>-</v>
       </c>
       <c r="F60" s="9" t="str">
-        <f>IF(ISNUMBER(E60),((E60*Datos!$B61)/(1+Datos!$C61)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E60),ISNUMBER($B$2)),((E60*Datos!$B61)/(1+Datos!$C61)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G60" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G61),$G$3*(1+Datos!G61)/Datos!B61,"-")</f>
         <v>-</v>
       </c>
       <c r="H60" s="9" t="str">
-        <f>IF(ISNUMBER(G60),((G60*Datos!$B61)/(1+Datos!$C61)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G60),ISNUMBER($B$2)),((G60*Datos!$B61)/(1+Datos!$C61)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I60" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H61),$I$3*(1+Datos!H61)/Datos!B61,"-")</f>
         <v>-</v>
       </c>
       <c r="J60" s="9" t="str">
-        <f>IF(ISNUMBER(I60),((I60*Datos!$B61)/(1+Datos!$C61)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I60),ISNUMBER($B$2)),((I60*Datos!$B61)/(1+Datos!$C61)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K60" s="48">
         <f>$K$3*(1+Datos!D61)/Datos!B61</f>
         <v>0</v>
       </c>
-      <c r="L60" s="9">
-        <f>((K60*Datos!$B61)/(1+Datos!$C61)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L60" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K60*Datos!$B61)/(1+Datos!$C61)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="61" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -5317,40 +5580,40 @@
         <v>-</v>
       </c>
       <c r="D61" s="9" t="str">
-        <f>IF(ISNUMBER(C61),((C61*Datos!$B62)/(1+Datos!$C62)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C61),ISNUMBER($B$2)),((C61*Datos!$B62)/(1+Datos!$C62)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E61" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F62),$E$3*(1+Datos!F62)/Datos!B62,"-")</f>
         <v>-</v>
       </c>
       <c r="F61" s="9" t="str">
-        <f>IF(ISNUMBER(E61),((E61*Datos!$B62)/(1+Datos!$C62)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E61),ISNUMBER($B$2)),((E61*Datos!$B62)/(1+Datos!$C62)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G61" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G62),$G$3*(1+Datos!G62)/Datos!B62,"-")</f>
         <v>-</v>
       </c>
       <c r="H61" s="9" t="str">
-        <f>IF(ISNUMBER(G61),((G61*Datos!$B62)/(1+Datos!$C62)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G61),ISNUMBER($B$2)),((G61*Datos!$B62)/(1+Datos!$C62)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I61" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H62),$I$3*(1+Datos!H62)/Datos!B62,"-")</f>
         <v>-</v>
       </c>
       <c r="J61" s="9" t="str">
-        <f>IF(ISNUMBER(I61),((I61*Datos!$B62)/(1+Datos!$C62)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I61),ISNUMBER($B$2)),((I61*Datos!$B62)/(1+Datos!$C62)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K61" s="48">
         <f>$K$3*(1+Datos!D62)/Datos!B62</f>
         <v>0</v>
       </c>
-      <c r="L61" s="9">
-        <f>((K61*Datos!$B62)/(1+Datos!$C62)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L61" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K61*Datos!$B62)/(1+Datos!$C62)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="62" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -5366,40 +5629,40 @@
         <v>-</v>
       </c>
       <c r="D62" s="9" t="str">
-        <f>IF(ISNUMBER(C62),((C62*Datos!$B63)/(1+Datos!$C63)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(C62),ISNUMBER($B$2)),((C62*Datos!$B63)/(1+Datos!$C63)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="E62" s="48" t="str">
         <f>IF(ISNUMBER(Datos!F63),$E$3*(1+Datos!F63)/Datos!B63,"-")</f>
         <v>-</v>
       </c>
       <c r="F62" s="9" t="str">
-        <f>IF(ISNUMBER(E62),((E62*Datos!$B63)/(1+Datos!$C63)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(E62),ISNUMBER($B$2)),((E62*Datos!$B63)/(1+Datos!$C63)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="G62" s="48" t="str">
         <f>IF(ISNUMBER(Datos!G63),$G$3*(1+Datos!G63)/Datos!B63,"-")</f>
         <v>-</v>
       </c>
       <c r="H62" s="9" t="str">
-        <f>IF(ISNUMBER(G62),((G62*Datos!$B63)/(1+Datos!$C63)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(G62),ISNUMBER($B$2)),((G62*Datos!$B63)/(1+Datos!$C63)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="I62" s="48" t="str">
         <f>IF(ISNUMBER(Datos!H63),$I$3*(1+Datos!H63)/Datos!B63,"-")</f>
         <v>-</v>
       </c>
       <c r="J62" s="9" t="str">
-        <f>IF(ISNUMBER(I62),((I62*Datos!$B63)/(1+Datos!$C63)/$B$2)-1,"-")</f>
-        <v>-</v>
+        <f>IF(AND(ISNUMBER(I62),ISNUMBER($B$2)),((I62*Datos!$B63)/(1+Datos!$C63)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K62" s="48">
         <f>$K$3*(1+Datos!D63)/Datos!B63</f>
         <v>0</v>
       </c>
-      <c r="L62" s="9">
-        <f>((K62*Datos!$B63)/(1+Datos!$C63)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L62" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K62*Datos!$B63)/(1+Datos!$C63)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="63" spans="1:13" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
@@ -5431,16 +5694,17 @@
       <c r="I63" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="J63" s="8" t="s">
-        <v>11</v>
+      <c r="J63" s="9" t="str">
+        <f>IF(AND(ISNUMBER(I63),ISNUMBER($B$2)),((I63*Datos!$B64)/(1+Datos!$C64)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K63" s="48">
         <f>$K$3*(1+Datos!D64)/Datos!B64</f>
         <v>0</v>
       </c>
-      <c r="L63" s="9">
-        <f>((K63*Datos!$B64)/(1+Datos!$C64)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L63" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K63*Datos!$B64)/(1+Datos!$C64)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
     <row r="64" spans="1:13" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
@@ -5472,16 +5736,17 @@
       <c r="I64" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="J64" s="8" t="s">
-        <v>11</v>
+      <c r="J64" s="9" t="str">
+        <f>IF(AND(ISNUMBER(I64),ISNUMBER($B$2)),((I64*Datos!$B65)/(1+Datos!$C65)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
+        <v>INSERTAR COSTO</v>
       </c>
       <c r="K64" s="48">
         <f>$K$3*(1+Datos!D65)/Datos!B65</f>
         <v>0</v>
       </c>
-      <c r="L64" s="9">
-        <f>((K64*Datos!$B65)/(1+Datos!$C65)/$B$2)-1</f>
-        <v>-1</v>
+      <c r="L64" s="9" t="str">
+        <f>IF(ISNUMBER($B$2),((K64*Datos!$B65)/(1+Datos!$C65)/$B$2)-1,"INSERTAR COSTO")</f>
+        <v>INSERTAR COSTO</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Excel pricing template
</commit_message>
<xml_diff>
--- a/backend/excel_template.xlsx
+++ b/backend/excel_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Frand\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Frand\Documents\Bots\ElectrodomesticsBot\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92466A16-5C18-4DA3-BFD9-653AB19E1405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{600F800A-DD53-4809-BFB3-A2177755419D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="15700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="15700" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="88">
   <si>
     <t>Interés</t>
   </si>
@@ -795,6 +795,7 @@
     <xf numFmtId="10" fontId="2" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="14" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -816,7 +817,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="14" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1042,7 +1042,7 @@
   <cols>
     <col min="1" max="1" width="21.26953125" customWidth="1"/>
     <col min="2" max="2" width="6.26953125" customWidth="1"/>
-    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="3" max="3" width="11.08984375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.08984375" customWidth="1"/>
     <col min="9" max="9" width="16.7265625" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
@@ -1061,14 +1061,14 @@
     <row r="2" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
-      <c r="C2" s="61" t="s">
+      <c r="C2" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="64"/>
     </row>
     <row r="3" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
@@ -1112,13 +1112,9 @@
       <c r="D4" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="54">
-        <v>55499</v>
-      </c>
+      <c r="E4" s="54"/>
       <c r="F4" s="54"/>
-      <c r="G4" s="55">
-        <v>58608</v>
-      </c>
+      <c r="G4" s="55"/>
       <c r="H4" s="56"/>
       <c r="I4" s="53" t="s">
         <v>10</v>
@@ -1137,13 +1133,9 @@
       <c r="D5" s="10">
         <v>-0.15</v>
       </c>
-      <c r="E5" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E5" s="57"/>
       <c r="F5" s="57"/>
-      <c r="G5" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G5" s="58"/>
       <c r="H5" s="58"/>
       <c r="I5" s="11" t="s">
         <v>13</v>
@@ -1162,13 +1154,9 @@
       <c r="D6" s="10">
         <v>-0.04</v>
       </c>
-      <c r="E6" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E6" s="57"/>
       <c r="F6" s="58"/>
-      <c r="G6" s="58">
-        <v>0</v>
-      </c>
+      <c r="G6" s="58"/>
       <c r="H6" s="58"/>
       <c r="I6" s="12" t="s">
         <v>15</v>
@@ -1187,13 +1175,9 @@
       <c r="D7" s="9">
         <v>0</v>
       </c>
-      <c r="E7" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E7" s="57"/>
       <c r="F7" s="58"/>
-      <c r="G7" s="58">
-        <v>0</v>
-      </c>
+      <c r="G7" s="58"/>
       <c r="H7" s="58"/>
       <c r="I7" s="12" t="s">
         <v>16</v>
@@ -1212,13 +1196,9 @@
       <c r="D8" s="9">
         <v>0</v>
       </c>
-      <c r="E8" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E8" s="57"/>
       <c r="F8" s="58"/>
-      <c r="G8" s="58">
-        <v>0</v>
-      </c>
+      <c r="G8" s="58"/>
       <c r="H8" s="58"/>
       <c r="I8" s="12" t="s">
         <v>17</v>
@@ -1237,13 +1217,9 @@
       <c r="D9" s="9">
         <v>0.05</v>
       </c>
-      <c r="E9" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E9" s="57"/>
       <c r="F9" s="58"/>
-      <c r="G9" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G9" s="58"/>
       <c r="H9" s="58"/>
       <c r="I9" s="12" t="s">
         <v>18</v>
@@ -1262,13 +1238,9 @@
       <c r="D10" s="9">
         <v>0</v>
       </c>
-      <c r="E10" s="59" t="s">
-        <v>11</v>
-      </c>
+      <c r="E10" s="59"/>
       <c r="F10" s="58"/>
-      <c r="G10" s="58">
-        <v>0</v>
-      </c>
+      <c r="G10" s="58"/>
       <c r="H10" s="58"/>
       <c r="I10" s="12" t="s">
         <v>19</v>
@@ -1287,13 +1259,9 @@
       <c r="D11" s="9">
         <v>0.1</v>
       </c>
-      <c r="E11" s="59" t="s">
-        <v>11</v>
-      </c>
+      <c r="E11" s="59"/>
       <c r="F11" s="58"/>
-      <c r="G11" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G11" s="58"/>
       <c r="H11" s="58"/>
       <c r="I11" s="12" t="s">
         <v>20</v>
@@ -1312,13 +1280,9 @@
       <c r="D12" s="9">
         <v>0</v>
       </c>
-      <c r="E12" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="E12" s="58"/>
       <c r="F12" s="59"/>
-      <c r="G12" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G12" s="58"/>
       <c r="H12" s="58"/>
       <c r="I12" s="12" t="s">
         <v>21</v>
@@ -1337,13 +1301,9 @@
       <c r="D13" s="9">
         <v>0.15</v>
       </c>
-      <c r="E13" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="E13" s="58"/>
       <c r="F13" s="59"/>
-      <c r="G13" s="58">
-        <v>1.95E-2</v>
-      </c>
+      <c r="G13" s="58"/>
       <c r="H13" s="58"/>
       <c r="I13" s="12" t="s">
         <v>22</v>
@@ -1362,13 +1322,9 @@
       <c r="D14" s="9">
         <v>0</v>
       </c>
-      <c r="E14" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="E14" s="58"/>
       <c r="F14" s="59"/>
-      <c r="G14" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G14" s="58"/>
       <c r="H14" s="58"/>
       <c r="I14" s="12" t="s">
         <v>23</v>
@@ -1387,13 +1343,9 @@
       <c r="D15" s="9">
         <v>0.21</v>
       </c>
-      <c r="E15" s="59" t="s">
-        <v>11</v>
-      </c>
+      <c r="E15" s="59"/>
       <c r="F15" s="59"/>
-      <c r="G15" s="58">
-        <v>7.0199999999999999E-2</v>
-      </c>
+      <c r="G15" s="58"/>
       <c r="H15" s="58"/>
       <c r="I15" s="12" t="s">
         <v>24</v>
@@ -1412,13 +1364,9 @@
       <c r="D16" s="10">
         <v>-0.05</v>
       </c>
-      <c r="E16" s="57">
-        <v>0</v>
-      </c>
+      <c r="E16" s="57"/>
       <c r="F16" s="58"/>
-      <c r="G16" s="58">
-        <v>0</v>
-      </c>
+      <c r="G16" s="58"/>
       <c r="H16" s="58"/>
       <c r="I16" s="17" t="s">
         <v>26</v>
@@ -1437,13 +1385,9 @@
       <c r="D17" s="10">
         <v>-0.05</v>
       </c>
-      <c r="E17" s="57">
-        <v>0</v>
-      </c>
+      <c r="E17" s="57"/>
       <c r="F17" s="58"/>
-      <c r="G17" s="58">
-        <v>0</v>
-      </c>
+      <c r="G17" s="58"/>
       <c r="H17" s="58"/>
       <c r="I17" s="17" t="s">
         <v>27</v>
@@ -1462,13 +1406,9 @@
       <c r="D18" s="10">
         <v>-0.05</v>
       </c>
-      <c r="E18" s="57">
-        <v>0</v>
-      </c>
+      <c r="E18" s="57"/>
       <c r="F18" s="58"/>
-      <c r="G18" s="58">
-        <v>0</v>
-      </c>
+      <c r="G18" s="58"/>
       <c r="H18" s="58"/>
       <c r="I18" s="17" t="s">
         <v>28</v>
@@ -1487,13 +1427,9 @@
       <c r="D19" s="9">
         <v>0</v>
       </c>
-      <c r="E19" s="57">
-        <v>0</v>
-      </c>
+      <c r="E19" s="57"/>
       <c r="F19" s="58"/>
-      <c r="G19" s="58">
-        <v>0</v>
-      </c>
+      <c r="G19" s="58"/>
       <c r="H19" s="58"/>
       <c r="I19" s="17" t="s">
         <v>29</v>
@@ -1512,13 +1448,9 @@
       <c r="D20" s="9">
         <v>0</v>
       </c>
-      <c r="E20" s="59">
-        <v>0</v>
-      </c>
+      <c r="E20" s="59"/>
       <c r="F20" s="59"/>
-      <c r="G20" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G20" s="58"/>
       <c r="H20" s="58"/>
       <c r="I20" s="17" t="s">
         <v>30</v>
@@ -1537,13 +1469,9 @@
       <c r="D21" s="9">
         <v>0.09</v>
       </c>
-      <c r="E21" s="59" t="s">
-        <v>11</v>
-      </c>
+      <c r="E21" s="59"/>
       <c r="F21" s="59"/>
-      <c r="G21" s="58">
-        <v>1.95E-2</v>
-      </c>
+      <c r="G21" s="58"/>
       <c r="H21" s="58"/>
       <c r="I21" s="17" t="s">
         <v>31</v>
@@ -1562,13 +1490,9 @@
       <c r="D22" s="9">
         <v>0</v>
       </c>
-      <c r="E22" s="59" t="s">
-        <v>11</v>
-      </c>
+      <c r="E22" s="59"/>
       <c r="F22" s="59"/>
-      <c r="G22" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G22" s="58"/>
       <c r="H22" s="58"/>
       <c r="I22" s="17" t="s">
         <v>32</v>
@@ -1587,13 +1511,9 @@
       <c r="D23" s="9">
         <v>0.15</v>
       </c>
-      <c r="E23" s="59">
-        <v>3.0598E-2</v>
-      </c>
+      <c r="E23" s="59"/>
       <c r="F23" s="59"/>
-      <c r="G23" s="58">
-        <v>7.0199999999999999E-2</v>
-      </c>
+      <c r="G23" s="58"/>
       <c r="H23" s="58"/>
       <c r="I23" s="17" t="s">
         <v>33</v>
@@ -1612,13 +1532,9 @@
       <c r="D24" s="9">
         <v>0</v>
       </c>
-      <c r="E24" s="59" t="s">
-        <v>11</v>
-      </c>
+      <c r="E24" s="59"/>
       <c r="F24" s="59"/>
-      <c r="G24" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G24" s="58"/>
       <c r="H24" s="58"/>
       <c r="I24" s="17" t="s">
         <v>34</v>
@@ -1637,13 +1553,9 @@
       <c r="D25" s="9">
         <v>0.18</v>
       </c>
-      <c r="E25" s="59">
-        <v>8.9997999999999995E-2</v>
-      </c>
+      <c r="E25" s="59"/>
       <c r="F25" s="59"/>
-      <c r="G25" s="58">
-        <v>0.1</v>
-      </c>
+      <c r="G25" s="58"/>
       <c r="H25" s="58"/>
       <c r="I25" s="17" t="s">
         <v>35</v>
@@ -1662,13 +1574,9 @@
       <c r="D26" s="10">
         <v>-0.15</v>
       </c>
-      <c r="E26" s="59" t="s">
-        <v>11</v>
-      </c>
+      <c r="E26" s="59"/>
       <c r="F26" s="57"/>
-      <c r="G26" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G26" s="58"/>
       <c r="H26" s="58"/>
       <c r="I26" s="19" t="s">
         <v>13</v>
@@ -1687,13 +1595,9 @@
       <c r="D27" s="10">
         <v>-0.04</v>
       </c>
-      <c r="E27" s="57">
-        <v>0</v>
-      </c>
+      <c r="E27" s="57"/>
       <c r="F27" s="58"/>
-      <c r="G27" s="58">
-        <v>0</v>
-      </c>
+      <c r="G27" s="58"/>
       <c r="H27" s="58"/>
       <c r="I27" s="19" t="s">
         <v>37</v>
@@ -1712,13 +1616,9 @@
       <c r="D28" s="9">
         <v>0</v>
       </c>
-      <c r="E28" s="57">
-        <v>0</v>
-      </c>
+      <c r="E28" s="57"/>
       <c r="F28" s="58"/>
-      <c r="G28" s="58">
-        <v>0</v>
-      </c>
+      <c r="G28" s="58"/>
       <c r="H28" s="58"/>
       <c r="I28" s="19" t="s">
         <v>38</v>
@@ -1737,13 +1637,9 @@
       <c r="D29" s="9">
         <v>0</v>
       </c>
-      <c r="E29" s="57">
-        <v>0</v>
-      </c>
+      <c r="E29" s="57"/>
       <c r="F29" s="58"/>
-      <c r="G29" s="58">
-        <v>0</v>
-      </c>
+      <c r="G29" s="58"/>
       <c r="H29" s="58"/>
       <c r="I29" s="19" t="s">
         <v>39</v>
@@ -1762,13 +1658,9 @@
       <c r="D30" s="9">
         <v>0.05</v>
       </c>
-      <c r="E30" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E30" s="57"/>
       <c r="F30" s="58"/>
-      <c r="G30" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G30" s="58"/>
       <c r="H30" s="58"/>
       <c r="I30" s="19" t="s">
         <v>40</v>
@@ -1787,13 +1679,9 @@
       <c r="D31" s="9">
         <v>0</v>
       </c>
-      <c r="E31" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="E31" s="58"/>
       <c r="F31" s="58"/>
-      <c r="G31" s="58">
-        <v>0</v>
-      </c>
+      <c r="G31" s="58"/>
       <c r="H31" s="59"/>
       <c r="I31" s="19" t="s">
         <v>41</v>
@@ -1812,13 +1700,9 @@
       <c r="D32" s="9">
         <v>0.05</v>
       </c>
-      <c r="E32" s="59" t="s">
-        <v>11</v>
-      </c>
+      <c r="E32" s="59"/>
       <c r="F32" s="58"/>
-      <c r="G32" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G32" s="58"/>
       <c r="H32" s="59"/>
       <c r="I32" s="19" t="s">
         <v>42</v>
@@ -1837,13 +1721,9 @@
       <c r="D33" s="9">
         <v>0</v>
       </c>
-      <c r="E33" s="57">
-        <v>0</v>
-      </c>
+      <c r="E33" s="57"/>
       <c r="F33" s="58"/>
-      <c r="G33" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G33" s="58"/>
       <c r="H33" s="58"/>
       <c r="I33" s="20" t="s">
         <v>43</v>
@@ -1862,13 +1742,9 @@
       <c r="D34" s="9">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E34" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E34" s="57"/>
       <c r="F34" s="58"/>
-      <c r="G34" s="58">
-        <v>0.09</v>
-      </c>
+      <c r="G34" s="58"/>
       <c r="H34" s="60"/>
       <c r="I34" s="20" t="s">
         <v>44</v>
@@ -1887,13 +1763,9 @@
       <c r="D35" s="9">
         <v>0</v>
       </c>
-      <c r="E35" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E35" s="57"/>
       <c r="F35" s="58"/>
-      <c r="G35" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G35" s="58"/>
       <c r="H35" s="59"/>
       <c r="I35" s="20" t="s">
         <v>45</v>
@@ -1912,13 +1784,9 @@
       <c r="D36" s="9">
         <v>0.09</v>
       </c>
-      <c r="E36" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E36" s="57"/>
       <c r="F36" s="59"/>
-      <c r="G36" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G36" s="58"/>
       <c r="H36" s="59"/>
       <c r="I36" s="20" t="s">
         <v>46</v>
@@ -1937,13 +1805,9 @@
       <c r="D37" s="9">
         <v>0</v>
       </c>
-      <c r="E37" s="59" t="s">
-        <v>11</v>
-      </c>
+      <c r="E37" s="59"/>
       <c r="F37" s="59"/>
-      <c r="G37" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G37" s="58"/>
       <c r="H37" s="59"/>
       <c r="I37" s="20" t="s">
         <v>47</v>
@@ -1962,13 +1826,9 @@
       <c r="D38" s="9">
         <v>0.18</v>
       </c>
-      <c r="E38" s="59" t="s">
-        <v>11</v>
-      </c>
+      <c r="E38" s="59"/>
       <c r="F38" s="59"/>
-      <c r="G38" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G38" s="58"/>
       <c r="H38" s="59"/>
       <c r="I38" s="20" t="s">
         <v>48</v>
@@ -1987,13 +1847,9 @@
       <c r="D39" s="10">
         <v>-0.15</v>
       </c>
-      <c r="E39" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E39" s="57"/>
       <c r="F39" s="57"/>
-      <c r="G39" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G39" s="58"/>
       <c r="H39" s="58"/>
       <c r="I39" s="22" t="s">
         <v>13</v>
@@ -2012,13 +1868,9 @@
       <c r="D40" s="10">
         <v>-0.04</v>
       </c>
-      <c r="E40" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E40" s="57"/>
       <c r="F40" s="58"/>
-      <c r="G40" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G40" s="58"/>
       <c r="H40" s="58"/>
       <c r="I40" s="22" t="s">
         <v>50</v>
@@ -2037,13 +1889,9 @@
       <c r="D41" s="9">
         <v>0</v>
       </c>
-      <c r="E41" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E41" s="57"/>
       <c r="F41" s="58"/>
-      <c r="G41" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G41" s="58"/>
       <c r="H41" s="58"/>
       <c r="I41" s="22" t="s">
         <v>51</v>
@@ -2062,13 +1910,9 @@
       <c r="D42" s="9">
         <v>0</v>
       </c>
-      <c r="E42" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E42" s="57"/>
       <c r="F42" s="58"/>
-      <c r="G42" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G42" s="58"/>
       <c r="H42" s="58"/>
       <c r="I42" s="22" t="s">
         <v>52</v>
@@ -2087,13 +1931,9 @@
       <c r="D43" s="9">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E43" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E43" s="57"/>
       <c r="F43" s="58"/>
-      <c r="G43" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G43" s="58"/>
       <c r="H43" s="58"/>
       <c r="I43" s="22" t="s">
         <v>53</v>
@@ -2112,13 +1952,9 @@
       <c r="D44" s="9">
         <v>0</v>
       </c>
-      <c r="E44" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E44" s="57"/>
       <c r="F44" s="58"/>
-      <c r="G44" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G44" s="58"/>
       <c r="H44" s="59"/>
       <c r="I44" s="23" t="s">
         <v>54</v>
@@ -2137,13 +1973,9 @@
       <c r="D45" s="9">
         <v>0.12</v>
       </c>
-      <c r="E45" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E45" s="57"/>
       <c r="F45" s="59"/>
-      <c r="G45" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G45" s="58"/>
       <c r="H45" s="58"/>
       <c r="I45" s="22" t="s">
         <v>55</v>
@@ -2162,13 +1994,9 @@
       <c r="D46" s="9">
         <v>0.25</v>
       </c>
-      <c r="E46" s="59" t="s">
-        <v>11</v>
-      </c>
+      <c r="E46" s="59"/>
       <c r="F46" s="59"/>
-      <c r="G46" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G46" s="58"/>
       <c r="H46" s="59"/>
       <c r="I46" s="23" t="s">
         <v>56</v>
@@ -2187,13 +2015,9 @@
       <c r="D47" s="9">
         <v>0.39</v>
       </c>
-      <c r="E47" s="59" t="s">
-        <v>11</v>
-      </c>
+      <c r="E47" s="59"/>
       <c r="F47" s="59"/>
-      <c r="G47" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G47" s="58"/>
       <c r="H47" s="59"/>
       <c r="I47" s="23" t="s">
         <v>57</v>
@@ -2212,13 +2036,9 @@
       <c r="D48" s="10">
         <v>-0.04</v>
       </c>
-      <c r="E48" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E48" s="57"/>
       <c r="F48" s="57"/>
-      <c r="G48" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G48" s="58"/>
       <c r="H48" s="58"/>
       <c r="I48" s="25" t="s">
         <v>59</v>
@@ -2237,13 +2057,9 @@
       <c r="D49" s="9">
         <v>0</v>
       </c>
-      <c r="E49" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E49" s="57"/>
       <c r="F49" s="57"/>
-      <c r="G49" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G49" s="58"/>
       <c r="H49" s="58"/>
       <c r="I49" s="25" t="s">
         <v>60</v>
@@ -2262,13 +2078,9 @@
       <c r="D50" s="9">
         <v>0</v>
       </c>
-      <c r="E50" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E50" s="57"/>
       <c r="F50" s="57"/>
-      <c r="G50" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G50" s="58"/>
       <c r="H50" s="58"/>
       <c r="I50" s="25" t="s">
         <v>61</v>
@@ -2287,13 +2099,9 @@
       <c r="D51" s="9">
         <v>0.05</v>
       </c>
-      <c r="E51" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E51" s="57"/>
       <c r="F51" s="57"/>
-      <c r="G51" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G51" s="58"/>
       <c r="H51" s="58"/>
       <c r="I51" s="25" t="s">
         <v>62</v>
@@ -2312,13 +2120,9 @@
       <c r="D52" s="9">
         <v>0</v>
       </c>
-      <c r="E52" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E52" s="57"/>
       <c r="F52" s="57"/>
-      <c r="G52" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G52" s="58"/>
       <c r="H52" s="58"/>
       <c r="I52" s="25" t="s">
         <v>63</v>
@@ -2337,13 +2141,9 @@
       <c r="D53" s="9">
         <v>0.12</v>
       </c>
-      <c r="E53" s="59" t="s">
-        <v>11</v>
-      </c>
+      <c r="E53" s="59"/>
       <c r="F53" s="57"/>
-      <c r="G53" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G53" s="58"/>
       <c r="H53" s="58"/>
       <c r="I53" s="25" t="s">
         <v>64</v>
@@ -2362,13 +2162,9 @@
       <c r="D54" s="10">
         <v>-7.0000000000000007E-2</v>
       </c>
-      <c r="E54" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E54" s="57"/>
       <c r="F54" s="59"/>
-      <c r="G54" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G54" s="58"/>
       <c r="H54" s="58"/>
       <c r="I54" s="27" t="s">
         <v>66</v>
@@ -2387,13 +2183,9 @@
       <c r="D55" s="9">
         <v>0</v>
       </c>
-      <c r="E55" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E55" s="57"/>
       <c r="F55" s="57"/>
-      <c r="G55" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G55" s="58"/>
       <c r="H55" s="58"/>
       <c r="I55" s="27" t="s">
         <v>67</v>
@@ -2412,13 +2204,9 @@
       <c r="D56" s="9">
         <v>0.06</v>
       </c>
-      <c r="E56" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E56" s="57"/>
       <c r="F56" s="57"/>
-      <c r="G56" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G56" s="58"/>
       <c r="H56" s="58"/>
       <c r="I56" s="27" t="s">
         <v>68</v>
@@ -2437,13 +2225,9 @@
       <c r="D57" s="10">
         <v>-0.09</v>
       </c>
-      <c r="E57" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E57" s="57"/>
       <c r="F57" s="57"/>
-      <c r="G57" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G57" s="58"/>
       <c r="H57" s="58"/>
       <c r="I57" s="29" t="s">
         <v>66</v>
@@ -2462,13 +2246,9 @@
       <c r="D58" s="10">
         <v>-0.04</v>
       </c>
-      <c r="E58" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E58" s="57"/>
       <c r="F58" s="57"/>
-      <c r="G58" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G58" s="58"/>
       <c r="H58" s="58"/>
       <c r="I58" s="29" t="s">
         <v>70</v>
@@ -2487,13 +2267,9 @@
       <c r="D59" s="9">
         <v>0</v>
       </c>
-      <c r="E59" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E59" s="57"/>
       <c r="F59" s="57"/>
-      <c r="G59" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G59" s="58"/>
       <c r="H59" s="58"/>
       <c r="I59" s="29" t="s">
         <v>71</v>
@@ -2512,13 +2288,9 @@
       <c r="D60" s="9">
         <v>0</v>
       </c>
-      <c r="E60" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E60" s="57"/>
       <c r="F60" s="57"/>
-      <c r="G60" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G60" s="58"/>
       <c r="H60" s="58"/>
       <c r="I60" s="29" t="s">
         <v>72</v>
@@ -2537,13 +2309,9 @@
       <c r="D61" s="9">
         <v>0.05</v>
       </c>
-      <c r="E61" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E61" s="57"/>
       <c r="F61" s="59"/>
-      <c r="G61" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G61" s="58"/>
       <c r="H61" s="58"/>
       <c r="I61" s="29" t="s">
         <v>73</v>
@@ -2562,13 +2330,9 @@
       <c r="D62" s="9">
         <v>0</v>
       </c>
-      <c r="E62" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E62" s="57"/>
       <c r="F62" s="59"/>
-      <c r="G62" s="58" t="s">
-        <v>11</v>
-      </c>
+      <c r="G62" s="58"/>
       <c r="H62" s="58"/>
       <c r="I62" s="29" t="s">
         <v>74</v>
@@ -2587,13 +2351,9 @@
       <c r="D63" s="9">
         <v>0.15</v>
       </c>
-      <c r="E63" s="57" t="s">
-        <v>11</v>
-      </c>
+      <c r="E63" s="57"/>
       <c r="F63" s="57"/>
-      <c r="G63" s="60" t="s">
-        <v>11</v>
-      </c>
+      <c r="G63" s="60"/>
       <c r="H63" s="59"/>
       <c r="I63" s="31" t="s">
         <v>75</v>
@@ -2674,7 +2434,7 @@
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.26953125" customWidth="1"/>
-    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="2" max="2" width="18.6328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.36328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.36328125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.36328125" bestFit="1" customWidth="1"/>
@@ -2687,30 +2447,30 @@
       <c r="B1" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="C1" s="64" t="s">
+      <c r="C1" s="65" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="63"/>
-      <c r="E1" s="66" t="s">
+      <c r="D1" s="64"/>
+      <c r="E1" s="67" t="s">
         <v>81</v>
       </c>
-      <c r="F1" s="63"/>
-      <c r="G1" s="65" t="s">
+      <c r="F1" s="64"/>
+      <c r="G1" s="66" t="s">
         <v>82</v>
       </c>
-      <c r="H1" s="63"/>
-      <c r="I1" s="69" t="s">
+      <c r="H1" s="64"/>
+      <c r="I1" s="70" t="s">
         <v>83</v>
       </c>
-      <c r="J1" s="63"/>
-      <c r="K1" s="67" t="s">
+      <c r="J1" s="64"/>
+      <c r="K1" s="68" t="s">
         <v>84</v>
       </c>
-      <c r="L1" s="68"/>
+      <c r="L1" s="69"/>
     </row>
     <row r="2" spans="1:13" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1"/>
-      <c r="B2" s="70" t="s">
+      <c r="B2" s="61" t="s">
         <v>87</v>
       </c>
       <c r="C2" s="2"/>
@@ -2743,7 +2503,7 @@
       </c>
       <c r="C3" s="43">
         <f>Datos!E4</f>
-        <v>55499</v>
+        <v>0</v>
       </c>
       <c r="D3" s="9" t="str">
         <f>IF(ISNUMBER($B$2),(C3/$B$2)-1,"INSERTAR COSTO")</f>
@@ -2759,7 +2519,7 @@
       </c>
       <c r="G3" s="45">
         <f>Datos!G4</f>
-        <v>58608</v>
+        <v>0</v>
       </c>
       <c r="H3" s="9" t="str">
         <f>IF(ISNUMBER($B$2),(G3/$B$2)-1,"INSERTAR COSTO")</f>
@@ -2773,15 +2533,14 @@
         <f>IF(ISNUMBER($B$2),(I3/$B$2)-1,"INSERTAR COSTO")</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K3" s="47"/>
+      <c r="K3" s="47">
+        <v>0</v>
+      </c>
       <c r="L3" s="9" t="str">
         <f>IF(ISNUMBER($B$2),(K3/$B$2)-1,"INSERTAR COSTO")</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="M3" s="36">
-        <f>K3*0.05</f>
-        <v>0</v>
-      </c>
+      <c r="M3" s="36"/>
     </row>
     <row r="4" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="str">
@@ -2792,7 +2551,7 @@
         <v>13</v>
       </c>
       <c r="C4" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E5),$C$3*(1-Datos!E5)/Datos!B5,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E5),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E5)/Datos!B5,"-")</f>
         <v>-</v>
       </c>
       <c r="D4" s="9" t="str">
@@ -2800,7 +2559,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E4" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F5),$E$3*(1-Datos!F5)/Datos!B5,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F5),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F5)/Datos!B5,"-")</f>
         <v>-</v>
       </c>
       <c r="F4" s="9" t="str">
@@ -2808,7 +2567,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G4" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G5),$G$3*(1-Datos!G5)/Datos!B5,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G5),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G5)/Datos!B5,"-")</f>
         <v>-</v>
       </c>
       <c r="H4" s="9" t="str">
@@ -2816,16 +2575,16 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="I4" s="8" t="str">
-        <f>IF(ISNUMBER(Datos!H5),$I$3*(1-Datos!H5)/Datos!B5,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!H5),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H5)/Datos!B5,"-")</f>
         <v>-</v>
       </c>
       <c r="J4" s="9" t="str">
         <f>IF(AND(ISNUMBER(I4),ISNUMBER($B$2)),((I4*Datos!$B5)/(1+Datos!$C5)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K4" s="48">
-        <f>$K$3*(1+Datos!D5)/Datos!B5</f>
-        <v>0</v>
+      <c r="K4" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D5),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D5)/Datos!B5,"-")</f>
+        <v>-</v>
       </c>
       <c r="L4" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K4*Datos!$B5)/(1+Datos!$C5)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -2841,7 +2600,7 @@
         <v>15</v>
       </c>
       <c r="C5" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E6),$C$3*(1+Datos!E6)/Datos!B6,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E6),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E6)/Datos!B6,"-")</f>
         <v>-</v>
       </c>
       <c r="D5" s="9" t="str">
@@ -2849,32 +2608,32 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E5" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F6),$E$3*(1+Datos!F6)/Datos!B6,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F6),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F6)/Datos!B6,"-")</f>
         <v>-</v>
       </c>
       <c r="F5" s="9" t="str">
         <f>IF(AND(ISNUMBER(E5),ISNUMBER($B$2)),((E5*Datos!$B6)/(1+Datos!$C6)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G5" s="48">
-        <f>IF(ISNUMBER(Datos!G6),$G$3*(1+Datos!G6)/Datos!B6,"-")</f>
-        <v>19536</v>
+      <c r="G5" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G6),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G6)/Datos!B6,"-")</f>
+        <v>-</v>
       </c>
       <c r="H5" s="9" t="str">
         <f>IF(AND(ISNUMBER(G5),ISNUMBER($B$2)),((G5*Datos!$B6)/(1+Datos!$C6)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I5" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H6),$I$3*(1+Datos!H6)/Datos!B6,"-")</f>
+      <c r="I5" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H6),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H6)/Datos!B6,"-")</f>
         <v>-</v>
       </c>
       <c r="J5" s="9" t="str">
         <f>IF(AND(ISNUMBER(I5),ISNUMBER($B$2)),((I5*Datos!$B6)/(1+Datos!$C6)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K5" s="48">
-        <f>$K$3*(1+Datos!D6)/Datos!B6</f>
-        <v>0</v>
+      <c r="K5" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D6),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D6)/Datos!B6,"-")</f>
+        <v>-</v>
       </c>
       <c r="L5" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K5*Datos!$B6)/(1+Datos!$C6)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -2890,7 +2649,7 @@
         <v>16</v>
       </c>
       <c r="C6" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E7),$C$3*(1+Datos!E7)/Datos!B7,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E7),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E7)/Datos!B7,"-")</f>
         <v>-</v>
       </c>
       <c r="D6" s="9" t="str">
@@ -2898,32 +2657,32 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E6" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F7),$E$3*(1+Datos!F7)/Datos!B7,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F7),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F7)/Datos!B7,"-")</f>
         <v>-</v>
       </c>
       <c r="F6" s="9" t="str">
         <f>IF(AND(ISNUMBER(E6),ISNUMBER($B$2)),((E6*Datos!$B7)/(1+Datos!$C7)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G6" s="48">
-        <f>IF(ISNUMBER(Datos!G7),$G$3*(1+Datos!G7)/Datos!B7,"-")</f>
-        <v>9768</v>
+      <c r="G6" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G7),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G7)/Datos!B7,"-")</f>
+        <v>-</v>
       </c>
       <c r="H6" s="9" t="str">
         <f>IF(AND(ISNUMBER(G6),ISNUMBER($B$2)),((G6*Datos!$B7)/(1+Datos!$C7)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I6" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H7),$I$3*(1+Datos!H7)/Datos!B7,"-")</f>
+      <c r="I6" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H7),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H7)/Datos!B7,"-")</f>
         <v>-</v>
       </c>
       <c r="J6" s="9" t="str">
         <f>IF(AND(ISNUMBER(I6),ISNUMBER($B$2)),((I6*Datos!$B7)/(1+Datos!$C7)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K6" s="48">
-        <f>$K$3*(1+Datos!D7)/Datos!B7</f>
-        <v>0</v>
+      <c r="K6" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D7),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D7)/Datos!B7,"-")</f>
+        <v>-</v>
       </c>
       <c r="L6" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K6*Datos!$B7)/(1+Datos!$C7)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -2939,7 +2698,7 @@
         <v>17</v>
       </c>
       <c r="C7" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E8),$C$3*(1+Datos!E8)/Datos!B8,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E8),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E8)/Datos!B8,"-")</f>
         <v>-</v>
       </c>
       <c r="D7" s="9" t="str">
@@ -2947,32 +2706,32 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E7" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F8),$E$3*(1+Datos!F8)/Datos!B8,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F8),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F8)/Datos!B8,"-")</f>
         <v>-</v>
       </c>
       <c r="F7" s="9" t="str">
         <f>IF(AND(ISNUMBER(E7),ISNUMBER($B$2)),((E7*Datos!$B8)/(1+Datos!$C8)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G7" s="48">
-        <f>IF(ISNUMBER(Datos!G8),$G$3*(1+Datos!G8)/Datos!B8,"-")</f>
-        <v>6512</v>
+      <c r="G7" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G8),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G8)/Datos!B8,"-")</f>
+        <v>-</v>
       </c>
       <c r="H7" s="9" t="str">
         <f>IF(AND(ISNUMBER(G7),ISNUMBER($B$2)),((G7*Datos!$B8)/(1+Datos!$C8)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I7" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H8),$I$3*(1+Datos!H8)/Datos!B8,"-")</f>
+      <c r="I7" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H8),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H8)/Datos!B8,"-")</f>
         <v>-</v>
       </c>
       <c r="J7" s="9" t="str">
         <f>IF(AND(ISNUMBER(I7),ISNUMBER($B$2)),((I7*Datos!$B8)/(1+Datos!$C8)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K7" s="48">
-        <f>$K$3*(1+Datos!D8)/Datos!B8</f>
-        <v>0</v>
+      <c r="K7" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D8),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D8)/Datos!B8,"-")</f>
+        <v>-</v>
       </c>
       <c r="L7" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K7*Datos!$B8)/(1+Datos!$C8)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -2988,7 +2747,7 @@
         <v>18</v>
       </c>
       <c r="C8" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E9),$C$3*(1+Datos!E9)/Datos!B9,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E9),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E9)/Datos!B9,"-")</f>
         <v>-</v>
       </c>
       <c r="D8" s="9" t="str">
@@ -2996,7 +2755,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E8" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F9),$E$3*(1+Datos!F9)/Datos!B9,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F9),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F9)/Datos!B9,"-")</f>
         <v>-</v>
       </c>
       <c r="F8" s="9" t="str">
@@ -3004,24 +2763,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G8" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G9),$G$3*(1+Datos!G9)/Datos!B9,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G9),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G9)/Datos!B9,"-")</f>
         <v>-</v>
       </c>
       <c r="H8" s="9" t="str">
         <f>IF(AND(ISNUMBER(G8),ISNUMBER($B$2)),((G8*Datos!$B9)/(1+Datos!$C9)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I8" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H9),$I$3*(1+Datos!H9)/Datos!B9,"-")</f>
+      <c r="I8" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H9),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H9)/Datos!B9,"-")</f>
         <v>-</v>
       </c>
       <c r="J8" s="9" t="str">
         <f>IF(AND(ISNUMBER(I8),ISNUMBER($B$2)),((I8*Datos!$B9)/(1+Datos!$C9)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K8" s="48">
-        <f>$K$3*(1+Datos!D9)/Datos!B9</f>
-        <v>0</v>
+      <c r="K8" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D9),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D9)/Datos!B9,"-")</f>
+        <v>-</v>
       </c>
       <c r="L8" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K8*Datos!$B9)/(1+Datos!$C9)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3037,7 +2796,7 @@
         <v>19</v>
       </c>
       <c r="C9" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E10),$C$3*(1+Datos!E10)/Datos!B10,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E10),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E10)/Datos!B10,"-")</f>
         <v>-</v>
       </c>
       <c r="D9" s="9" t="str">
@@ -3045,32 +2804,32 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E9" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F10),$E$3*(1+Datos!F10)/Datos!B10,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F10),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F10)/Datos!B10,"-")</f>
         <v>-</v>
       </c>
       <c r="F9" s="9" t="str">
         <f>IF(AND(ISNUMBER(E9),ISNUMBER($B$2)),((E9*Datos!$B10)/(1+Datos!$C10)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G9" s="48">
-        <f>IF(ISNUMBER(Datos!G10),$G$3*(1+Datos!G10)/Datos!B10,"-")</f>
-        <v>4884</v>
+      <c r="G9" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G10),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G10)/Datos!B10,"-")</f>
+        <v>-</v>
       </c>
       <c r="H9" s="9" t="str">
         <f>IF(AND(ISNUMBER(G9),ISNUMBER($B$2)),((G9*Datos!$B10)/(1+Datos!$C10)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I9" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H10),$I$3*(1+Datos!H10)/Datos!B10,"-")</f>
+      <c r="I9" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H10),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H10)/Datos!B10,"-")</f>
         <v>-</v>
       </c>
       <c r="J9" s="9" t="str">
         <f>IF(AND(ISNUMBER(I9),ISNUMBER($B$2)),((I9*Datos!$B10)/(1+Datos!$C10)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K9" s="48">
-        <f>$K$3*(1+Datos!D10)/Datos!B10</f>
-        <v>0</v>
+      <c r="K9" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D10),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D10)/Datos!B10,"-")</f>
+        <v>-</v>
       </c>
       <c r="L9" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K9*Datos!$B10)/(1+Datos!$C10)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3086,7 +2845,7 @@
         <v>20</v>
       </c>
       <c r="C10" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E11),$C$3*(1+Datos!E11)/Datos!B11,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E11),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E11)/Datos!B11,"-")</f>
         <v>-</v>
       </c>
       <c r="D10" s="9" t="str">
@@ -3094,7 +2853,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E10" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F11),$E$3*(1+Datos!F11)/Datos!B11,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F11),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F11)/Datos!B11,"-")</f>
         <v>-</v>
       </c>
       <c r="F10" s="9" t="str">
@@ -3102,24 +2861,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G10" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G11),$G$3*(1+Datos!G11)/Datos!B11,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G11),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G11)/Datos!B11,"-")</f>
         <v>-</v>
       </c>
       <c r="H10" s="9" t="str">
         <f>IF(AND(ISNUMBER(G10),ISNUMBER($B$2)),((G10*Datos!$B11)/(1+Datos!$C11)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I10" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H11),$I$3*(1+Datos!H11)/Datos!B11,"-")</f>
+      <c r="I10" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H11),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H11)/Datos!B11,"-")</f>
         <v>-</v>
       </c>
       <c r="J10" s="9" t="str">
         <f>IF(AND(ISNUMBER(I10),ISNUMBER($B$2)),((I10*Datos!$B11)/(1+Datos!$C11)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K10" s="48">
-        <f>$K$3*(1+Datos!D11)/Datos!B11</f>
-        <v>0</v>
+      <c r="K10" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D11),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D11)/Datos!B11,"-")</f>
+        <v>-</v>
       </c>
       <c r="L10" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K10*Datos!$B11)/(1+Datos!$C11)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3135,7 +2894,7 @@
         <v>21</v>
       </c>
       <c r="C11" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E12),$C$3*(1+Datos!E12)/Datos!B12,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E12),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E12)/Datos!B12,"-")</f>
         <v>-</v>
       </c>
       <c r="D11" s="9" t="str">
@@ -3143,7 +2902,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E11" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F12),$E$3*(1+Datos!F12)/Datos!B12,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F12),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F12)/Datos!B12,"-")</f>
         <v>-</v>
       </c>
       <c r="F11" s="9" t="str">
@@ -3151,24 +2910,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G11" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G12),$G$3*(1+Datos!G12)/Datos!B12,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G12),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G12)/Datos!B12,"-")</f>
         <v>-</v>
       </c>
       <c r="H11" s="9" t="str">
         <f>IF(AND(ISNUMBER(G11),ISNUMBER($B$2)),((G11*Datos!$B12)/(1+Datos!$C12)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I11" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H12),$I$3*(1+Datos!H12)/Datos!B12,"-")</f>
+      <c r="I11" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H12),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H12)/Datos!B12,"-")</f>
         <v>-</v>
       </c>
       <c r="J11" s="9" t="str">
         <f>IF(AND(ISNUMBER(I11),ISNUMBER($B$2)),((I11*Datos!$B12)/(1+Datos!$C12)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K11" s="48">
-        <f>$K$3*(1+Datos!D12)/Datos!B12</f>
-        <v>0</v>
+      <c r="K11" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D12),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D12)/Datos!B12,"-")</f>
+        <v>-</v>
       </c>
       <c r="L11" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K11*Datos!$B12)/(1+Datos!$C12)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3184,7 +2943,7 @@
         <v>22</v>
       </c>
       <c r="C12" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E13),$C$3*(1+Datos!E13)/Datos!B13,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E13),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E13)/Datos!B13,"-")</f>
         <v>-</v>
       </c>
       <c r="D12" s="9" t="str">
@@ -3192,32 +2951,32 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E12" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F13),$E$3*(1+Datos!F13)/Datos!B13,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F13),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F13)/Datos!B13,"-")</f>
         <v>-</v>
       </c>
       <c r="F12" s="9" t="str">
         <f>IF(AND(ISNUMBER(E12),ISNUMBER($B$2)),((E12*Datos!$B13)/(1+Datos!$C13)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G12" s="48">
-        <f>IF(ISNUMBER(Datos!G13),$G$3*(1+Datos!G13)/Datos!B13,"-")</f>
-        <v>3983.3904000000007</v>
+      <c r="G12" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G13),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G13)/Datos!B13,"-")</f>
+        <v>-</v>
       </c>
       <c r="H12" s="9" t="str">
         <f>IF(AND(ISNUMBER(G12),ISNUMBER($B$2)),((G12*Datos!$B13)/(1+Datos!$C13)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I12" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H13),$I$3*(1+Datos!H13)/Datos!B13,"-")</f>
+      <c r="I12" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H13),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H13)/Datos!B13,"-")</f>
         <v>-</v>
       </c>
       <c r="J12" s="9" t="str">
         <f>IF(AND(ISNUMBER(I12),ISNUMBER($B$2)),((I12*Datos!$B13)/(1+Datos!$C13)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K12" s="48">
-        <f>$K$3*(1+Datos!D13)/Datos!B13</f>
-        <v>0</v>
+      <c r="K12" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D13),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D13)/Datos!B13,"-")</f>
+        <v>-</v>
       </c>
       <c r="L12" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K12*Datos!$B13)/(1+Datos!$C13)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3233,7 +2992,7 @@
         <v>23</v>
       </c>
       <c r="C13" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E14),$C$3*(1+Datos!E14)/Datos!B14,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E14),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E14)/Datos!B14,"-")</f>
         <v>-</v>
       </c>
       <c r="D13" s="9" t="str">
@@ -3241,7 +3000,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E13" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F14),$E$3*(1+Datos!F14)/Datos!B14,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F14),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F14)/Datos!B14,"-")</f>
         <v>-</v>
       </c>
       <c r="F13" s="9" t="str">
@@ -3249,24 +3008,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G13" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G14),$G$3*(1+Datos!G14)/Datos!B14,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G14),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G14)/Datos!B14,"-")</f>
         <v>-</v>
       </c>
       <c r="H13" s="9" t="str">
         <f>IF(AND(ISNUMBER(G13),ISNUMBER($B$2)),((G13*Datos!$B14)/(1+Datos!$C14)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I13" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H14),$I$3*(1+Datos!H14)/Datos!B14,"-")</f>
+      <c r="I13" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H14),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H14)/Datos!B14,"-")</f>
         <v>-</v>
       </c>
       <c r="J13" s="9" t="str">
         <f>IF(AND(ISNUMBER(I13),ISNUMBER($B$2)),((I13*Datos!$B14)/(1+Datos!$C14)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K13" s="48">
-        <f>$K$3*(1+Datos!D14)/Datos!B14</f>
-        <v>0</v>
+      <c r="K13" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D14),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D14)/Datos!B14,"-")</f>
+        <v>-</v>
       </c>
       <c r="L13" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K13*Datos!$B14)/(1+Datos!$C14)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3282,7 +3041,7 @@
         <v>24</v>
       </c>
       <c r="C14" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E15),$C$3*(1+Datos!E15)/Datos!B15,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E15),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E15)/Datos!B15,"-")</f>
         <v>-</v>
       </c>
       <c r="D14" s="9" t="str">
@@ -3290,32 +3049,32 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E14" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F15),$E$3*(1+Datos!F15)/Datos!B15,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F15),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F15)/Datos!B15,"-")</f>
         <v>-</v>
       </c>
       <c r="F14" s="9" t="str">
         <f>IF(AND(ISNUMBER(E14),ISNUMBER($B$2)),((E14*Datos!$B15)/(1+Datos!$C15)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G14" s="48">
-        <f>IF(ISNUMBER(Datos!G15),$G$3*(1+Datos!G15)/Datos!B15,"-")</f>
-        <v>3484.5712000000003</v>
+      <c r="G14" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G15),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G15)/Datos!B15,"-")</f>
+        <v>-</v>
       </c>
       <c r="H14" s="9" t="str">
         <f>IF(AND(ISNUMBER(G14),ISNUMBER($B$2)),((G14*Datos!$B15)/(1+Datos!$C15)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I14" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H15),$I$3*(1+Datos!H15)/Datos!B15,"-")</f>
+      <c r="I14" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H15),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H15)/Datos!B15,"-")</f>
         <v>-</v>
       </c>
       <c r="J14" s="9" t="str">
         <f>IF(AND(ISNUMBER(I14),ISNUMBER($B$2)),((I14*Datos!$B15)/(1+Datos!$C15)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K14" s="48">
-        <f>$K$3*(1+Datos!D15)/Datos!B15</f>
-        <v>0</v>
+      <c r="K14" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D15),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D15)/Datos!B15,"-")</f>
+        <v>-</v>
       </c>
       <c r="L14" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K14*Datos!$B15)/(1+Datos!$C15)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3329,41 +3088,41 @@
       <c r="B15" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="48">
-        <f>IF(ISNUMBER(Datos!E16),$C$3*(1+Datos!E16)/Datos!B16,"-")</f>
-        <v>18499.666666666668</v>
+      <c r="C15" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!E16),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E16)/Datos!B16,"-")</f>
+        <v>-</v>
       </c>
       <c r="D15" s="9" t="str">
         <f>IF(AND(ISNUMBER(C15),ISNUMBER($B$2)),((C15*Datos!$B16)/(1+Datos!$C16)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E15" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F16),$E$3*(1+Datos!F16)/Datos!B16,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F16),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F16)/Datos!B16,"-")</f>
         <v>-</v>
       </c>
       <c r="F15" s="9" t="str">
         <f>IF(AND(ISNUMBER(E15),ISNUMBER($B$2)),((E15*Datos!$B16)/(1+Datos!$C16)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G15" s="48">
-        <f>IF(ISNUMBER(Datos!G16),$G$3*(1+Datos!G16)/Datos!B16,"-")</f>
-        <v>19536</v>
+      <c r="G15" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G16),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G16)/Datos!B16,"-")</f>
+        <v>-</v>
       </c>
       <c r="H15" s="9" t="str">
         <f>IF(AND(ISNUMBER(G15),ISNUMBER($B$2)),((G15*Datos!$B16)/(1+Datos!$C16)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I15" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H16),$I$3*(1+Datos!H16)/Datos!B16,"-")</f>
+      <c r="I15" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H16),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H16)/Datos!B16,"-")</f>
         <v>-</v>
       </c>
       <c r="J15" s="9" t="str">
         <f>IF(AND(ISNUMBER(I15),ISNUMBER($B$2)),((I15*Datos!$B16)/(1+Datos!$C16)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K15" s="48">
-        <f>$K$3*(1+Datos!D16)/Datos!B16</f>
-        <v>0</v>
+      <c r="K15" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D16),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D16)/Datos!B16,"-")</f>
+        <v>-</v>
       </c>
       <c r="L15" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K15*Datos!$B16)/(1+Datos!$C16)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3377,41 +3136,41 @@
       <c r="B16" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="48">
-        <f>IF(ISNUMBER(Datos!E17),$C$3*(1+Datos!E17)/Datos!B17,"-")</f>
-        <v>9249.8333333333339</v>
+      <c r="C16" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!E17),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E17)/Datos!B17,"-")</f>
+        <v>-</v>
       </c>
       <c r="D16" s="9" t="str">
         <f>IF(AND(ISNUMBER(C16),ISNUMBER($B$2)),((C16*Datos!$B17)/(1+Datos!$C17)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E16" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F17),$E$3*(1+Datos!F17)/Datos!B17,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F17),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F17)/Datos!B17,"-")</f>
         <v>-</v>
       </c>
       <c r="F16" s="9" t="str">
         <f>IF(AND(ISNUMBER(E16),ISNUMBER($B$2)),((E16*Datos!$B17)/(1+Datos!$C17)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G16" s="48">
-        <f>IF(ISNUMBER(Datos!G17),$G$3*(1+Datos!G17)/Datos!B17,"-")</f>
-        <v>9768</v>
+      <c r="G16" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G17),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G17)/Datos!B17,"-")</f>
+        <v>-</v>
       </c>
       <c r="H16" s="9" t="str">
         <f>IF(AND(ISNUMBER(G16),ISNUMBER($B$2)),((G16*Datos!$B17)/(1+Datos!$C17)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I16" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H17),$I$3*(1+Datos!H17)/Datos!B17,"-")</f>
+      <c r="I16" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H17),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H17)/Datos!B17,"-")</f>
         <v>-</v>
       </c>
       <c r="J16" s="9" t="str">
         <f>IF(AND(ISNUMBER(I16),ISNUMBER($B$2)),((I16*Datos!$B17)/(1+Datos!$C17)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K16" s="48">
-        <f>$K$3*(1+Datos!D17)/Datos!B17</f>
-        <v>0</v>
+      <c r="K16" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D17),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D17)/Datos!B17,"-")</f>
+        <v>-</v>
       </c>
       <c r="L16" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K16*Datos!$B17)/(1+Datos!$C17)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3425,41 +3184,41 @@
       <c r="B17" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="48">
-        <f>IF(ISNUMBER(Datos!E18),$C$3*(1+Datos!E18)/Datos!B18,"-")</f>
-        <v>4624.916666666667</v>
+      <c r="C17" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!E18),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E18)/Datos!B18,"-")</f>
+        <v>-</v>
       </c>
       <c r="D17" s="9" t="str">
         <f>IF(AND(ISNUMBER(C17),ISNUMBER($B$2)),((C17*Datos!$B18)/(1+Datos!$C18)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E17" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F18),$E$3*(1+Datos!F18)/Datos!B18,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F18),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F18)/Datos!B18,"-")</f>
         <v>-</v>
       </c>
       <c r="F17" s="9" t="str">
         <f>IF(AND(ISNUMBER(E17),ISNUMBER($B$2)),((E17*Datos!$B18)/(1+Datos!$C18)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G17" s="48">
-        <f>IF(ISNUMBER(Datos!G18),$G$3*(1+Datos!G18)/Datos!B18,"-")</f>
-        <v>4884</v>
+      <c r="G17" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G18),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G18)/Datos!B18,"-")</f>
+        <v>-</v>
       </c>
       <c r="H17" s="9" t="str">
         <f>IF(AND(ISNUMBER(G17),ISNUMBER($B$2)),((G17*Datos!$B18)/(1+Datos!$C18)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I17" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H18),$I$3*(1+Datos!H18)/Datos!B18,"-")</f>
+      <c r="I17" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H18),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H18)/Datos!B18,"-")</f>
         <v>-</v>
       </c>
       <c r="J17" s="9" t="str">
         <f>IF(AND(ISNUMBER(I17),ISNUMBER($B$2)),((I17*Datos!$B18)/(1+Datos!$C18)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K17" s="48">
-        <f>$K$3*(1+Datos!D18)/Datos!B18</f>
-        <v>0</v>
+      <c r="K17" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D18),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D18)/Datos!B18,"-")</f>
+        <v>-</v>
       </c>
       <c r="L17" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K17*Datos!$B18)/(1+Datos!$C18)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3473,41 +3232,41 @@
       <c r="B18" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="48">
-        <f>IF(ISNUMBER(Datos!E19),$C$3*(1+Datos!E19)/Datos!B19,"-")</f>
-        <v>4624.916666666667</v>
+      <c r="C18" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!E19),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E19)/Datos!B19,"-")</f>
+        <v>-</v>
       </c>
       <c r="D18" s="9" t="str">
         <f>IF(AND(ISNUMBER(C18),ISNUMBER($B$2)),((C18*Datos!$B19)/(1+Datos!$C19)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E18" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F19),$E$3*(1+Datos!F19)/Datos!B19,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F19),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F19)/Datos!B19,"-")</f>
         <v>-</v>
       </c>
       <c r="F18" s="9" t="str">
         <f>IF(AND(ISNUMBER(E18),ISNUMBER($B$2)),((E18*Datos!$B19)/(1+Datos!$C19)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G18" s="48">
-        <f>IF(ISNUMBER(Datos!G19),$G$3*(1+Datos!G19)/Datos!B19,"-")</f>
-        <v>4884</v>
+      <c r="G18" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G19),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G19)/Datos!B19,"-")</f>
+        <v>-</v>
       </c>
       <c r="H18" s="9" t="str">
         <f>IF(AND(ISNUMBER(G18),ISNUMBER($B$2)),((G18*Datos!$B19)/(1+Datos!$C19)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I18" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H19),$I$3*(1+Datos!H19)/Datos!B19,"-")</f>
+      <c r="I18" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H19),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H19)/Datos!B19,"-")</f>
         <v>-</v>
       </c>
       <c r="J18" s="9" t="str">
         <f>IF(AND(ISNUMBER(I18),ISNUMBER($B$2)),((I18*Datos!$B19)/(1+Datos!$C19)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K18" s="48">
-        <f>$K$3*(1+Datos!D19)/Datos!B19</f>
-        <v>0</v>
+      <c r="K18" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D19),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D19)/Datos!B19,"-")</f>
+        <v>-</v>
       </c>
       <c r="L18" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K18*Datos!$B19)/(1+Datos!$C19)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3521,16 +3280,16 @@
       <c r="B19" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="48">
-        <f>IF(ISNUMBER(Datos!E20),$C$3*(1+Datos!E20)/Datos!B20,"-")</f>
-        <v>3699.9333333333334</v>
+      <c r="C19" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!E20),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E20)/Datos!B20,"-")</f>
+        <v>-</v>
       </c>
       <c r="D19" s="9" t="str">
         <f>IF(AND(ISNUMBER(C19),ISNUMBER($B$2)),((C19*Datos!$B20)/(1+Datos!$C20)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E19" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F20),$E$3*(1+Datos!F20)/Datos!B20,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F20),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F20)/Datos!B20,"-")</f>
         <v>-</v>
       </c>
       <c r="F19" s="9" t="str">
@@ -3538,24 +3297,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G19" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G20),$G$3*(1+Datos!G20)/Datos!B20,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G20),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G20)/Datos!B20,"-")</f>
         <v>-</v>
       </c>
       <c r="H19" s="9" t="str">
         <f>IF(AND(ISNUMBER(G19),ISNUMBER($B$2)),((G19*Datos!$B20)/(1+Datos!$C20)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I19" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H20),$I$3*(1+Datos!H20)/Datos!B20,"-")</f>
+      <c r="I19" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H20),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H20)/Datos!B20,"-")</f>
         <v>-</v>
       </c>
       <c r="J19" s="9" t="str">
         <f>IF(AND(ISNUMBER(I19),ISNUMBER($B$2)),((I19*Datos!$B20)/(1+Datos!$C20)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K19" s="48">
-        <f>$K$3*(1+Datos!D20)/Datos!B20</f>
-        <v>0</v>
+      <c r="K19" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D20),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D20)/Datos!B20,"-")</f>
+        <v>-</v>
       </c>
       <c r="L19" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K19*Datos!$B20)/(1+Datos!$C20)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3570,7 +3329,7 @@
         <v>31</v>
       </c>
       <c r="C20" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E21),$C$3*(1+Datos!E21)/Datos!B21,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E21),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E21)/Datos!B21,"-")</f>
         <v>-</v>
       </c>
       <c r="D20" s="9" t="str">
@@ -3578,32 +3337,32 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E20" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F21),$E$3*(1+Datos!F21)/Datos!B21,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F21),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F21)/Datos!B21,"-")</f>
         <v>-</v>
       </c>
       <c r="F20" s="9" t="str">
         <f>IF(AND(ISNUMBER(E20),ISNUMBER($B$2)),((E20*Datos!$B21)/(1+Datos!$C21)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G20" s="48">
-        <f>IF(ISNUMBER(Datos!G21),$G$3*(1+Datos!G21)/Datos!B21,"-")</f>
-        <v>3983.3904000000007</v>
+      <c r="G20" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G21),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G21)/Datos!B21,"-")</f>
+        <v>-</v>
       </c>
       <c r="H20" s="9" t="str">
         <f>IF(AND(ISNUMBER(G20),ISNUMBER($B$2)),((G20*Datos!$B21)/(1+Datos!$C21)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I20" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H21),$I$3*(1+Datos!H21)/Datos!B21,"-")</f>
+      <c r="I20" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H21),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H21)/Datos!B21,"-")</f>
         <v>-</v>
       </c>
       <c r="J20" s="9" t="str">
         <f>IF(AND(ISNUMBER(I20),ISNUMBER($B$2)),((I20*Datos!$B21)/(1+Datos!$C21)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K20" s="48">
-        <f>$K$3*(1+Datos!D21)/Datos!B21</f>
-        <v>0</v>
+      <c r="K20" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D21),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D21)/Datos!B21,"-")</f>
+        <v>-</v>
       </c>
       <c r="L20" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K20*Datos!$B21)/(1+Datos!$C21)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3618,7 +3377,7 @@
         <v>32</v>
       </c>
       <c r="C21" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E22),$C$3*(1+Datos!E22)/Datos!B22,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E22),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E22)/Datos!B22,"-")</f>
         <v>-</v>
       </c>
       <c r="D21" s="9" t="str">
@@ -3626,7 +3385,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E21" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F22),$E$3*(1+Datos!F22)/Datos!B22,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F22),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F22)/Datos!B22,"-")</f>
         <v>-</v>
       </c>
       <c r="F21" s="9" t="str">
@@ -3634,24 +3393,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G21" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G22),$G$3*(1+Datos!G22)/Datos!B22,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G22),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G22)/Datos!B22,"-")</f>
         <v>-</v>
       </c>
       <c r="H21" s="9" t="str">
         <f>IF(AND(ISNUMBER(G21),ISNUMBER($B$2)),((G21*Datos!$B22)/(1+Datos!$C22)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I21" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H22),$I$3*(1+Datos!H22)/Datos!B22,"-")</f>
+      <c r="I21" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H22),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H22)/Datos!B22,"-")</f>
         <v>-</v>
       </c>
       <c r="J21" s="9" t="str">
         <f>IF(AND(ISNUMBER(I21),ISNUMBER($B$2)),((I21*Datos!$B22)/(1+Datos!$C22)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K21" s="48">
-        <f>$K$3*(1+Datos!D22)/Datos!B22</f>
-        <v>0</v>
+      <c r="K21" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D22),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D22)/Datos!B22,"-")</f>
+        <v>-</v>
       </c>
       <c r="L21" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K21*Datos!$B22)/(1+Datos!$C22)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3665,41 +3424,41 @@
       <c r="B22" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="48">
-        <f>IF(ISNUMBER(Datos!E23),$C$3*(1+Datos!E23)/Datos!B23,"-")</f>
-        <v>3177.6199112222221</v>
+      <c r="C22" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!E23),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E23)/Datos!B23,"-")</f>
+        <v>-</v>
       </c>
       <c r="D22" s="9" t="str">
         <f>IF(AND(ISNUMBER(C22),ISNUMBER($B$2)),((C22*Datos!$B23)/(1+Datos!$C23)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E22" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F23),$E$3*(1+Datos!F23)/Datos!B23,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F23),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F23)/Datos!B23,"-")</f>
         <v>-</v>
       </c>
       <c r="F22" s="9" t="str">
         <f>IF(AND(ISNUMBER(E22),ISNUMBER($B$2)),((E22*Datos!$B23)/(1+Datos!$C23)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G22" s="48">
-        <f>IF(ISNUMBER(Datos!G23),$G$3*(1+Datos!G23)/Datos!B23,"-")</f>
-        <v>3484.5712000000003</v>
+      <c r="G22" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G23),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G23)/Datos!B23,"-")</f>
+        <v>-</v>
       </c>
       <c r="H22" s="9" t="str">
         <f>IF(AND(ISNUMBER(G22),ISNUMBER($B$2)),((G22*Datos!$B23)/(1+Datos!$C23)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I22" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H23),$I$3*(1+Datos!H23)/Datos!B23,"-")</f>
+      <c r="I22" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H23),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H23)/Datos!B23,"-")</f>
         <v>-</v>
       </c>
       <c r="J22" s="9" t="str">
         <f>IF(AND(ISNUMBER(I22),ISNUMBER($B$2)),((I22*Datos!$B23)/(1+Datos!$C23)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K22" s="48">
-        <f>$K$3*(1+Datos!D23)/Datos!B23</f>
-        <v>0</v>
+      <c r="K22" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D23),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D23)/Datos!B23,"-")</f>
+        <v>-</v>
       </c>
       <c r="L22" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K22*Datos!$B23)/(1+Datos!$C23)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3714,7 +3473,7 @@
         <v>34</v>
       </c>
       <c r="C23" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E24),$C$3*(1+Datos!E24)/Datos!B24,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E24),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E24)/Datos!B24,"-")</f>
         <v>-</v>
       </c>
       <c r="D23" s="9" t="str">
@@ -3722,7 +3481,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E23" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F24),$E$3*(1+Datos!F24)/Datos!B24,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F24),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F24)/Datos!B24,"-")</f>
         <v>-</v>
       </c>
       <c r="F23" s="9" t="str">
@@ -3730,24 +3489,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G23" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G24),$G$3*(1+Datos!G24)/Datos!B24,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G24),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G24)/Datos!B24,"-")</f>
         <v>-</v>
       </c>
       <c r="H23" s="9" t="str">
         <f>IF(AND(ISNUMBER(G23),ISNUMBER($B$2)),((G23*Datos!$B24)/(1+Datos!$C24)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I23" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H24),$I$3*(1+Datos!H24)/Datos!B24,"-")</f>
+      <c r="I23" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H24),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H24)/Datos!B24,"-")</f>
         <v>-</v>
       </c>
       <c r="J23" s="9" t="str">
         <f>IF(AND(ISNUMBER(I23),ISNUMBER($B$2)),((I23*Datos!$B24)/(1+Datos!$C24)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K23" s="48">
-        <f>$K$3*(1+Datos!D24)/Datos!B24</f>
-        <v>0</v>
+      <c r="K23" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D24),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D24)/Datos!B24,"-")</f>
+        <v>-</v>
       </c>
       <c r="L23" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K23*Datos!$B24)/(1+Datos!$C24)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3761,41 +3520,41 @@
       <c r="B24" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="48">
-        <f>IF(ISNUMBER(Datos!E25),$C$3*(1+Datos!E25)/Datos!B25,"-")</f>
-        <v>3024.6899500999998</v>
+      <c r="C24" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!E25),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E25)/Datos!B25,"-")</f>
+        <v>-</v>
       </c>
       <c r="D24" s="9" t="str">
         <f>IF(AND(ISNUMBER(C24),ISNUMBER($B$2)),((C24*Datos!$B25)/(1+Datos!$C25)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E24" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F25),$E$3*(1+Datos!F25)/Datos!B25,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F25),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F25)/Datos!B25,"-")</f>
         <v>-</v>
       </c>
       <c r="F24" s="9" t="str">
         <f>IF(AND(ISNUMBER(E24),ISNUMBER($B$2)),((E24*Datos!$B25)/(1+Datos!$C25)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G24" s="48">
-        <f>IF(ISNUMBER(Datos!G25),$G$3*(1+Datos!G25)/Datos!B25,"-")</f>
-        <v>3223.44</v>
+      <c r="G24" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G25),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G25)/Datos!B25,"-")</f>
+        <v>-</v>
       </c>
       <c r="H24" s="9" t="str">
         <f>IF(AND(ISNUMBER(G24),ISNUMBER($B$2)),((G24*Datos!$B25)/(1+Datos!$C25)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I24" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H25),$I$3*(1+Datos!H25)/Datos!B25,"-")</f>
+      <c r="I24" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H25),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H25)/Datos!B25,"-")</f>
         <v>-</v>
       </c>
       <c r="J24" s="9" t="str">
         <f>IF(AND(ISNUMBER(I24),ISNUMBER($B$2)),((I24*Datos!$B25)/(1+Datos!$C25)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K24" s="48">
-        <f>$K$3*(1+Datos!D25)/Datos!B25</f>
-        <v>0</v>
+      <c r="K24" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D25),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D25)/Datos!B25,"-")</f>
+        <v>-</v>
       </c>
       <c r="L24" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K24*Datos!$B25)/(1+Datos!$C25)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3811,7 +3570,7 @@
         <v>13</v>
       </c>
       <c r="C25" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E26),$C$3*(1+Datos!E26)/Datos!B26,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E26),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E26)/Datos!B26,"-")</f>
         <v>-</v>
       </c>
       <c r="D25" s="9" t="str">
@@ -3819,7 +3578,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E25" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F26),$E$3*(1+Datos!F26)/Datos!B26,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F26),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F26)/Datos!B26,"-")</f>
         <v>-</v>
       </c>
       <c r="F25" s="9" t="str">
@@ -3827,24 +3586,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G25" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G26),$G$3*(1+Datos!G26)/Datos!B26,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G26),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G26)/Datos!B26,"-")</f>
         <v>-</v>
       </c>
       <c r="H25" s="9" t="str">
         <f>IF(AND(ISNUMBER(G25),ISNUMBER($B$2)),((G25*Datos!$B26)/(1+Datos!$C26)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I25" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H26),$I$3*(1+Datos!H26)/Datos!B26,"-")</f>
+      <c r="I25" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H26),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H26)/Datos!B26,"-")</f>
         <v>-</v>
       </c>
       <c r="J25" s="9" t="str">
         <f>IF(AND(ISNUMBER(I25),ISNUMBER($B$2)),((I25*Datos!$B26)/(1+Datos!$C26)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K25" s="48">
-        <f>$K$3*(1+Datos!D26)/Datos!B26</f>
-        <v>0</v>
+      <c r="K25" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D26),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D26)/Datos!B26,"-")</f>
+        <v>-</v>
       </c>
       <c r="L25" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K25*Datos!$B26)/(1+Datos!$C26)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3859,41 +3618,41 @@
       <c r="B26" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="C26" s="48">
-        <f>IF(ISNUMBER(Datos!E27),$C$3*(1+Datos!E27)/Datos!B27,"-")</f>
-        <v>18499.666666666668</v>
+      <c r="C26" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!E27),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E27)/Datos!B27,"-")</f>
+        <v>-</v>
       </c>
       <c r="D26" s="9" t="str">
         <f>IF(AND(ISNUMBER(C26),ISNUMBER($B$2)),((C26*Datos!$B27)/(1+Datos!$C27)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E26" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F27),$E$3*(1+Datos!F27)/Datos!B27,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F27),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F27)/Datos!B27,"-")</f>
         <v>-</v>
       </c>
       <c r="F26" s="9" t="str">
         <f>IF(AND(ISNUMBER(E26),ISNUMBER($B$2)),((E26*Datos!$B27)/(1+Datos!$C27)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G26" s="48">
-        <f>IF(ISNUMBER(Datos!G27),$G$3*(1+Datos!G27)/Datos!B27,"-")</f>
-        <v>19536</v>
+      <c r="G26" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G27),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G27)/Datos!B27,"-")</f>
+        <v>-</v>
       </c>
       <c r="H26" s="9" t="str">
         <f>IF(AND(ISNUMBER(G26),ISNUMBER($B$2)),((G26*Datos!$B27)/(1+Datos!$C27)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I26" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H27),$I$3*(1+Datos!H27)/Datos!B27,"-")</f>
+      <c r="I26" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H27),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H27)/Datos!B27,"-")</f>
         <v>-</v>
       </c>
       <c r="J26" s="9" t="str">
         <f>IF(AND(ISNUMBER(I26),ISNUMBER($B$2)),((I26*Datos!$B27)/(1+Datos!$C27)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K26" s="48">
-        <f>$K$3*(1+Datos!D27)/Datos!B27</f>
-        <v>0</v>
+      <c r="K26" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D27),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D27)/Datos!B27,"-")</f>
+        <v>-</v>
       </c>
       <c r="L26" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K26*Datos!$B27)/(1+Datos!$C27)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3908,41 +3667,41 @@
       <c r="B27" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="C27" s="48">
-        <f>IF(ISNUMBER(Datos!E28),$C$3*(1+Datos!E28)/Datos!B28,"-")</f>
-        <v>9249.8333333333339</v>
+      <c r="C27" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!E28),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E28)/Datos!B28,"-")</f>
+        <v>-</v>
       </c>
       <c r="D27" s="9" t="str">
         <f>IF(AND(ISNUMBER(C27),ISNUMBER($B$2)),((C27*Datos!$B28)/(1+Datos!$C28)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E27" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F28),$E$3*(1+Datos!F28)/Datos!B28,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F28),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F28)/Datos!B28,"-")</f>
         <v>-</v>
       </c>
       <c r="F27" s="9" t="str">
         <f>IF(AND(ISNUMBER(E27),ISNUMBER($B$2)),((E27*Datos!$B28)/(1+Datos!$C28)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G27" s="48">
-        <f>IF(ISNUMBER(Datos!G28),$G$3*(1+Datos!G28)/Datos!B28,"-")</f>
-        <v>9768</v>
+      <c r="G27" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G28),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G28)/Datos!B28,"-")</f>
+        <v>-</v>
       </c>
       <c r="H27" s="9" t="str">
         <f>IF(AND(ISNUMBER(G27),ISNUMBER($B$2)),((G27*Datos!$B28)/(1+Datos!$C28)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I27" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H28),$I$3*(1+Datos!H28)/Datos!B28,"-")</f>
+      <c r="I27" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H28),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H28)/Datos!B28,"-")</f>
         <v>-</v>
       </c>
       <c r="J27" s="9" t="str">
         <f>IF(AND(ISNUMBER(I27),ISNUMBER($B$2)),((I27*Datos!$B28)/(1+Datos!$C28)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K27" s="48">
-        <f>$K$3*(1+Datos!D28)/Datos!B28</f>
-        <v>0</v>
+      <c r="K27" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D28),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D28)/Datos!B28,"-")</f>
+        <v>-</v>
       </c>
       <c r="L27" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K27*Datos!$B28)/(1+Datos!$C28)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -3957,41 +3716,41 @@
       <c r="B28" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="C28" s="48">
-        <f>IF(ISNUMBER(Datos!E29),$C$3*(1+Datos!E29)/Datos!B29,"-")</f>
-        <v>6166.5555555555557</v>
+      <c r="C28" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!E29),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E29)/Datos!B29,"-")</f>
+        <v>-</v>
       </c>
       <c r="D28" s="9" t="str">
         <f>IF(AND(ISNUMBER(C28),ISNUMBER($B$2)),((C28*Datos!$B29)/(1+Datos!$C29)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E28" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F29),$E$3*(1+Datos!F29)/Datos!B29,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F29),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F29)/Datos!B29,"-")</f>
         <v>-</v>
       </c>
       <c r="F28" s="9" t="str">
         <f>IF(AND(ISNUMBER(E28),ISNUMBER($B$2)),((E28*Datos!$B29)/(1+Datos!$C29)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G28" s="48">
-        <f>IF(ISNUMBER(Datos!G29),$G$3*(1+Datos!G29)/Datos!B29,"-")</f>
-        <v>6512</v>
+      <c r="G28" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G29),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G29)/Datos!B29,"-")</f>
+        <v>-</v>
       </c>
       <c r="H28" s="9" t="str">
         <f>IF(AND(ISNUMBER(G28),ISNUMBER($B$2)),((G28*Datos!$B29)/(1+Datos!$C29)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I28" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H29),$I$3*(1+Datos!H29)/Datos!B29,"-")</f>
+      <c r="I28" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H29),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H29)/Datos!B29,"-")</f>
         <v>-</v>
       </c>
       <c r="J28" s="9" t="str">
         <f>IF(AND(ISNUMBER(I28),ISNUMBER($B$2)),((I28*Datos!$B29)/(1+Datos!$C29)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K28" s="48">
-        <f>$K$3*(1+Datos!D29)/Datos!B29</f>
-        <v>0</v>
+      <c r="K28" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D29),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D29)/Datos!B29,"-")</f>
+        <v>-</v>
       </c>
       <c r="L28" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K28*Datos!$B29)/(1+Datos!$C29)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4007,7 +3766,7 @@
         <v>40</v>
       </c>
       <c r="C29" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E30),$C$3*(1+Datos!E30)/Datos!B30,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E30),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E30)/Datos!B30,"-")</f>
         <v>-</v>
       </c>
       <c r="D29" s="9" t="str">
@@ -4015,7 +3774,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E29" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F30),$E$3*(1+Datos!F30)/Datos!B30,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F30),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F30)/Datos!B30,"-")</f>
         <v>-</v>
       </c>
       <c r="F29" s="9" t="str">
@@ -4023,24 +3782,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G29" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G30),$G$3*(1+Datos!G30)/Datos!B30,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G30),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G30)/Datos!B30,"-")</f>
         <v>-</v>
       </c>
       <c r="H29" s="9" t="str">
         <f>IF(AND(ISNUMBER(G29),ISNUMBER($B$2)),((G29*Datos!$B30)/(1+Datos!$C30)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I29" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H30),$I$3*(1+Datos!H30)/Datos!B30,"-")</f>
+      <c r="I29" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H30),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H30)/Datos!B30,"-")</f>
         <v>-</v>
       </c>
       <c r="J29" s="9" t="str">
         <f>IF(AND(ISNUMBER(I29),ISNUMBER($B$2)),((I29*Datos!$B30)/(1+Datos!$C30)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K29" s="48">
-        <f>$K$3*(1+Datos!D30)/Datos!B30</f>
-        <v>0</v>
+      <c r="K29" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D30),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D30)/Datos!B30,"-")</f>
+        <v>-</v>
       </c>
       <c r="L29" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K29*Datos!$B30)/(1+Datos!$C30)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4056,7 +3815,7 @@
         <v>41</v>
       </c>
       <c r="C30" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E31),$C$3*(1+Datos!E31)/Datos!B31,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E31),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E31)/Datos!B31,"-")</f>
         <v>-</v>
       </c>
       <c r="D30" s="9" t="str">
@@ -4064,32 +3823,32 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E30" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F31),$E$3*(1+Datos!F31)/Datos!B31,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F31),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F31)/Datos!B31,"-")</f>
         <v>-</v>
       </c>
       <c r="F30" s="9" t="str">
         <f>IF(AND(ISNUMBER(E30),ISNUMBER($B$2)),((E30*Datos!$B31)/(1+Datos!$C31)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G30" s="48">
-        <f>IF(ISNUMBER(Datos!G31),$G$3*(1+Datos!G31)/Datos!B31,"-")</f>
-        <v>5860.8</v>
+      <c r="G30" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G31),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G31)/Datos!B31,"-")</f>
+        <v>-</v>
       </c>
       <c r="H30" s="9" t="str">
         <f>IF(AND(ISNUMBER(G30),ISNUMBER($B$2)),((G30*Datos!$B31)/(1+Datos!$C31)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I30" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H31),$I$3*(1+Datos!H31)/Datos!B31,"-")</f>
+      <c r="I30" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H31),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H31)/Datos!B31,"-")</f>
         <v>-</v>
       </c>
       <c r="J30" s="9" t="str">
         <f>IF(AND(ISNUMBER(I30),ISNUMBER($B$2)),((I30*Datos!$B31)/(1+Datos!$C31)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K30" s="48">
-        <f>$K$3*(1+Datos!D31)/Datos!B31</f>
-        <v>0</v>
+      <c r="K30" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D31),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D31)/Datos!B31,"-")</f>
+        <v>-</v>
       </c>
       <c r="L30" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K30*Datos!$B31)/(1+Datos!$C31)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4105,7 +3864,7 @@
         <v>42</v>
       </c>
       <c r="C31" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E32),$C$3*(1+Datos!E32)/Datos!B32,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E32),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E32)/Datos!B32,"-")</f>
         <v>-</v>
       </c>
       <c r="D31" s="9" t="str">
@@ -4113,7 +3872,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E31" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F32),$E$3*(1+Datos!F32)/Datos!B32,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F32),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F32)/Datos!B32,"-")</f>
         <v>-</v>
       </c>
       <c r="F31" s="9" t="str">
@@ -4121,24 +3880,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G31" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G32),$G$3*(1+Datos!G32)/Datos!B32,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G32),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G32)/Datos!B32,"-")</f>
         <v>-</v>
       </c>
       <c r="H31" s="9" t="str">
         <f>IF(AND(ISNUMBER(G31),ISNUMBER($B$2)),((G31*Datos!$B32)/(1+Datos!$C32)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I31" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H32),$I$3*(1+Datos!H32)/Datos!B32,"-")</f>
+      <c r="I31" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H32),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H32)/Datos!B32,"-")</f>
         <v>-</v>
       </c>
       <c r="J31" s="9" t="str">
         <f>IF(AND(ISNUMBER(I31),ISNUMBER($B$2)),((I31*Datos!$B32)/(1+Datos!$C32)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K31" s="48">
-        <f>$K$3*(1+Datos!D32)/Datos!B32</f>
-        <v>0</v>
+      <c r="K31" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D32),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D32)/Datos!B32,"-")</f>
+        <v>-</v>
       </c>
       <c r="L31" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K31*Datos!$B32)/(1+Datos!$C32)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4153,16 +3912,16 @@
       <c r="B32" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="C32" s="48">
-        <f>IF(ISNUMBER(Datos!E33),$C$3*(1+Datos!E33)/Datos!B33,"-")</f>
-        <v>4624.916666666667</v>
+      <c r="C32" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!E33),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E33)/Datos!B33,"-")</f>
+        <v>-</v>
       </c>
       <c r="D32" s="9" t="str">
         <f>IF(AND(ISNUMBER(C32),ISNUMBER($B$2)),((C32*Datos!$B33)/(1+Datos!$C33)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E32" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F33),$E$3*(1+Datos!F33)/Datos!B33,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F33),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F33)/Datos!B33,"-")</f>
         <v>-</v>
       </c>
       <c r="F32" s="9" t="str">
@@ -4170,24 +3929,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G32" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G33),$G$3*(1+Datos!G33)/Datos!B33,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G33),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G33)/Datos!B33,"-")</f>
         <v>-</v>
       </c>
       <c r="H32" s="9" t="str">
         <f>IF(AND(ISNUMBER(G32),ISNUMBER($B$2)),((G32*Datos!$B33)/(1+Datos!$C33)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I32" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H33),$I$3*(1+Datos!H33)/Datos!B33,"-")</f>
+      <c r="I32" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H33),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H33)/Datos!B33,"-")</f>
         <v>-</v>
       </c>
       <c r="J32" s="9" t="str">
         <f>IF(AND(ISNUMBER(I32),ISNUMBER($B$2)),((I32*Datos!$B33)/(1+Datos!$C33)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K32" s="48">
-        <f>$K$3*(1+Datos!D33)/Datos!B33</f>
-        <v>0</v>
+      <c r="K32" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D33),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D33)/Datos!B33,"-")</f>
+        <v>-</v>
       </c>
       <c r="L32" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K32*Datos!$B33)/(1+Datos!$C33)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4203,7 +3962,7 @@
         <v>44</v>
       </c>
       <c r="C33" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E34),$C$3*(1+Datos!E34)/Datos!B34,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E34),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E34)/Datos!B34,"-")</f>
         <v>-</v>
       </c>
       <c r="D33" s="9" t="str">
@@ -4211,32 +3970,32 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E33" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F34),$E$3*(1+Datos!F34)/Datos!B34,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F34),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F34)/Datos!B34,"-")</f>
         <v>-</v>
       </c>
       <c r="F33" s="9" t="str">
         <f>IF(AND(ISNUMBER(E33),ISNUMBER($B$2)),((E33*Datos!$B34)/(1+Datos!$C34)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="G33" s="48">
-        <f>IF(ISNUMBER(Datos!G34),$G$3*(1+Datos!G34)/Datos!B34,"-")</f>
-        <v>5323.56</v>
+      <c r="G33" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G34),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G34)/Datos!B34,"-")</f>
+        <v>-</v>
       </c>
       <c r="H33" s="9" t="str">
         <f>IF(AND(ISNUMBER(G33),ISNUMBER($B$2)),((G33*Datos!$B34)/(1+Datos!$C34)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I33" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H34),$I$3*(1+Datos!H34)/Datos!B34,"-")</f>
+      <c r="I33" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H34),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H34)/Datos!B34,"-")</f>
         <v>-</v>
       </c>
       <c r="J33" s="9" t="str">
         <f>IF(AND(ISNUMBER(I33),ISNUMBER($B$2)),((I33*Datos!$B34)/(1+Datos!$C34)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K33" s="48">
-        <f>$K$3*(1+Datos!D34)/Datos!B34</f>
-        <v>0</v>
+      <c r="K33" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D34),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D34)/Datos!B34,"-")</f>
+        <v>-</v>
       </c>
       <c r="L33" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K33*Datos!$B34)/(1+Datos!$C34)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4252,7 +4011,7 @@
         <v>45</v>
       </c>
       <c r="C34" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E35),$C$3*(1+Datos!E35)/Datos!B35,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E35),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E35)/Datos!B35,"-")</f>
         <v>-</v>
       </c>
       <c r="D34" s="9" t="str">
@@ -4260,7 +4019,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E34" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F35),$E$3*(1+Datos!F35)/Datos!B35,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F35),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F35)/Datos!B35,"-")</f>
         <v>-</v>
       </c>
       <c r="F34" s="9" t="str">
@@ -4268,24 +4027,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G34" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G35),$G$3*(1+Datos!G35)/Datos!B35,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G35),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G35)/Datos!B35,"-")</f>
         <v>-</v>
       </c>
       <c r="H34" s="9" t="str">
         <f>IF(AND(ISNUMBER(G34),ISNUMBER($B$2)),((G34*Datos!$B35)/(1+Datos!$C35)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I34" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H35),$I$3*(1+Datos!H35)/Datos!B35,"-")</f>
+      <c r="I34" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H35),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H35)/Datos!B35,"-")</f>
         <v>-</v>
       </c>
       <c r="J34" s="9" t="str">
         <f>IF(AND(ISNUMBER(I34),ISNUMBER($B$2)),((I34*Datos!$B35)/(1+Datos!$C35)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K34" s="48">
-        <f>$K$3*(1+Datos!D35)/Datos!B35</f>
-        <v>0</v>
+      <c r="K34" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D35),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D35)/Datos!B35,"-")</f>
+        <v>-</v>
       </c>
       <c r="L34" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K34*Datos!$B35)/(1+Datos!$C35)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4301,7 +4060,7 @@
         <v>46</v>
       </c>
       <c r="C35" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E36),$C$3*(1+Datos!E36)/Datos!B36,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E36),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E36)/Datos!B36,"-")</f>
         <v>-</v>
       </c>
       <c r="D35" s="9" t="str">
@@ -4309,7 +4068,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E35" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F36),$E$3*(1+Datos!F36)/Datos!B36,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F36),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F36)/Datos!B36,"-")</f>
         <v>-</v>
       </c>
       <c r="F35" s="9" t="str">
@@ -4317,24 +4076,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G35" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G36),$G$3*(1+Datos!G36)/Datos!B36,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G36),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G36)/Datos!B36,"-")</f>
         <v>-</v>
       </c>
       <c r="H35" s="9" t="str">
         <f>IF(AND(ISNUMBER(G35),ISNUMBER($B$2)),((G35*Datos!$B36)/(1+Datos!$C36)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I35" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H36),$I$3*(1+Datos!H36)/Datos!B36,"-")</f>
+      <c r="I35" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H36),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H36)/Datos!B36,"-")</f>
         <v>-</v>
       </c>
       <c r="J35" s="9" t="str">
         <f>IF(AND(ISNUMBER(I35),ISNUMBER($B$2)),((I35*Datos!$B36)/(1+Datos!$C36)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K35" s="48">
-        <f>$K$3*(1+Datos!D36)/Datos!B36</f>
-        <v>0</v>
+      <c r="K35" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D36),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D36)/Datos!B36,"-")</f>
+        <v>-</v>
       </c>
       <c r="L35" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K35*Datos!$B36)/(1+Datos!$C36)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4350,7 +4109,7 @@
         <v>47</v>
       </c>
       <c r="C36" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E37),$C$3*(1+Datos!E37)/Datos!B37,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E37),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E37)/Datos!B37,"-")</f>
         <v>-</v>
       </c>
       <c r="D36" s="9" t="str">
@@ -4358,7 +4117,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E36" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F37),$E$3*(1+Datos!F37)/Datos!B37,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F37),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F37)/Datos!B37,"-")</f>
         <v>-</v>
       </c>
       <c r="F36" s="9" t="str">
@@ -4366,24 +4125,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G36" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G37),$G$3*(1+Datos!G37)/Datos!B37,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G37),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G37)/Datos!B37,"-")</f>
         <v>-</v>
       </c>
       <c r="H36" s="9" t="str">
         <f>IF(AND(ISNUMBER(G36),ISNUMBER($B$2)),((G36*Datos!$B37)/(1+Datos!$C37)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I36" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H37),$I$3*(1+Datos!H37)/Datos!B37,"-")</f>
+      <c r="I36" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H37),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H37)/Datos!B37,"-")</f>
         <v>-</v>
       </c>
       <c r="J36" s="9" t="str">
         <f>IF(AND(ISNUMBER(I36),ISNUMBER($B$2)),((I36*Datos!$B37)/(1+Datos!$C37)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K36" s="48">
-        <f>$K$3*(1+Datos!D37)/Datos!B37</f>
-        <v>0</v>
+      <c r="K36" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D37),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D37)/Datos!B37,"-")</f>
+        <v>-</v>
       </c>
       <c r="L36" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K36*Datos!$B37)/(1+Datos!$C37)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4399,7 +4158,7 @@
         <v>48</v>
       </c>
       <c r="C37" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E38),$C$3*(1+Datos!E38)/Datos!B38,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E38),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E38)/Datos!B38,"-")</f>
         <v>-</v>
       </c>
       <c r="D37" s="9" t="str">
@@ -4407,7 +4166,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E37" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F38),$E$3*(1+Datos!F38)/Datos!B38,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F38),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F38)/Datos!B38,"-")</f>
         <v>-</v>
       </c>
       <c r="F37" s="9" t="str">
@@ -4415,24 +4174,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G37" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G38),$G$3*(1+Datos!G38)/Datos!B38,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G38),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G38)/Datos!B38,"-")</f>
         <v>-</v>
       </c>
       <c r="H37" s="9" t="str">
         <f>IF(AND(ISNUMBER(G37),ISNUMBER($B$2)),((G37*Datos!$B38)/(1+Datos!$C38)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I37" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H38),$I$3*(1+Datos!H38)/Datos!B38,"-")</f>
+      <c r="I37" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H38),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H38)/Datos!B38,"-")</f>
         <v>-</v>
       </c>
       <c r="J37" s="9" t="str">
         <f>IF(AND(ISNUMBER(I37),ISNUMBER($B$2)),((I37*Datos!$B38)/(1+Datos!$C38)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K37" s="48">
-        <f>$K$3*(1+Datos!D38)/Datos!B38</f>
-        <v>0</v>
+      <c r="K37" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D38),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D38)/Datos!B38,"-")</f>
+        <v>-</v>
       </c>
       <c r="L37" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K37*Datos!$B38)/(1+Datos!$C38)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4448,7 +4207,7 @@
         <v>13</v>
       </c>
       <c r="C38" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E39),$C$3*(1+Datos!E39)/Datos!B39,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E39),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E39)/Datos!B39,"-")</f>
         <v>-</v>
       </c>
       <c r="D38" s="9" t="str">
@@ -4456,7 +4215,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E38" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F39),$E$3*(1+Datos!F39)/Datos!B39,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F39),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F39)/Datos!B39,"-")</f>
         <v>-</v>
       </c>
       <c r="F38" s="9" t="str">
@@ -4464,24 +4223,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G38" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G39),$G$3*(1+Datos!G39)/Datos!B39,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G39),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G39)/Datos!B39,"-")</f>
         <v>-</v>
       </c>
       <c r="H38" s="9" t="str">
         <f>IF(AND(ISNUMBER(G38),ISNUMBER($B$2)),((G38*Datos!$B39)/(1+Datos!$C39)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I38" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H39),$I$3*(1+Datos!H39)/Datos!B39,"-")</f>
+      <c r="I38" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H39),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H39)/Datos!B39,"-")</f>
         <v>-</v>
       </c>
       <c r="J38" s="9" t="str">
         <f>IF(AND(ISNUMBER(I38),ISNUMBER($B$2)),((I38*Datos!$B39)/(1+Datos!$C39)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K38" s="48">
-        <f>$K$3*(1+Datos!D39)/Datos!B39</f>
-        <v>0</v>
+      <c r="K38" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D39),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D39)/Datos!B39,"-")</f>
+        <v>-</v>
       </c>
       <c r="L38" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K38*Datos!$B39)/(1+Datos!$C39)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4497,7 +4256,7 @@
         <v>50</v>
       </c>
       <c r="C39" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E40),$C$3*(1+Datos!E40)/Datos!B40,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E40),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E40)/Datos!B40,"-")</f>
         <v>-</v>
       </c>
       <c r="D39" s="9" t="str">
@@ -4505,7 +4264,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E39" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F40),$E$3*(1+Datos!F40)/Datos!B40,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F40),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F40)/Datos!B40,"-")</f>
         <v>-</v>
       </c>
       <c r="F39" s="9" t="str">
@@ -4513,24 +4272,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G39" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G40),$G$3*(1+Datos!G40)/Datos!B40,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G40),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G40)/Datos!B40,"-")</f>
         <v>-</v>
       </c>
       <c r="H39" s="9" t="str">
         <f>IF(AND(ISNUMBER(G39),ISNUMBER($B$2)),((G39*Datos!$B40)/(1+Datos!$C40)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I39" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H40),$I$3*(1+Datos!H40)/Datos!B40,"-")</f>
+      <c r="I39" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H40),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H40)/Datos!B40,"-")</f>
         <v>-</v>
       </c>
       <c r="J39" s="9" t="str">
         <f>IF(AND(ISNUMBER(I39),ISNUMBER($B$2)),((I39*Datos!$B40)/(1+Datos!$C40)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K39" s="48">
-        <f>$K$3*(1+Datos!D40)/Datos!B40</f>
-        <v>0</v>
+      <c r="K39" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D40),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D40)/Datos!B40,"-")</f>
+        <v>-</v>
       </c>
       <c r="L39" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K39*Datos!$B40)/(1+Datos!$C40)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4546,7 +4305,7 @@
         <v>51</v>
       </c>
       <c r="C40" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E41),$C$3*(1+Datos!E41)/Datos!B41,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E41),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E41)/Datos!B41,"-")</f>
         <v>-</v>
       </c>
       <c r="D40" s="9" t="str">
@@ -4554,7 +4313,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E40" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F41),$E$3*(1+Datos!F41)/Datos!B41,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F41),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F41)/Datos!B41,"-")</f>
         <v>-</v>
       </c>
       <c r="F40" s="9" t="str">
@@ -4562,24 +4321,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G40" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G41),$G$3*(1+Datos!G41)/Datos!B41,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G41),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G41)/Datos!B41,"-")</f>
         <v>-</v>
       </c>
       <c r="H40" s="9" t="str">
         <f>IF(AND(ISNUMBER(G40),ISNUMBER($B$2)),((G40*Datos!$B41)/(1+Datos!$C41)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I40" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H41),$I$3*(1+Datos!H41)/Datos!B41,"-")</f>
+      <c r="I40" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H41),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H41)/Datos!B41,"-")</f>
         <v>-</v>
       </c>
       <c r="J40" s="9" t="str">
         <f>IF(AND(ISNUMBER(I40),ISNUMBER($B$2)),((I40*Datos!$B41)/(1+Datos!$C41)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K40" s="48">
-        <f>$K$3*(1+Datos!D41)/Datos!B41</f>
-        <v>0</v>
+      <c r="K40" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D41),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D41)/Datos!B41,"-")</f>
+        <v>-</v>
       </c>
       <c r="L40" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K40*Datos!$B41)/(1+Datos!$C41)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4595,7 +4354,7 @@
         <v>52</v>
       </c>
       <c r="C41" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E42),$C$3*(1+Datos!E42)/Datos!B42,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E42),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E42)/Datos!B42,"-")</f>
         <v>-</v>
       </c>
       <c r="D41" s="9" t="str">
@@ -4603,7 +4362,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E41" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F42),$E$3*(1+Datos!F42)/Datos!B42,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F42),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F42)/Datos!B42,"-")</f>
         <v>-</v>
       </c>
       <c r="F41" s="9" t="str">
@@ -4611,24 +4370,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G41" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G42),$G$3*(1+Datos!G42)/Datos!B42,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G42),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G42)/Datos!B42,"-")</f>
         <v>-</v>
       </c>
       <c r="H41" s="9" t="str">
         <f>IF(AND(ISNUMBER(G41),ISNUMBER($B$2)),((G41*Datos!$B42)/(1+Datos!$C42)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I41" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H42),$I$3*(1+Datos!H42)/Datos!B42,"-")</f>
+      <c r="I41" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H42),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H42)/Datos!B42,"-")</f>
         <v>-</v>
       </c>
       <c r="J41" s="9" t="str">
         <f>IF(AND(ISNUMBER(I41),ISNUMBER($B$2)),((I41*Datos!$B42)/(1+Datos!$C42)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K41" s="48">
-        <f>$K$3*(1+Datos!D42)/Datos!B42</f>
-        <v>0</v>
+      <c r="K41" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D42),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D42)/Datos!B42,"-")</f>
+        <v>-</v>
       </c>
       <c r="L41" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K41*Datos!$B42)/(1+Datos!$C42)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4644,7 +4403,7 @@
         <v>53</v>
       </c>
       <c r="C42" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E43),$C$3*(1+Datos!E43)/Datos!B43,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E43),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E43)/Datos!B43,"-")</f>
         <v>-</v>
       </c>
       <c r="D42" s="9" t="str">
@@ -4652,7 +4411,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E42" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F43),$E$3*(1+Datos!F43)/Datos!B43,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F43),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F43)/Datos!B43,"-")</f>
         <v>-</v>
       </c>
       <c r="F42" s="9" t="str">
@@ -4660,24 +4419,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G42" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G43),$G$3*(1+Datos!G43)/Datos!B43,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G43),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G43)/Datos!B43,"-")</f>
         <v>-</v>
       </c>
       <c r="H42" s="9" t="str">
         <f>IF(AND(ISNUMBER(G42),ISNUMBER($B$2)),((G42*Datos!$B43)/(1+Datos!$C43)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I42" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H43),$I$3*(1+Datos!H43)/Datos!B43,"-")</f>
+      <c r="I42" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H43),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H43)/Datos!B43,"-")</f>
         <v>-</v>
       </c>
       <c r="J42" s="9" t="str">
         <f>IF(AND(ISNUMBER(I42),ISNUMBER($B$2)),((I42*Datos!$B43)/(1+Datos!$C43)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K42" s="48">
-        <f>$K$3*(1+Datos!D43)/Datos!B43</f>
-        <v>0</v>
+      <c r="K42" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D43),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D43)/Datos!B43,"-")</f>
+        <v>-</v>
       </c>
       <c r="L42" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K42*Datos!$B43)/(1+Datos!$C43)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4693,7 +4452,7 @@
         <v>54</v>
       </c>
       <c r="C43" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E44),$C$3*(1+Datos!E44)/Datos!B44,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E44),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E44)/Datos!B44,"-")</f>
         <v>-</v>
       </c>
       <c r="D43" s="9" t="str">
@@ -4701,7 +4460,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E43" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F44),$E$3*(1+Datos!F44)/Datos!B44,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F44),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F44)/Datos!B44,"-")</f>
         <v>-</v>
       </c>
       <c r="F43" s="9" t="str">
@@ -4709,24 +4468,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G43" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G44),$G$3*(1+Datos!G44)/Datos!B44,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G44),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G44)/Datos!B44,"-")</f>
         <v>-</v>
       </c>
       <c r="H43" s="9" t="str">
         <f>IF(AND(ISNUMBER(G43),ISNUMBER($B$2)),((G43*Datos!$B44)/(1+Datos!$C44)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I43" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H44),$I$3*(1+Datos!H44)/Datos!B44,"-")</f>
+      <c r="I43" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H44),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H44)/Datos!B44,"-")</f>
         <v>-</v>
       </c>
       <c r="J43" s="9" t="str">
         <f>IF(AND(ISNUMBER(I43),ISNUMBER($B$2)),((I43*Datos!$B44)/(1+Datos!$C44)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K43" s="48">
-        <f>$K$3*(1+Datos!D44)/Datos!B44</f>
-        <v>0</v>
+      <c r="K43" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D44),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D44)/Datos!B44,"-")</f>
+        <v>-</v>
       </c>
       <c r="L43" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K43*Datos!$B44)/(1+Datos!$C44)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4742,7 +4501,7 @@
         <v>55</v>
       </c>
       <c r="C44" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E45),$C$3*(1+Datos!E45)/Datos!B45,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E45),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E45)/Datos!B45,"-")</f>
         <v>-</v>
       </c>
       <c r="D44" s="9" t="str">
@@ -4750,7 +4509,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E44" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F45),$E$3*(1+Datos!F45)/Datos!B45,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F45),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F45)/Datos!B45,"-")</f>
         <v>-</v>
       </c>
       <c r="F44" s="9" t="str">
@@ -4758,24 +4517,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G44" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G45),$G$3*(1+Datos!G45)/Datos!B45,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G45),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G45)/Datos!B45,"-")</f>
         <v>-</v>
       </c>
       <c r="H44" s="9" t="str">
         <f>IF(AND(ISNUMBER(G44),ISNUMBER($B$2)),((G44*Datos!$B45)/(1+Datos!$C45)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I44" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H45),$I$3*(1+Datos!H45)/Datos!B45,"-")</f>
+      <c r="I44" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H45),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H45)/Datos!B45,"-")</f>
         <v>-</v>
       </c>
       <c r="J44" s="9" t="str">
         <f>IF(AND(ISNUMBER(I44),ISNUMBER($B$2)),((I44*Datos!$B45)/(1+Datos!$C45)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K44" s="48">
-        <f>$K$3*(1+Datos!D45)/Datos!B45</f>
-        <v>0</v>
+      <c r="K44" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D45),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D45)/Datos!B45,"-")</f>
+        <v>-</v>
       </c>
       <c r="L44" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K44*Datos!$B45)/(1+Datos!$C45)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4791,7 +4550,7 @@
         <v>56</v>
       </c>
       <c r="C45" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E46),$C$3*(1+Datos!E46)/Datos!B46,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E46),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E46)/Datos!B46,"-")</f>
         <v>-</v>
       </c>
       <c r="D45" s="9" t="str">
@@ -4799,7 +4558,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E45" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F46),$E$3*(1+Datos!F46)/Datos!B46,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F46),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F46)/Datos!B46,"-")</f>
         <v>-</v>
       </c>
       <c r="F45" s="9" t="str">
@@ -4807,24 +4566,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G45" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G46),$G$3*(1+Datos!G46)/Datos!B46,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G46),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G46)/Datos!B46,"-")</f>
         <v>-</v>
       </c>
       <c r="H45" s="9" t="str">
         <f>IF(AND(ISNUMBER(G45),ISNUMBER($B$2)),((G45*Datos!$B46)/(1+Datos!$C46)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I45" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H46),$I$3*(1+Datos!H46)/Datos!B46,"-")</f>
+      <c r="I45" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H46),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H46)/Datos!B46,"-")</f>
         <v>-</v>
       </c>
       <c r="J45" s="9" t="str">
         <f>IF(AND(ISNUMBER(I45),ISNUMBER($B$2)),((I45*Datos!$B46)/(1+Datos!$C46)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K45" s="48">
-        <f>$K$3*(1+Datos!D46)/Datos!B46</f>
-        <v>0</v>
+      <c r="K45" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D46),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D46)/Datos!B46,"-")</f>
+        <v>-</v>
       </c>
       <c r="L45" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K45*Datos!$B46)/(1+Datos!$C46)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4840,7 +4599,7 @@
         <v>57</v>
       </c>
       <c r="C46" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E47),$C$3*(1+Datos!E47)/Datos!B47,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E47),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E47)/Datos!B47,"-")</f>
         <v>-</v>
       </c>
       <c r="D46" s="9" t="str">
@@ -4848,7 +4607,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E46" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F47),$E$3*(1+Datos!F47)/Datos!B47,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F47),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F47)/Datos!B47,"-")</f>
         <v>-</v>
       </c>
       <c r="F46" s="9" t="str">
@@ -4856,24 +4615,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G46" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G47),$G$3*(1+Datos!G47)/Datos!B47,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G47),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G47)/Datos!B47,"-")</f>
         <v>-</v>
       </c>
       <c r="H46" s="9" t="str">
         <f>IF(AND(ISNUMBER(G46),ISNUMBER($B$2)),((G46*Datos!$B47)/(1+Datos!$C47)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I46" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H47),$I$3*(1+Datos!H47)/Datos!B47,"-")</f>
+      <c r="I46" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H47),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H47)/Datos!B47,"-")</f>
         <v>-</v>
       </c>
       <c r="J46" s="9" t="str">
         <f>IF(AND(ISNUMBER(I46),ISNUMBER($B$2)),((I46*Datos!$B47)/(1+Datos!$C47)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K46" s="48">
-        <f>$K$3*(1+Datos!D47)/Datos!B47</f>
-        <v>0</v>
+      <c r="K46" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D47),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D47)/Datos!B47,"-")</f>
+        <v>-</v>
       </c>
       <c r="L46" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K46*Datos!$B47)/(1+Datos!$C47)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4889,7 +4648,7 @@
         <v>59</v>
       </c>
       <c r="C47" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E48),$C$3*(1+Datos!E48)/Datos!B48,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E48),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E48)/Datos!B48,"-")</f>
         <v>-</v>
       </c>
       <c r="D47" s="9" t="str">
@@ -4897,7 +4656,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E47" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F48),$E$3*(1+Datos!F48)/Datos!B48,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F48),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F48)/Datos!B48,"-")</f>
         <v>-</v>
       </c>
       <c r="F47" s="9" t="str">
@@ -4905,24 +4664,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G47" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G48),$G$3*(1+Datos!G48)/Datos!B48,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G48),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G48)/Datos!B48,"-")</f>
         <v>-</v>
       </c>
       <c r="H47" s="9" t="str">
         <f>IF(AND(ISNUMBER(G47),ISNUMBER($B$2)),((G47*Datos!$B48)/(1+Datos!$C48)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I47" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H48),$I$3*(1+Datos!H48)/Datos!B48,"-")</f>
+      <c r="I47" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H48),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H48)/Datos!B48,"-")</f>
         <v>-</v>
       </c>
       <c r="J47" s="9" t="str">
         <f>IF(AND(ISNUMBER(I47),ISNUMBER($B$2)),((I47*Datos!$B48)/(1+Datos!$C48)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K47" s="48">
-        <f>$K$3*(1+Datos!D48)/Datos!B48</f>
-        <v>0</v>
+      <c r="K47" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D48),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D48)/Datos!B48,"-")</f>
+        <v>-</v>
       </c>
       <c r="L47" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K47*Datos!$B48)/(1+Datos!$C48)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4938,7 +4697,7 @@
         <v>60</v>
       </c>
       <c r="C48" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E49),$C$3*(1+Datos!E49)/Datos!B49,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E49),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E49)/Datos!B49,"-")</f>
         <v>-</v>
       </c>
       <c r="D48" s="9" t="str">
@@ -4946,7 +4705,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E48" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F49),$E$3*(1+Datos!F49)/Datos!B49,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F49),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F49)/Datos!B49,"-")</f>
         <v>-</v>
       </c>
       <c r="F48" s="9" t="str">
@@ -4954,24 +4713,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G48" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G49),$G$3*(1+Datos!G49)/Datos!B49,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G49),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G49)/Datos!B49,"-")</f>
         <v>-</v>
       </c>
       <c r="H48" s="9" t="str">
         <f>IF(AND(ISNUMBER(G48),ISNUMBER($B$2)),((G48*Datos!$B49)/(1+Datos!$C49)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I48" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H49),$I$3*(1+Datos!H49)/Datos!B49,"-")</f>
+      <c r="I48" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H49),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H49)/Datos!B49,"-")</f>
         <v>-</v>
       </c>
       <c r="J48" s="9" t="str">
         <f>IF(AND(ISNUMBER(I48),ISNUMBER($B$2)),((I48*Datos!$B49)/(1+Datos!$C49)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K48" s="48">
-        <f>$K$3*(1+Datos!D49)/Datos!B49</f>
-        <v>0</v>
+      <c r="K48" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D49),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D49)/Datos!B49,"-")</f>
+        <v>-</v>
       </c>
       <c r="L48" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K48*Datos!$B49)/(1+Datos!$C49)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -4987,7 +4746,7 @@
         <v>61</v>
       </c>
       <c r="C49" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E50),$C$3*(1+Datos!E50)/Datos!B50,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E50),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E50)/Datos!B50,"-")</f>
         <v>-</v>
       </c>
       <c r="D49" s="9" t="str">
@@ -4995,7 +4754,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E49" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F50),$E$3*(1+Datos!F50)/Datos!B50,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F50),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F50)/Datos!B50,"-")</f>
         <v>-</v>
       </c>
       <c r="F49" s="9" t="str">
@@ -5003,24 +4762,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G49" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G50),$G$3*(1+Datos!G50)/Datos!B50,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G50),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G50)/Datos!B50,"-")</f>
         <v>-</v>
       </c>
       <c r="H49" s="9" t="str">
         <f>IF(AND(ISNUMBER(G49),ISNUMBER($B$2)),((G49*Datos!$B50)/(1+Datos!$C50)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I49" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H50),$I$3*(1+Datos!H50)/Datos!B50,"-")</f>
+      <c r="I49" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H50),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H50)/Datos!B50,"-")</f>
         <v>-</v>
       </c>
       <c r="J49" s="9" t="str">
         <f>IF(AND(ISNUMBER(I49),ISNUMBER($B$2)),((I49*Datos!$B50)/(1+Datos!$C50)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K49" s="48">
-        <f>$K$3*(1+Datos!D50)/Datos!B50</f>
-        <v>0</v>
+      <c r="K49" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D50),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D50)/Datos!B50,"-")</f>
+        <v>-</v>
       </c>
       <c r="L49" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K49*Datos!$B50)/(1+Datos!$C50)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -5036,7 +4795,7 @@
         <v>62</v>
       </c>
       <c r="C50" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E51),$C$3*(1+Datos!E51)/Datos!B51,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E51),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E51)/Datos!B51,"-")</f>
         <v>-</v>
       </c>
       <c r="D50" s="9" t="str">
@@ -5044,7 +4803,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E50" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F51),$E$3*(1+Datos!F51)/Datos!B51,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F51),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F51)/Datos!B51,"-")</f>
         <v>-</v>
       </c>
       <c r="F50" s="9" t="str">
@@ -5052,24 +4811,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G50" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G51),$G$3*(1+Datos!G51)/Datos!B51,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G51),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G51)/Datos!B51,"-")</f>
         <v>-</v>
       </c>
       <c r="H50" s="9" t="str">
         <f>IF(AND(ISNUMBER(G50),ISNUMBER($B$2)),((G50*Datos!$B51)/(1+Datos!$C51)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I50" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H51),$I$3*(1+Datos!H51)/Datos!B51,"-")</f>
+      <c r="I50" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H51),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H51)/Datos!B51,"-")</f>
         <v>-</v>
       </c>
       <c r="J50" s="9" t="str">
         <f>IF(AND(ISNUMBER(I50),ISNUMBER($B$2)),((I50*Datos!$B51)/(1+Datos!$C51)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K50" s="48">
-        <f>$K$3*(1+Datos!D51)/Datos!B51</f>
-        <v>0</v>
+      <c r="K50" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D51),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D51)/Datos!B51,"-")</f>
+        <v>-</v>
       </c>
       <c r="L50" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K50*Datos!$B51)/(1+Datos!$C51)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -5085,7 +4844,7 @@
         <v>63</v>
       </c>
       <c r="C51" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E52),$C$3*(1+Datos!E52)/Datos!B52,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E52),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E52)/Datos!B52,"-")</f>
         <v>-</v>
       </c>
       <c r="D51" s="9" t="str">
@@ -5093,7 +4852,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E51" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F52),$E$3*(1+Datos!F52)/Datos!B52,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F52),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F52)/Datos!B52,"-")</f>
         <v>-</v>
       </c>
       <c r="F51" s="9" t="str">
@@ -5101,24 +4860,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G51" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G52),$G$3*(1+Datos!G52)/Datos!B52,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G52),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G52)/Datos!B52,"-")</f>
         <v>-</v>
       </c>
       <c r="H51" s="9" t="str">
         <f>IF(AND(ISNUMBER(G51),ISNUMBER($B$2)),((G51*Datos!$B52)/(1+Datos!$C52)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I51" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H52),$I$3*(1+Datos!H52)/Datos!B52,"-")</f>
+      <c r="I51" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H52),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H52)/Datos!B52,"-")</f>
         <v>-</v>
       </c>
       <c r="J51" s="9" t="str">
         <f>IF(AND(ISNUMBER(I51),ISNUMBER($B$2)),((I51*Datos!$B52)/(1+Datos!$C52)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K51" s="48">
-        <f>$K$3*(1+Datos!D52)/Datos!B52</f>
-        <v>0</v>
+      <c r="K51" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D52),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D52)/Datos!B52,"-")</f>
+        <v>-</v>
       </c>
       <c r="L51" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K51*Datos!$B52)/(1+Datos!$C52)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -5134,7 +4893,7 @@
         <v>64</v>
       </c>
       <c r="C52" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E53),$C$3*(1+Datos!E53)/Datos!B53,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E53),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E53)/Datos!B53,"-")</f>
         <v>-</v>
       </c>
       <c r="D52" s="9" t="str">
@@ -5142,7 +4901,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E52" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F53),$E$3*(1+Datos!F53)/Datos!B53,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F53),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F53)/Datos!B53,"-")</f>
         <v>-</v>
       </c>
       <c r="F52" s="9" t="str">
@@ -5150,24 +4909,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G52" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G53),$G$3*(1+Datos!G53)/Datos!B53,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G53),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G53)/Datos!B53,"-")</f>
         <v>-</v>
       </c>
       <c r="H52" s="9" t="str">
         <f>IF(AND(ISNUMBER(G52),ISNUMBER($B$2)),((G52*Datos!$B53)/(1+Datos!$C53)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I52" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H53),$I$3*(1+Datos!H53)/Datos!B53,"-")</f>
+      <c r="I52" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H53),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H53)/Datos!B53,"-")</f>
         <v>-</v>
       </c>
       <c r="J52" s="9" t="str">
         <f>IF(AND(ISNUMBER(I52),ISNUMBER($B$2)),((I52*Datos!$B53)/(1+Datos!$C53)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K52" s="48">
-        <f>$K$3*(1+Datos!D53)/Datos!B53</f>
-        <v>0</v>
+      <c r="K52" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D53),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D53)/Datos!B53,"-")</f>
+        <v>-</v>
       </c>
       <c r="L52" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K52*Datos!$B53)/(1+Datos!$C53)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -5183,7 +4942,7 @@
         <v>66</v>
       </c>
       <c r="C53" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E54),$C$3*(1+Datos!E54)/Datos!B54,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E54),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E54)/Datos!B54,"-")</f>
         <v>-</v>
       </c>
       <c r="D53" s="9" t="str">
@@ -5191,7 +4950,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E53" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F54),$E$3*(1+Datos!F54)/Datos!B54,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F54),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F54)/Datos!B54,"-")</f>
         <v>-</v>
       </c>
       <c r="F53" s="9" t="str">
@@ -5199,24 +4958,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G53" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G54),$G$3*(1+Datos!G54)/Datos!B54,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G54),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G54)/Datos!B54,"-")</f>
         <v>-</v>
       </c>
       <c r="H53" s="9" t="str">
         <f>IF(AND(ISNUMBER(G53),ISNUMBER($B$2)),((G53*Datos!$B54)/(1+Datos!$C54)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I53" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H54),$I$3*(1+Datos!H54)/Datos!B54,"-")</f>
+      <c r="I53" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H54),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H54)/Datos!B54,"-")</f>
         <v>-</v>
       </c>
       <c r="J53" s="9" t="str">
         <f>IF(AND(ISNUMBER(I53),ISNUMBER($B$2)),((I53*Datos!$B54)/(1+Datos!$C54)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K53" s="48">
-        <f>$K$3*(1+Datos!D54)/Datos!B54</f>
-        <v>0</v>
+      <c r="K53" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D54),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D54)/Datos!B54,"-")</f>
+        <v>-</v>
       </c>
       <c r="L53" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K53*Datos!$B54)/(1+Datos!$C54)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -5232,7 +4991,7 @@
         <v>67</v>
       </c>
       <c r="C54" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E55),$C$3*(1+Datos!E55)/Datos!B55,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E55),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E55)/Datos!B55,"-")</f>
         <v>-</v>
       </c>
       <c r="D54" s="9" t="str">
@@ -5240,7 +4999,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E54" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F55),$E$3*(1+Datos!F55)/Datos!B55,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F55),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F55)/Datos!B55,"-")</f>
         <v>-</v>
       </c>
       <c r="F54" s="9" t="str">
@@ -5248,24 +5007,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G54" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G55),$G$3*(1+Datos!G55)/Datos!B55,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G55),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G55)/Datos!B55,"-")</f>
         <v>-</v>
       </c>
       <c r="H54" s="9" t="str">
         <f>IF(AND(ISNUMBER(G54),ISNUMBER($B$2)),((G54*Datos!$B55)/(1+Datos!$C55)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I54" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H55),$I$3*(1+Datos!H55)/Datos!B55,"-")</f>
+      <c r="I54" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H55),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H55)/Datos!B55,"-")</f>
         <v>-</v>
       </c>
       <c r="J54" s="9" t="str">
         <f>IF(AND(ISNUMBER(I54),ISNUMBER($B$2)),((I54*Datos!$B55)/(1+Datos!$C55)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K54" s="48">
-        <f>$K$3*(1+Datos!D55)/Datos!B55</f>
-        <v>0</v>
+      <c r="K54" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D55),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D55)/Datos!B55,"-")</f>
+        <v>-</v>
       </c>
       <c r="L54" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K54*Datos!$B55)/(1+Datos!$C55)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -5281,7 +5040,7 @@
         <v>68</v>
       </c>
       <c r="C55" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E56),$C$3*(1+Datos!E56)/Datos!B56,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E56),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E56)/Datos!B56,"-")</f>
         <v>-</v>
       </c>
       <c r="D55" s="9" t="str">
@@ -5289,7 +5048,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E55" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F56),$E$3*(1+Datos!F56)/Datos!B56,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F56),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F56)/Datos!B56,"-")</f>
         <v>-</v>
       </c>
       <c r="F55" s="9" t="str">
@@ -5297,24 +5056,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G55" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G56),$G$3*(1+Datos!G56)/Datos!B56,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G56),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G56)/Datos!B56,"-")</f>
         <v>-</v>
       </c>
       <c r="H55" s="9" t="str">
         <f>IF(AND(ISNUMBER(G55),ISNUMBER($B$2)),((G55*Datos!$B56)/(1+Datos!$C56)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I55" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H56),$I$3*(1+Datos!H56)/Datos!B56,"-")</f>
+      <c r="I55" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H56),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H56)/Datos!B56,"-")</f>
         <v>-</v>
       </c>
       <c r="J55" s="9" t="str">
         <f>IF(AND(ISNUMBER(I55),ISNUMBER($B$2)),((I55*Datos!$B56)/(1+Datos!$C56)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K55" s="48">
-        <f>$K$3*(1+Datos!D56)/Datos!B56</f>
-        <v>0</v>
+      <c r="K55" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D56),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D56)/Datos!B56,"-")</f>
+        <v>-</v>
       </c>
       <c r="L55" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K55*Datos!$B56)/(1+Datos!$C56)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -5330,7 +5089,7 @@
         <v>66</v>
       </c>
       <c r="C56" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E57),$C$3*(1+Datos!E57)/Datos!B57,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E57),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E57)/Datos!B57,"-")</f>
         <v>-</v>
       </c>
       <c r="D56" s="9" t="str">
@@ -5338,7 +5097,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E56" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F57),$E$3*(1+Datos!F57)/Datos!B57,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F57),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F57)/Datos!B57,"-")</f>
         <v>-</v>
       </c>
       <c r="F56" s="9" t="str">
@@ -5346,24 +5105,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G56" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G57),$G$3*(1+Datos!G57)/Datos!B57,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G57),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G57)/Datos!B57,"-")</f>
         <v>-</v>
       </c>
       <c r="H56" s="9" t="str">
         <f>IF(AND(ISNUMBER(G56),ISNUMBER($B$2)),((G56*Datos!$B57)/(1+Datos!$C57)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I56" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H57),$I$3*(1+Datos!H57)/Datos!B57,"-")</f>
+      <c r="I56" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H57),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H57)/Datos!B57,"-")</f>
         <v>-</v>
       </c>
       <c r="J56" s="9" t="str">
         <f>IF(AND(ISNUMBER(I56),ISNUMBER($B$2)),((I56*Datos!$B57)/(1+Datos!$C57)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K56" s="48">
-        <f>$K$3*(1+Datos!D57)/Datos!B57</f>
-        <v>0</v>
+      <c r="K56" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D57),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D57)/Datos!B57,"-")</f>
+        <v>-</v>
       </c>
       <c r="L56" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K56*Datos!$B57)/(1+Datos!$C57)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -5380,7 +5139,7 @@
         <v>70</v>
       </c>
       <c r="C57" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E58),$C$3*(1+Datos!E58)/Datos!B58,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E58),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E58)/Datos!B58,"-")</f>
         <v>-</v>
       </c>
       <c r="D57" s="9" t="str">
@@ -5388,7 +5147,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E57" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F58),$E$3*(1+Datos!F58)/Datos!B58,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F58),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F58)/Datos!B58,"-")</f>
         <v>-</v>
       </c>
       <c r="F57" s="9" t="str">
@@ -5396,24 +5155,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G57" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G58),$G$3*(1+Datos!G58)/Datos!B58,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G58),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G58)/Datos!B58,"-")</f>
         <v>-</v>
       </c>
       <c r="H57" s="9" t="str">
         <f>IF(AND(ISNUMBER(G57),ISNUMBER($B$2)),((G57*Datos!$B58)/(1+Datos!$C58)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I57" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H58),$I$3*(1+Datos!H58)/Datos!B58,"-")</f>
+      <c r="I57" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H58),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H58)/Datos!B58,"-")</f>
         <v>-</v>
       </c>
       <c r="J57" s="9" t="str">
         <f>IF(AND(ISNUMBER(I57),ISNUMBER($B$2)),((I57*Datos!$B58)/(1+Datos!$C58)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K57" s="48">
-        <f>$K$3*(1+Datos!D58)/Datos!B58</f>
-        <v>0</v>
+      <c r="K57" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D58),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D58)/Datos!B58,"-")</f>
+        <v>-</v>
       </c>
       <c r="L57" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K57*Datos!$B58)/(1+Datos!$C58)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -5429,7 +5188,7 @@
         <v>71</v>
       </c>
       <c r="C58" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E59),$C$3*(1+Datos!E59)/Datos!B59,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E59),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E59)/Datos!B59,"-")</f>
         <v>-</v>
       </c>
       <c r="D58" s="9" t="str">
@@ -5437,7 +5196,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E58" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F59),$E$3*(1+Datos!F59)/Datos!B59,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F59),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F59)/Datos!B59,"-")</f>
         <v>-</v>
       </c>
       <c r="F58" s="9" t="str">
@@ -5445,24 +5204,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G58" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G59),$G$3*(1+Datos!G59)/Datos!B59,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G59),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G59)/Datos!B59,"-")</f>
         <v>-</v>
       </c>
       <c r="H58" s="9" t="str">
         <f>IF(AND(ISNUMBER(G58),ISNUMBER($B$2)),((G58*Datos!$B59)/(1+Datos!$C59)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I58" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H59),$I$3*(1+Datos!H59)/Datos!B59,"-")</f>
+      <c r="I58" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H59),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H59)/Datos!B59,"-")</f>
         <v>-</v>
       </c>
       <c r="J58" s="9" t="str">
         <f>IF(AND(ISNUMBER(I58),ISNUMBER($B$2)),((I58*Datos!$B59)/(1+Datos!$C59)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K58" s="48">
-        <f>$K$3*(1+Datos!D59)/Datos!B59</f>
-        <v>0</v>
+      <c r="K58" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D59),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D59)/Datos!B59,"-")</f>
+        <v>-</v>
       </c>
       <c r="L58" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K58*Datos!$B59)/(1+Datos!$C59)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -5478,7 +5237,7 @@
         <v>72</v>
       </c>
       <c r="C59" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E60),$C$3*(1+Datos!E60)/Datos!B60,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E60),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E60)/Datos!B60,"-")</f>
         <v>-</v>
       </c>
       <c r="D59" s="9" t="str">
@@ -5486,7 +5245,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E59" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F60),$E$3*(1+Datos!F60)/Datos!B60,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F60),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F60)/Datos!B60,"-")</f>
         <v>-</v>
       </c>
       <c r="F59" s="9" t="str">
@@ -5494,24 +5253,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G59" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G60),$G$3*(1+Datos!G60)/Datos!B60,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G60),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G60)/Datos!B60,"-")</f>
         <v>-</v>
       </c>
       <c r="H59" s="9" t="str">
         <f>IF(AND(ISNUMBER(G59),ISNUMBER($B$2)),((G59*Datos!$B60)/(1+Datos!$C60)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I59" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H60),$I$3*(1+Datos!H60)/Datos!B60,"-")</f>
+      <c r="I59" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H60),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H60)/Datos!B60,"-")</f>
         <v>-</v>
       </c>
       <c r="J59" s="9" t="str">
         <f>IF(AND(ISNUMBER(I59),ISNUMBER($B$2)),((I59*Datos!$B60)/(1+Datos!$C60)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K59" s="48">
-        <f>$K$3*(1+Datos!D60)/Datos!B60</f>
-        <v>0</v>
+      <c r="K59" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D60),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D60)/Datos!B60,"-")</f>
+        <v>-</v>
       </c>
       <c r="L59" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K59*Datos!$B60)/(1+Datos!$C60)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -5527,7 +5286,7 @@
         <v>73</v>
       </c>
       <c r="C60" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E61),$C$3*(1+Datos!E61)/Datos!B61,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E61),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E61)/Datos!B61,"-")</f>
         <v>-</v>
       </c>
       <c r="D60" s="9" t="str">
@@ -5535,7 +5294,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E60" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F61),$E$3*(1+Datos!F61)/Datos!B61,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F61),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F61)/Datos!B61,"-")</f>
         <v>-</v>
       </c>
       <c r="F60" s="9" t="str">
@@ -5543,24 +5302,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G60" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G61),$G$3*(1+Datos!G61)/Datos!B61,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G61),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G61)/Datos!B61,"-")</f>
         <v>-</v>
       </c>
       <c r="H60" s="9" t="str">
         <f>IF(AND(ISNUMBER(G60),ISNUMBER($B$2)),((G60*Datos!$B61)/(1+Datos!$C61)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I60" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H61),$I$3*(1+Datos!H61)/Datos!B61,"-")</f>
+      <c r="I60" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H61),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H61)/Datos!B61,"-")</f>
         <v>-</v>
       </c>
       <c r="J60" s="9" t="str">
         <f>IF(AND(ISNUMBER(I60),ISNUMBER($B$2)),((I60*Datos!$B61)/(1+Datos!$C61)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K60" s="48">
-        <f>$K$3*(1+Datos!D61)/Datos!B61</f>
-        <v>0</v>
+      <c r="K60" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D61),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D61)/Datos!B61,"-")</f>
+        <v>-</v>
       </c>
       <c r="L60" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K60*Datos!$B61)/(1+Datos!$C61)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -5576,7 +5335,7 @@
         <v>74</v>
       </c>
       <c r="C61" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E62),$C$3*(1+Datos!E62)/Datos!B62,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E62),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E62)/Datos!B62,"-")</f>
         <v>-</v>
       </c>
       <c r="D61" s="9" t="str">
@@ -5584,7 +5343,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E61" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F62),$E$3*(1+Datos!F62)/Datos!B62,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F62),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F62)/Datos!B62,"-")</f>
         <v>-</v>
       </c>
       <c r="F61" s="9" t="str">
@@ -5592,24 +5351,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G61" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G62),$G$3*(1+Datos!G62)/Datos!B62,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G62),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G62)/Datos!B62,"-")</f>
         <v>-</v>
       </c>
       <c r="H61" s="9" t="str">
         <f>IF(AND(ISNUMBER(G61),ISNUMBER($B$2)),((G61*Datos!$B62)/(1+Datos!$C62)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I61" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H62),$I$3*(1+Datos!H62)/Datos!B62,"-")</f>
+      <c r="I61" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H62),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H62)/Datos!B62,"-")</f>
         <v>-</v>
       </c>
       <c r="J61" s="9" t="str">
         <f>IF(AND(ISNUMBER(I61),ISNUMBER($B$2)),((I61*Datos!$B62)/(1+Datos!$C62)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K61" s="48">
-        <f>$K$3*(1+Datos!D62)/Datos!B62</f>
-        <v>0</v>
+      <c r="K61" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D62),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D62)/Datos!B62,"-")</f>
+        <v>-</v>
       </c>
       <c r="L61" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K61*Datos!$B62)/(1+Datos!$C62)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -5625,7 +5384,7 @@
         <v>75</v>
       </c>
       <c r="C62" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!E63),$C$3*(1+Datos!E63)/Datos!B63,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!E63),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E63)/Datos!B63,"-")</f>
         <v>-</v>
       </c>
       <c r="D62" s="9" t="str">
@@ -5633,7 +5392,7 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="E62" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!F63),$E$3*(1+Datos!F63)/Datos!B63,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!F63),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F63)/Datos!B63,"-")</f>
         <v>-</v>
       </c>
       <c r="F62" s="9" t="str">
@@ -5641,24 +5400,24 @@
         <v>INSERTAR COSTO</v>
       </c>
       <c r="G62" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!G63),$G$3*(1+Datos!G63)/Datos!B63,"-")</f>
+        <f>IF(AND(ISNUMBER(Datos!G63),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G63)/Datos!B63,"-")</f>
         <v>-</v>
       </c>
       <c r="H62" s="9" t="str">
         <f>IF(AND(ISNUMBER(G62),ISNUMBER($B$2)),((G62*Datos!$B63)/(1+Datos!$C63)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="I62" s="48" t="str">
-        <f>IF(ISNUMBER(Datos!H63),$I$3*(1+Datos!H63)/Datos!B63,"-")</f>
+      <c r="I62" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H63),ISNUMBER($I$3),$I$3&gt;0),$I$3*(1-Datos!H63)/Datos!B63,"-")</f>
         <v>-</v>
       </c>
       <c r="J62" s="9" t="str">
         <f>IF(AND(ISNUMBER(I62),ISNUMBER($B$2)),((I62*Datos!$B63)/(1+Datos!$C63)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
         <v>INSERTAR COSTO</v>
       </c>
-      <c r="K62" s="48">
-        <f>$K$3*(1+Datos!D63)/Datos!B63</f>
-        <v>0</v>
+      <c r="K62" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!D63),ISNUMBER($K$3),$K$3&gt;0),$K$3*(1+Datos!D63)/Datos!B63,"-")</f>
+        <v>-</v>
       </c>
       <c r="L62" s="9" t="str">
         <f>IF(ISNUMBER($B$2),((K62*Datos!$B63)/(1+Datos!$C63)/$B$2)-1,"INSERTAR COSTO")</f>
@@ -5673,26 +5432,30 @@
       <c r="B63" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="C63" s="8" t="s">
-        <v>11</v>
+      <c r="C63" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!E64),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E64)/Datos!B64,"-")</f>
+        <v>-</v>
       </c>
       <c r="D63" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E63" s="8" t="s">
-        <v>11</v>
+      <c r="E63" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!F64),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F64)/Datos!B64,"-")</f>
+        <v>-</v>
       </c>
       <c r="F63" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G63" s="8" t="s">
-        <v>11</v>
+      <c r="G63" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G64),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G64)/Datos!B64,"-")</f>
+        <v>-</v>
       </c>
       <c r="H63" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="I63" s="8" t="s">
-        <v>11</v>
+      <c r="I63" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H64),ISNUMBER($I$3)),$I$3*(1-Datos!H64)/Datos!B64,"-")</f>
+        <v>-</v>
       </c>
       <c r="J63" s="9" t="str">
         <f>IF(AND(ISNUMBER(I63),ISNUMBER($B$2)),((I63*Datos!$B64)/(1+Datos!$C64)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>
@@ -5715,26 +5478,30 @@
       <c r="B64" s="34" t="s">
         <v>78</v>
       </c>
-      <c r="C64" s="8" t="s">
-        <v>11</v>
+      <c r="C64" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!E65),ISNUMBER($C$3),$C$3&gt;0),$C$3*(1-Datos!E65)/Datos!B65,"-")</f>
+        <v>-</v>
       </c>
       <c r="D64" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E64" s="8" t="s">
-        <v>11</v>
+      <c r="E64" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!F65),ISNUMBER($E$3),$E$3&gt;0),$E$3*(1-Datos!F65)/Datos!B65,"-")</f>
+        <v>-</v>
       </c>
       <c r="F64" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G64" s="8" t="s">
-        <v>11</v>
+      <c r="G64" s="48" t="str">
+        <f>IF(AND(ISNUMBER(Datos!G65),ISNUMBER($G$3),$G$3&gt;0),$G$3*(1-Datos!G65)/Datos!B65,"-")</f>
+        <v>-</v>
       </c>
       <c r="H64" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="I64" s="8" t="s">
-        <v>11</v>
+      <c r="I64" s="8" t="str">
+        <f>IF(AND(ISNUMBER(Datos!H65),ISNUMBER($I$3)),$I$3*(1-Datos!H65)/Datos!B65,"-")</f>
+        <v>-</v>
       </c>
       <c r="J64" s="9" t="str">
         <f>IF(AND(ISNUMBER(I64),ISNUMBER($B$2)),((I64*Datos!$B65)/(1+Datos!$C65)/$B$2)-1,IF(ISNUMBER($B$2),"-","INSERTAR COSTO"))</f>

</xml_diff>